<commit_message>
data: screening master 2026-03-30
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -647,7 +647,7 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="n">
-        <v>13800</v>
+        <v>14200</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2298</v>
+        <v>2133</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -716,7 +716,7 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
-        <v>2079840</v>
+        <v>2021360</v>
       </c>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
@@ -761,7 +761,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -785,7 +785,7 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="n">
-        <v>63700</v>
+        <v>40220</v>
       </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>859</v>
+        <v>838</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>86180</v>
+        <v>82900</v>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
@@ -907,7 +907,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1287</v>
+        <v>1231</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>40660</v>
+        <v>37240</v>
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>707</v>
+        <v>672</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1004,7 +1004,7 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="n">
-        <v>406400</v>
+        <v>318525</v>
       </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>738</v>
+        <v>681</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1069,7 +1069,7 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="n">
-        <v>608533.3333333334</v>
+        <v>540325</v>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1520</v>
+        <v>1423</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1134,7 +1134,7 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="n">
-        <v>7132800</v>
+        <v>7535550</v>
       </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -1266,7 +1266,7 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="n">
-        <v>2238110.2</v>
+        <v>1966370.8</v>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>

</xml_diff>

<commit_message>
data: screening master 2026-03-31
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -641,13 +641,13 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>46000</v>
+        <v>43000</v>
       </c>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="n">
-        <v>14200</v>
+        <v>16000</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2133</v>
+        <v>2063</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -707,16 +707,16 @@
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>283300</v>
+        <v>227300</v>
       </c>
       <c r="W3" t="n">
-        <v>2911500</v>
+        <v>3235400</v>
       </c>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
-        <v>2021360</v>
+        <v>2032180</v>
       </c>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
@@ -779,13 +779,13 @@
         <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>80100</v>
+        <v>76600</v>
       </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="n">
-        <v>40220</v>
+        <v>33720</v>
       </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>838</v>
+        <v>803</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -845,10 +845,10 @@
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="W5" t="n">
-        <v>212600</v>
+        <v>227900</v>
       </c>
       <c r="X5" t="inlineStr">
         <is>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>82900</v>
+        <v>86440</v>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
@@ -907,7 +907,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1231</v>
+        <v>1260</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -925,7 +925,7 @@
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>183800</v>
+        <v>200400</v>
       </c>
       <c r="X6" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>37240</v>
+        <v>37800</v>
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -998,13 +998,17 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>49900</v>
+      </c>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="n">
-        <v>318525</v>
+        <v>262360</v>
       </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
@@ -1049,7 +1053,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>681</v>
+        <v>729</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1063,13 +1067,17 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="V8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="W8" t="n">
+        <v>70700</v>
+      </c>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="n">
-        <v>540325</v>
+        <v>484140</v>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
@@ -1114,7 +1122,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1423</v>
+        <v>1597</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1128,13 +1136,17 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="n">
+        <v>408200</v>
+      </c>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="n">
-        <v>7535550</v>
+        <v>7379033.333333333</v>
       </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -1178,7 +1190,9 @@
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>24500</v>
+      </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
@@ -1260,13 +1274,13 @@
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>99264</v>
+        <v>96080</v>
       </c>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="n">
-        <v>1966370.8</v>
+        <v>1602701</v>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>

</xml_diff>

<commit_message>
data: screening master 2026-04-01
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -623,7 +623,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -647,7 +647,7 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="n">
-        <v>16000</v>
+        <v>14600</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2063</v>
+        <v>2232</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -716,7 +716,7 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
-        <v>2032180</v>
+        <v>1890100</v>
       </c>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
@@ -785,7 +785,7 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="n">
-        <v>33720</v>
+        <v>28740</v>
       </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>803</v>
+        <v>834</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>86440</v>
+        <v>96620</v>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
@@ -907,7 +907,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1260</v>
+        <v>1292</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>37800</v>
+        <v>38260</v>
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
@@ -1008,7 +1008,7 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="n">
-        <v>262360</v>
+        <v>116000</v>
       </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>729</v>
+        <v>703</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1077,7 +1077,7 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="n">
-        <v>484140</v>
+        <v>313140</v>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1597</v>
+        <v>1540</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="n">
-        <v>7379033.333333333</v>
+        <v>6388500</v>
       </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -1156,27 +1156,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>543A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>日本銀行</t>
+          <t>ＡＲＣＨＩＯＮ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>スタンダード</t>
+          <t>プライム</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>銀行</t>
+          <t>自動車・輸送機</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>銀行業</t>
+          <t>輸送用機器</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>24500</v>
+        <v>431</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -1211,7 +1211,7 @@
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="n">
-        <v>250</v>
+        <v>10246600</v>
       </c>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
@@ -1221,27 +1221,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9399</t>
+          <t>544A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+          <t>ＧＭＳグループ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>スタンダード</t>
+          <t>プライム</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>28</v>
+        <v>419</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -1270,23 +1270,348 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" t="n">
-        <v>96080</v>
-      </c>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="n">
-        <v>1602701</v>
+        <v>244800</v>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>545A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>トランヴィア</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>プライム</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>情報通信・サービスその他</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>情報･通信業</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>906</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="n">
+        <v>91400</v>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>546A</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ＭＩＲＡＩＮＩホールディングス</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>プライム</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>商社・卸売</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>卸売業</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>1771</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="n">
+        <v>157200</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>547A</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ムニノバホールディングス</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>プライム</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>金融（除く銀行）</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>その他金融業</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>455</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="n">
+        <v>2383200</v>
+      </c>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>8301</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>日本銀行</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>スタンダード</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>銀行</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>銀行業</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>24510</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="n">
+        <v>266.6666666666667</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9399</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>スタンダード</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>情報通信・サービスその他</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>情報･通信業</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>29</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" t="n">
+        <v>96080</v>
+      </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="n">
+        <v>1520583.8</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: screening master 2026-04-02
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -623,7 +623,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -647,7 +647,7 @@
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="n">
-        <v>14600</v>
+        <v>19600</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
@@ -692,7 +692,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2232</v>
+        <v>2281</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -716,7 +716,7 @@
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="n">
-        <v>1890100</v>
+        <v>2330460</v>
       </c>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
@@ -761,7 +761,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -785,7 +785,7 @@
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="n">
-        <v>28740</v>
+        <v>28680</v>
       </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
@@ -830,7 +830,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>834</v>
+        <v>801</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>96620</v>
+        <v>93360</v>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
@@ -907,7 +907,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1292</v>
+        <v>1289</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -939,7 +939,7 @@
         <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>38260</v>
+        <v>34480</v>
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
@@ -984,7 +984,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>677</v>
+        <v>684</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1008,7 +1008,7 @@
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="n">
-        <v>116000</v>
+        <v>81840</v>
       </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>703</v>
+        <v>692</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1077,7 +1077,7 @@
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="n">
-        <v>313140</v>
+        <v>268820</v>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1540</v>
+        <v>1486</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="n">
-        <v>6388500</v>
+        <v>5316140</v>
       </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
@@ -1156,27 +1156,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>543A</t>
+          <t>542A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ＡＲＣＨＩＯＮ</t>
+          <t>ビタブリッドジャパン</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>プライム</t>
+          <t>グロース</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>自動車・輸送機</t>
+          <t>素材・化学</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>輸送用機器</t>
+          <t>化学</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>431</v>
+        <v>1279</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -1211,7 +1211,7 @@
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="n">
-        <v>10246600</v>
+        <v>1505100</v>
       </c>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
@@ -1221,12 +1221,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>544A</t>
+          <t>543A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ＧＭＳグループ</t>
+          <t>ＡＲＣＨＩＯＮ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1236,12 +1236,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>機械</t>
+          <t>自動車・輸送機</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>機械</t>
+          <t>輸送用機器</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>419</v>
+        <v>465</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -1276,7 +1276,7 @@
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="n">
-        <v>244800</v>
+        <v>10922450</v>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
@@ -1286,12 +1286,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>545A</t>
+          <t>544A</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>トランヴィア</t>
+          <t>ＧＭＳグループ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1301,12 +1301,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>906</v>
+        <v>413</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -1341,7 +1341,7 @@
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="n">
-        <v>91400</v>
+        <v>247150</v>
       </c>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
@@ -1351,12 +1351,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>546A</t>
+          <t>545A</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ＭＩＲＡＩＮＩホールディングス</t>
+          <t>トランヴィア</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1366,12 +1366,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>商社・卸売</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>卸売業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>1771</v>
+        <v>932</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -1406,7 +1406,7 @@
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="n">
-        <v>157200</v>
+        <v>155450</v>
       </c>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
@@ -1416,12 +1416,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>547A</t>
+          <t>546A</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ムニノバホールディングス</t>
+          <t>ＭＩＲＡＩＮＩホールディングス</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1431,12 +1431,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>金融（除く銀行）</t>
+          <t>商社・卸売</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>その他金融業</t>
+          <t>卸売業</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>455</v>
+        <v>1789</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -1471,7 +1471,7 @@
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="n">
-        <v>2383200</v>
+        <v>195250</v>
       </c>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
@@ -1481,27 +1481,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>547A</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>日本銀行</t>
+          <t>ムニノバホールディングス</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>スタンダード</t>
+          <t>プライム</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>銀行</t>
+          <t>金融（除く銀行）</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>銀行業</t>
+          <t>その他金融業</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>24510</v>
+        <v>434</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -1536,7 +1536,7 @@
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="n">
-        <v>266.6666666666667</v>
+        <v>2210850</v>
       </c>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
@@ -1546,12 +1546,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>9399</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+          <t>日本銀行</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1561,12 +1561,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>銀行</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>銀行業</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1580,9 +1580,7 @@
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
-        <v>29</v>
-      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
@@ -1595,23 +1593,88 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" t="n">
-        <v>96080</v>
-      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="n">
-        <v>1520583.8</v>
+        <v>300</v>
       </c>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>9399</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>スタンダード</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>情報通信・サービスその他</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>情報･通信業</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>27</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
+        <v>96080</v>
+      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="n">
+        <v>1764609.6</v>
+      </c>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: screening master 2026-04-05
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:BW18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,62 +526,282 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>NetSales_TwoYearsPrior_Actual</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>OperatingProfit_TwoYearsPrior_Actual</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Profit_TwoYearsPrior_Actual</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>CashAndEquivalents_LatestFY</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Equity_LatestFY</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>PER_Trailing</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>PBR_Trailing</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>ROE_LatestYear</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>EquityToAssetRatio</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>NumberOfIssuedAndOutstandingSharesAtTheEndOfFiscalYearIncludingTreasuryStock</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>ShortMarginTradeVolume</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>LongMarginTradeVolume</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq01</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq02</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq03</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq04</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq05</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq06</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq07</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>LongMargin_WkSeq08</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq01</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq02</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq03</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq04</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq05</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq06</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq07</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>ShortMargin_WkSeq08</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>DiscretionaryInvestmentContractorName</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>ShortPositionsToSharesOutstandingRatio</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>ShortPositionsInSharesNumber</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>AvgDailyVolume5d</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq01</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq02</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq03</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq04</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq05</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq06</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq07</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>VolAvg5d_BlkSeq08</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>AvgDailyValue5d</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq01</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq02</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq03</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq04</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq05</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq06</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq07</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>ValAvg5d_BlkSeq08</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>AnnouncementDate</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>FiscalQuarter</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>FiscalYear</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>YFinance_Supplemented</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>ETLRunId</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>ETLStartedAtUTC</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>ETLStartedAtJST</t>
         </is>
       </c>
     </row>
@@ -623,7 +843,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -637,22 +857,140 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
-        <v>43000</v>
-      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="n">
-        <v>19600</v>
-      </c>
+      <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>43000</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>17000</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>16000</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>33000</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>45000</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>46000</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>43000</v>
+      </c>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="n">
+        <v>27200</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>14200</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>8600</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>13400</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>14800</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>22800</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>14000</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>13800</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>27200</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>1862000</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>1141800</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>677000</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>1074800</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>1151800</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>1615200</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>981400</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>947600</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>1862000</v>
+      </c>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -692,7 +1030,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2281</v>
+        <v>2297</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -706,22 +1044,148 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" t="n">
-        <v>227300</v>
-      </c>
-      <c r="W3" t="n">
-        <v>3235400</v>
-      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="n">
-        <v>2330460</v>
-      </c>
+      <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AD3" t="n">
+        <v>227300</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>3235400</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>3576100</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>3398500</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>3082900</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>3002100</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>2859200</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>2911500</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>3235400</v>
+      </c>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="n">
+        <v>762600</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>619800</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>650000</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>269900</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>275900</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>283300</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>227300</v>
+      </c>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>モルガン・スタンレーMUFG証券株式会社、Nomura International plc</t>
+        </is>
+      </c>
+      <c r="AW3" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>362132</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>2432780</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>2069240</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>1374680</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>1707980</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>2332920</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>1349720</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>3208240</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>2079840</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>2432780</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>5462913800</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>4184797840</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>2781072700</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>3574143180</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>5081670080</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>2747044860</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>7781799320</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>4889458760</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>5462913800</v>
+      </c>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW3" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -761,7 +1225,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -775,22 +1239,140 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" t="n">
-        <v>76600</v>
-      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="n">
-        <v>28680</v>
-      </c>
+      <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>76600</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>58100</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>57400</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>57100</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>57700</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>78800</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>80100</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>76600</v>
+      </c>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="n">
+        <v>26220</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>61580</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>79860</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>59380</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>68320</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>58860</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>79320</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>63700</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>26220</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>5820080</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>16253560</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>20766940</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>14569660</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>15978460</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>13221880</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>18258940</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>14797380</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>5820080</v>
+      </c>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -830,7 +1412,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>801</v>
+        <v>810</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -844,30 +1426,132 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="n">
-        <v>400</v>
-      </c>
-      <c r="W5" t="n">
-        <v>227900</v>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>野村證券株式会社</t>
-        </is>
-      </c>
-      <c r="Y5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>93360</v>
-      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
+      <c r="AD5" t="n">
+        <v>400</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>227900</v>
+      </c>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="n">
+        <v>222300</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>216400</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>204600</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>212600</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>227900</v>
+      </c>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>400</v>
+      </c>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>野村證券株式会社</t>
+        </is>
+      </c>
+      <c r="AW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>82320</v>
+      </c>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="n">
+        <v>1302366.666666667</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>300260</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>111260</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>117620</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>86180</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>82320</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>67033160</v>
+      </c>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="n">
+        <v>1383993266.666667</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>305469720</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>113793920</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>118662180</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>74449720</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>67033160</v>
+      </c>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW5" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -907,7 +1591,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -921,30 +1605,128 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="n">
-        <v>200400</v>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>野村證券株式会社</t>
-        </is>
-      </c>
-      <c r="Y6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>34480</v>
-      </c>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>200400</v>
+      </c>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="n">
+        <v>101900</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>201600</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>200600</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>183800</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>200400</v>
+      </c>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>野村證券株式会社</t>
+        </is>
+      </c>
+      <c r="AW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>32720</v>
+      </c>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="n">
+        <v>387740</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>57680</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>51540</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>40660</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>32720</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>41588180</v>
+      </c>
+      <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="n">
+        <v>626504680</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>81473640</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>69089120</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>50832820</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>41588180</v>
+      </c>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV6" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW6" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -984,7 +1766,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>684</v>
+        <v>675</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -998,22 +1780,92 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>49900</v>
-      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="n">
-        <v>81840</v>
-      </c>
+      <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
+      <c r="AD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>49900</v>
+      </c>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="n">
+        <v>49900</v>
+      </c>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="n">
+        <v>38440</v>
+      </c>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="n">
+        <v>406400</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>38440</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>26133940</v>
+      </c>
+      <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="n">
+        <v>316942333.3333333</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>26133940</v>
+      </c>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW7" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1053,7 +1905,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1067,22 +1919,92 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="W8" t="n">
-        <v>70700</v>
-      </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="n">
-        <v>268820</v>
-      </c>
+      <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AD8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>70700</v>
+      </c>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="n">
+        <v>70700</v>
+      </c>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="n">
+        <v>187780</v>
+      </c>
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="n">
+        <v>608533.3333333334</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>187780</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>129544760</v>
+      </c>
+      <c r="BI8" t="inlineStr"/>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="n">
+        <v>445297133.3333333</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>129544760</v>
+      </c>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1122,7 +2044,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1486</v>
+        <v>1349</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -1136,22 +2058,92 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
-      <c r="V9" t="n">
-        <v>0</v>
-      </c>
-      <c r="W9" t="n">
-        <v>408200</v>
-      </c>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="n">
-        <v>5316140</v>
-      </c>
+      <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr"/>
+      <c r="AD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>408200</v>
+      </c>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="n">
+        <v>408200</v>
+      </c>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="n">
+        <v>4071720</v>
+      </c>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="n">
+        <v>7132800</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>4071720</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>6341660460</v>
+      </c>
+      <c r="BI9" t="inlineStr"/>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="n">
+        <v>9710768600</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>6341660460</v>
+      </c>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV9" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW9" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1191,7 +2183,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1279</v>
+        <v>1200</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -1210,13 +2202,75 @@
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="n">
-        <v>1505100</v>
-      </c>
+      <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="n">
+        <v>917800</v>
+      </c>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="n">
+        <v>917800</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>1198242850</v>
+      </c>
+      <c r="BI10" t="inlineStr"/>
+      <c r="BJ10" t="inlineStr"/>
+      <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="n">
+        <v>1198242850</v>
+      </c>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV10" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW10" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1256,7 +2310,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>465</v>
+        <v>519</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -1275,13 +2329,75 @@
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="n">
-        <v>10922450</v>
-      </c>
+      <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="n">
+        <v>15476400</v>
+      </c>
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
+      <c r="BG11" t="n">
+        <v>15476400</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>7270849000</v>
+      </c>
+      <c r="BI11" t="inlineStr"/>
+      <c r="BJ11" t="inlineStr"/>
+      <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="inlineStr"/>
+      <c r="BP11" t="n">
+        <v>7270849000</v>
+      </c>
+      <c r="BQ11" t="inlineStr"/>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV11" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW11" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1321,7 +2437,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -1340,13 +2456,75 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="n">
-        <v>247150</v>
-      </c>
+      <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="n">
+        <v>245833.3333333333</v>
+      </c>
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
+      <c r="BB12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr"/>
+      <c r="BG12" t="n">
+        <v>245833.3333333333</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>102468266.6666667</v>
+      </c>
+      <c r="BI12" t="inlineStr"/>
+      <c r="BJ12" t="inlineStr"/>
+      <c r="BK12" t="inlineStr"/>
+      <c r="BL12" t="inlineStr"/>
+      <c r="BM12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
+      <c r="BO12" t="inlineStr"/>
+      <c r="BP12" t="n">
+        <v>102468266.6666667</v>
+      </c>
+      <c r="BQ12" t="inlineStr"/>
+      <c r="BR12" t="inlineStr"/>
+      <c r="BS12" t="inlineStr"/>
+      <c r="BT12" t="inlineStr"/>
+      <c r="BU12" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV12" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW12" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1386,7 +2564,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>932</v>
+        <v>921</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -1405,13 +2583,75 @@
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="n">
-        <v>155450</v>
-      </c>
+      <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="n">
+        <v>198733.3333333333</v>
+      </c>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="n">
+        <v>198733.3333333333</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>185306366.6666667</v>
+      </c>
+      <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="n">
+        <v>185306366.6666667</v>
+      </c>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr"/>
+      <c r="BU13" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW13" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1451,7 +2691,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1789</v>
+        <v>1874</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -1470,13 +2710,83 @@
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="n">
-        <v>195250</v>
-      </c>
+      <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>GOLDMAN SACHS INTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="AW14" t="n">
+        <v>0.0054</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>194633</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>206866.6666666667</v>
+      </c>
+      <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr"/>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="n">
+        <v>206866.6666666667</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>375613033.3333333</v>
+      </c>
+      <c r="BI14" t="inlineStr"/>
+      <c r="BJ14" t="inlineStr"/>
+      <c r="BK14" t="inlineStr"/>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="inlineStr"/>
+      <c r="BP14" t="n">
+        <v>375613033.3333333</v>
+      </c>
+      <c r="BQ14" t="inlineStr"/>
+      <c r="BR14" t="inlineStr"/>
+      <c r="BS14" t="inlineStr"/>
+      <c r="BT14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV14" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW14" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1516,7 +2826,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>434</v>
+        <v>422</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -1535,23 +2845,85 @@
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="n">
-        <v>2210850</v>
-      </c>
+      <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="n">
+        <v>2252600</v>
+      </c>
+      <c r="AZ15" t="inlineStr"/>
+      <c r="BA15" t="inlineStr"/>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="n">
+        <v>2252600</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>988981966.6666666</v>
+      </c>
+      <c r="BI15" t="inlineStr"/>
+      <c r="BJ15" t="inlineStr"/>
+      <c r="BK15" t="inlineStr"/>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
+      <c r="BO15" t="inlineStr"/>
+      <c r="BP15" t="n">
+        <v>988981966.6666666</v>
+      </c>
+      <c r="BQ15" t="inlineStr"/>
+      <c r="BR15" t="inlineStr"/>
+      <c r="BS15" t="inlineStr"/>
+      <c r="BT15" t="inlineStr"/>
+      <c r="BU15" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV15" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW15" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>548A</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>日本銀行</t>
+          <t>システムエグゼ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1561,12 +2933,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>銀行</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>銀行業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1598,23 +2970,77 @@
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="n">
-        <v>300</v>
-      </c>
+      <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr"/>
+      <c r="BH16" t="inlineStr"/>
+      <c r="BI16" t="inlineStr"/>
+      <c r="BJ16" t="inlineStr"/>
+      <c r="BK16" t="inlineStr"/>
+      <c r="BL16" t="inlineStr"/>
+      <c r="BM16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
+      <c r="BO16" t="inlineStr"/>
+      <c r="BP16" t="inlineStr"/>
+      <c r="BQ16" t="inlineStr"/>
+      <c r="BR16" t="inlineStr"/>
+      <c r="BS16" t="inlineStr"/>
+      <c r="BT16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV16" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW16" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9399</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+          <t>日本銀行</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1624,12 +3050,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>銀行</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>銀行業</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1643,9 +3069,7 @@
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>27</v>
-      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -1658,22 +3082,295 @@
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
-      <c r="V17" t="n">
-        <v>0</v>
-      </c>
-      <c r="W17" t="n">
-        <v>96080</v>
-      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="n">
-        <v>1764609.6</v>
-      </c>
+      <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
       <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="n">
+        <v>300</v>
+      </c>
+      <c r="AZ17" t="n">
+        <v>475</v>
+      </c>
+      <c r="BA17" t="n">
+        <v>925</v>
+      </c>
+      <c r="BB17" t="n">
+        <v>100</v>
+      </c>
+      <c r="BC17" t="n">
+        <v>450</v>
+      </c>
+      <c r="BD17" t="n">
+        <v>200</v>
+      </c>
+      <c r="BE17" t="n">
+        <v>300</v>
+      </c>
+      <c r="BF17" t="n">
+        <v>250</v>
+      </c>
+      <c r="BG17" t="n">
+        <v>300</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>7372000</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>12469250</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>25063500</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>2645000</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>11285000</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>4993250</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>7443250</v>
+      </c>
+      <c r="BO17" t="n">
+        <v>6260000</v>
+      </c>
+      <c r="BP17" t="n">
+        <v>7372000</v>
+      </c>
+      <c r="BQ17" t="inlineStr"/>
+      <c r="BR17" t="inlineStr"/>
+      <c r="BS17" t="inlineStr"/>
+      <c r="BT17" t="inlineStr"/>
+      <c r="BU17" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV17" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW17" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>9399</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>スタンダード</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>情報通信・サービスその他</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>情報･通信業</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>26</v>
+      </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>96080</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>202741</v>
+      </c>
+      <c r="AG18" t="n">
+        <v>204885</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>97185</v>
+      </c>
+      <c r="AI18" t="n">
+        <v>93675</v>
+      </c>
+      <c r="AJ18" t="n">
+        <v>126528</v>
+      </c>
+      <c r="AK18" t="n">
+        <v>99264</v>
+      </c>
+      <c r="AL18" t="n">
+        <v>96080</v>
+      </c>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="n">
+        <v>1913806.6</v>
+      </c>
+      <c r="AZ18" t="n">
+        <v>3353161.6</v>
+      </c>
+      <c r="BA18" t="n">
+        <v>12912269</v>
+      </c>
+      <c r="BB18" t="n">
+        <v>7299611.6</v>
+      </c>
+      <c r="BC18" t="n">
+        <v>2742294</v>
+      </c>
+      <c r="BD18" t="n">
+        <v>3912781</v>
+      </c>
+      <c r="BE18" t="n">
+        <v>4714386.8</v>
+      </c>
+      <c r="BF18" t="n">
+        <v>2238110.2</v>
+      </c>
+      <c r="BG18" t="n">
+        <v>1913806.6</v>
+      </c>
+      <c r="BH18" t="n">
+        <v>52170691.2</v>
+      </c>
+      <c r="BI18" t="n">
+        <v>134552872</v>
+      </c>
+      <c r="BJ18" t="n">
+        <v>314646947.2</v>
+      </c>
+      <c r="BK18" t="n">
+        <v>226772440</v>
+      </c>
+      <c r="BL18" t="n">
+        <v>69693452.8</v>
+      </c>
+      <c r="BM18" t="n">
+        <v>114743178.6</v>
+      </c>
+      <c r="BN18" t="n">
+        <v>148128099</v>
+      </c>
+      <c r="BO18" t="n">
+        <v>67164683.59999999</v>
+      </c>
+      <c r="BP18" t="n">
+        <v>52170691.2</v>
+      </c>
+      <c r="BQ18" t="inlineStr"/>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr">
+        <is>
+          <t>20260405-120859</t>
+        </is>
+      </c>
+      <c r="BV18" t="inlineStr">
+        <is>
+          <t>2026-04-05T03:08:59+00:00</t>
+        </is>
+      </c>
+      <c r="BW18" t="inlineStr">
+        <is>
+          <t>2026-04-05T12:08:59+09:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: screening master 2026-04-06
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -967,58 +967,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>27200</v>
+        <v>25400</v>
       </c>
       <c r="BH2" t="n">
+        <v>15400</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>10400</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>15400</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>11000</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>25800</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>15800</v>
+      </c>
+      <c r="BN2" t="n">
         <v>14200</v>
       </c>
-      <c r="BI2" t="n">
-        <v>8600</v>
-      </c>
-      <c r="BJ2" t="n">
-        <v>13400</v>
-      </c>
-      <c r="BK2" t="n">
-        <v>14800</v>
-      </c>
-      <c r="BL2" t="n">
-        <v>22800</v>
-      </c>
-      <c r="BM2" t="n">
-        <v>14000</v>
-      </c>
-      <c r="BN2" t="n">
-        <v>13800</v>
-      </c>
       <c r="BO2" t="n">
-        <v>27200</v>
+        <v>25400</v>
       </c>
       <c r="BP2" t="n">
-        <v>1862000</v>
+        <v>1778000</v>
       </c>
       <c r="BQ2" t="n">
-        <v>1141800</v>
+        <v>1231800</v>
       </c>
       <c r="BR2" t="n">
-        <v>677000</v>
+        <v>831600</v>
       </c>
       <c r="BS2" t="n">
-        <v>1074800</v>
+        <v>1212800</v>
       </c>
       <c r="BT2" t="n">
-        <v>1151800</v>
+        <v>852400</v>
       </c>
       <c r="BU2" t="n">
-        <v>1615200</v>
+        <v>1810200</v>
       </c>
       <c r="BV2" t="n">
-        <v>981400</v>
+        <v>1101600</v>
       </c>
       <c r="BW2" t="n">
-        <v>947600</v>
+        <v>955400</v>
       </c>
       <c r="BX2" t="n">
-        <v>1862000</v>
+        <v>1778000</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1026,17 +1026,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2297</v>
+        <v>2413</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1186,58 +1186,58 @@
         <v>362132</v>
       </c>
       <c r="BG3" t="n">
-        <v>2432780</v>
+        <v>2349540</v>
       </c>
       <c r="BH3" t="n">
-        <v>2069240</v>
+        <v>1946920</v>
       </c>
       <c r="BI3" t="n">
-        <v>1374680</v>
+        <v>1159980</v>
       </c>
       <c r="BJ3" t="n">
-        <v>1707980</v>
+        <v>2018340</v>
       </c>
       <c r="BK3" t="n">
-        <v>2332920</v>
+        <v>2095360</v>
       </c>
       <c r="BL3" t="n">
-        <v>1349720</v>
+        <v>1645340</v>
       </c>
       <c r="BM3" t="n">
-        <v>3208240</v>
+        <v>3224160</v>
       </c>
       <c r="BN3" t="n">
-        <v>2079840</v>
+        <v>2021360</v>
       </c>
       <c r="BO3" t="n">
-        <v>2432780</v>
+        <v>2349540</v>
       </c>
       <c r="BP3" t="n">
-        <v>5462913800</v>
+        <v>5396505260</v>
       </c>
       <c r="BQ3" t="n">
-        <v>4184797840</v>
+        <v>3963348740</v>
       </c>
       <c r="BR3" t="n">
-        <v>2781072700</v>
+        <v>2343385220</v>
       </c>
       <c r="BS3" t="n">
-        <v>3574143180</v>
+        <v>4290307920</v>
       </c>
       <c r="BT3" t="n">
-        <v>5081670080</v>
+        <v>4517672440</v>
       </c>
       <c r="BU3" t="n">
-        <v>2747044860</v>
+        <v>3430335160</v>
       </c>
       <c r="BV3" t="n">
-        <v>7781799320</v>
+        <v>7888006660</v>
       </c>
       <c r="BW3" t="n">
-        <v>4889458760</v>
+        <v>4656243060</v>
       </c>
       <c r="BX3" t="n">
-        <v>5462913800</v>
+        <v>5396505260</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1245,17 +1245,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1297,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1381,58 +1381,58 @@
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="n">
-        <v>26220</v>
+        <v>16280</v>
       </c>
       <c r="BH4" t="n">
-        <v>61580</v>
+        <v>64680</v>
       </c>
       <c r="BI4" t="n">
-        <v>79860</v>
+        <v>75940</v>
       </c>
       <c r="BJ4" t="n">
-        <v>59380</v>
+        <v>63460</v>
       </c>
       <c r="BK4" t="n">
-        <v>68320</v>
+        <v>68420</v>
       </c>
       <c r="BL4" t="n">
-        <v>58860</v>
+        <v>58460</v>
       </c>
       <c r="BM4" t="n">
-        <v>79320</v>
+        <v>101700</v>
       </c>
       <c r="BN4" t="n">
-        <v>63700</v>
+        <v>40220</v>
       </c>
       <c r="BO4" t="n">
-        <v>26220</v>
+        <v>16280</v>
       </c>
       <c r="BP4" t="n">
-        <v>5820080</v>
+        <v>3639380</v>
       </c>
       <c r="BQ4" t="n">
-        <v>16253560</v>
+        <v>17128720</v>
       </c>
       <c r="BR4" t="n">
-        <v>20766940</v>
+        <v>19566000</v>
       </c>
       <c r="BS4" t="n">
-        <v>14569660</v>
+        <v>15580660</v>
       </c>
       <c r="BT4" t="n">
-        <v>15978460</v>
+        <v>15720080</v>
       </c>
       <c r="BU4" t="n">
-        <v>13221880</v>
+        <v>13031980</v>
       </c>
       <c r="BV4" t="n">
-        <v>18258940</v>
+        <v>23672580</v>
       </c>
       <c r="BW4" t="n">
-        <v>14797380</v>
+        <v>9151220</v>
       </c>
       <c r="BX4" t="n">
-        <v>5820080</v>
+        <v>3639380</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1440,17 +1440,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1588,50 +1588,50 @@
         <v>0</v>
       </c>
       <c r="BG5" t="n">
-        <v>82320</v>
+        <v>61860</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="n">
-        <v>1302366.666666667</v>
+        <v>1096975</v>
       </c>
       <c r="BK5" t="n">
-        <v>300260</v>
+        <v>229200</v>
       </c>
       <c r="BL5" t="n">
-        <v>111260</v>
+        <v>104900</v>
       </c>
       <c r="BM5" t="n">
-        <v>117620</v>
+        <v>127240</v>
       </c>
       <c r="BN5" t="n">
-        <v>86180</v>
+        <v>82900</v>
       </c>
       <c r="BO5" t="n">
-        <v>82320</v>
+        <v>61860</v>
       </c>
       <c r="BP5" t="n">
-        <v>67033160</v>
+        <v>50250980</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="inlineStr"/>
       <c r="BS5" t="n">
-        <v>1383993266.666667</v>
+        <v>1152932450</v>
       </c>
       <c r="BT5" t="n">
-        <v>305469720</v>
+        <v>238575980</v>
       </c>
       <c r="BU5" t="n">
-        <v>113793920</v>
+        <v>108578560</v>
       </c>
       <c r="BV5" t="n">
-        <v>118662180</v>
+        <v>123609800</v>
       </c>
       <c r="BW5" t="n">
-        <v>74449720</v>
+        <v>70208720</v>
       </c>
       <c r="BX5" t="n">
-        <v>67033160</v>
+        <v>50250980</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1639,17 +1639,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1290</v>
+        <v>1295</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1785,46 +1785,50 @@
         <v>0</v>
       </c>
       <c r="BG6" t="n">
-        <v>32720</v>
+        <v>31640</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="inlineStr"/>
+      <c r="BJ6" t="n">
+        <v>1061600</v>
+      </c>
       <c r="BK6" t="n">
-        <v>387740</v>
+        <v>190460</v>
       </c>
       <c r="BL6" t="n">
-        <v>57680</v>
+        <v>54580</v>
       </c>
       <c r="BM6" t="n">
-        <v>51540</v>
+        <v>50760</v>
       </c>
       <c r="BN6" t="n">
-        <v>40660</v>
+        <v>37240</v>
       </c>
       <c r="BO6" t="n">
-        <v>32720</v>
+        <v>31640</v>
       </c>
       <c r="BP6" t="n">
-        <v>41588180</v>
+        <v>40719960</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
-      <c r="BS6" t="inlineStr"/>
+      <c r="BS6" t="n">
+        <v>1824386500</v>
+      </c>
       <c r="BT6" t="n">
-        <v>626504680</v>
+        <v>283021740</v>
       </c>
       <c r="BU6" t="n">
-        <v>81473640</v>
+        <v>76531300</v>
       </c>
       <c r="BV6" t="n">
-        <v>69089120</v>
+        <v>66217080</v>
       </c>
       <c r="BW6" t="n">
-        <v>50832820</v>
+        <v>46786260</v>
       </c>
       <c r="BX6" t="n">
-        <v>41588180</v>
+        <v>40719960</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1832,17 +1836,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1948,7 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>38440</v>
+        <v>30900</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1953,13 +1957,13 @@
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="inlineStr"/>
       <c r="BN7" t="n">
-        <v>406400</v>
+        <v>318525</v>
       </c>
       <c r="BO7" t="n">
-        <v>38440</v>
+        <v>30900</v>
       </c>
       <c r="BP7" t="n">
-        <v>26133940</v>
+        <v>21013720</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
@@ -1968,10 +1972,10 @@
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="n">
-        <v>316942333.3333333</v>
+        <v>247000550</v>
       </c>
       <c r="BX7" t="n">
-        <v>26133940</v>
+        <v>21013720</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -1979,17 +1983,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2035,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>686</v>
+        <v>665</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2091,7 +2095,7 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
-        <v>187780</v>
+        <v>140100</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
@@ -2100,13 +2104,13 @@
       <c r="BL8" t="inlineStr"/>
       <c r="BM8" t="inlineStr"/>
       <c r="BN8" t="n">
-        <v>608533.3333333334</v>
+        <v>540325</v>
       </c>
       <c r="BO8" t="n">
-        <v>187780</v>
+        <v>140100</v>
       </c>
       <c r="BP8" t="n">
-        <v>129544760</v>
+        <v>98474520</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
@@ -2115,10 +2119,10 @@
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="inlineStr"/>
       <c r="BW8" t="n">
-        <v>445297133.3333333</v>
+        <v>389225050</v>
       </c>
       <c r="BX8" t="n">
-        <v>129544760</v>
+        <v>98474520</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2126,17 +2130,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2182,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1349</v>
+        <v>1362</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2238,7 +2242,7 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>4071720</v>
+        <v>2620900</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
@@ -2247,13 +2251,13 @@
       <c r="BL9" t="inlineStr"/>
       <c r="BM9" t="inlineStr"/>
       <c r="BN9" t="n">
-        <v>7132800</v>
+        <v>7535550</v>
       </c>
       <c r="BO9" t="n">
-        <v>4071720</v>
+        <v>2620900</v>
       </c>
       <c r="BP9" t="n">
-        <v>6341660460</v>
+        <v>3937584140</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
@@ -2262,10 +2266,10 @@
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="inlineStr"/>
       <c r="BW9" t="n">
-        <v>9710768600</v>
+        <v>11342836750</v>
       </c>
       <c r="BX9" t="n">
-        <v>6341660460</v>
+        <v>3937584140</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2273,17 +2277,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2329,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1200</v>
+        <v>1184</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2377,7 +2381,7 @@
       <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="n">
-        <v>917800</v>
+        <v>675266.6666666666</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2387,10 +2391,10 @@
       <c r="BM10" t="inlineStr"/>
       <c r="BN10" t="inlineStr"/>
       <c r="BO10" t="n">
-        <v>917800</v>
+        <v>675266.6666666666</v>
       </c>
       <c r="BP10" t="n">
-        <v>1198242850</v>
+        <v>873361533.3333334</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2400,7 +2404,7 @@
       <c r="BV10" t="inlineStr"/>
       <c r="BW10" t="inlineStr"/>
       <c r="BX10" t="n">
-        <v>1198242850</v>
+        <v>873361533.3333334</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2408,17 +2412,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2464,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>519</v>
+        <v>475</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2512,7 +2516,7 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>15476400</v>
+        <v>22304225</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2522,10 +2526,10 @@
       <c r="BM11" t="inlineStr"/>
       <c r="BN11" t="inlineStr"/>
       <c r="BO11" t="n">
-        <v>15476400</v>
+        <v>22304225</v>
       </c>
       <c r="BP11" t="n">
-        <v>7270849000</v>
+        <v>10645521900</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2535,7 +2539,7 @@
       <c r="BV11" t="inlineStr"/>
       <c r="BW11" t="inlineStr"/>
       <c r="BX11" t="n">
-        <v>7270849000</v>
+        <v>10645521900</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2543,17 +2547,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2599,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>429</v>
+        <v>417</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2635,9 +2639,17 @@
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="inlineStr"/>
       <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>GOLDMAN SACHS INTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="AW12" t="n">
+        <v>0.0053</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>382685</v>
+      </c>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
       <c r="BA12" t="inlineStr"/>
@@ -2647,7 +2659,7 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>245833.3333333333</v>
+        <v>248475</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2657,10 +2669,10 @@
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="inlineStr"/>
       <c r="BO12" t="n">
-        <v>245833.3333333333</v>
+        <v>248475</v>
       </c>
       <c r="BP12" t="n">
-        <v>102468266.6666667</v>
+        <v>103489250</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2670,7 +2682,7 @@
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="inlineStr"/>
       <c r="BX12" t="n">
-        <v>102468266.6666667</v>
+        <v>103489250</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2678,17 +2690,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2742,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>921</v>
+        <v>932</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2782,7 +2794,7 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="n">
-        <v>198733.3333333333</v>
+        <v>171850</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2792,10 +2804,10 @@
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="inlineStr"/>
       <c r="BO13" t="n">
-        <v>198733.3333333333</v>
+        <v>171850</v>
       </c>
       <c r="BP13" t="n">
-        <v>185306366.6666667</v>
+        <v>160315700</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2805,7 +2817,7 @@
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="inlineStr"/>
       <c r="BX13" t="n">
-        <v>185306366.6666667</v>
+        <v>160315700</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2813,17 +2825,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2877,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1874</v>
+        <v>1861</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -2927,7 +2939,7 @@
         <v>194633</v>
       </c>
       <c r="BG14" t="n">
-        <v>206866.6666666667</v>
+        <v>201300</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -2937,10 +2949,10 @@
       <c r="BM14" t="inlineStr"/>
       <c r="BN14" t="inlineStr"/>
       <c r="BO14" t="n">
-        <v>206866.6666666667</v>
+        <v>201300</v>
       </c>
       <c r="BP14" t="n">
-        <v>375613033.3333333</v>
+        <v>366972875</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -2950,7 +2962,7 @@
       <c r="BV14" t="inlineStr"/>
       <c r="BW14" t="inlineStr"/>
       <c r="BX14" t="n">
-        <v>375613033.3333333</v>
+        <v>366972875</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -2958,17 +2970,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3022,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -3062,7 +3074,7 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>2252600</v>
+        <v>2140650</v>
       </c>
       <c r="BH15" t="inlineStr"/>
       <c r="BI15" t="inlineStr"/>
@@ -3072,10 +3084,10 @@
       <c r="BM15" t="inlineStr"/>
       <c r="BN15" t="inlineStr"/>
       <c r="BO15" t="n">
-        <v>2252600</v>
+        <v>2140650</v>
       </c>
       <c r="BP15" t="n">
-        <v>988981966.6666666</v>
+        <v>932730175</v>
       </c>
       <c r="BQ15" t="inlineStr"/>
       <c r="BR15" t="inlineStr"/>
@@ -3085,7 +3097,7 @@
       <c r="BV15" t="inlineStr"/>
       <c r="BW15" t="inlineStr"/>
       <c r="BX15" t="n">
-        <v>988981966.6666666</v>
+        <v>932730175</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3093,17 +3105,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3156,9 @@
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>951</v>
+      </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
@@ -3194,7 +3208,9 @@
       <c r="BD16" t="inlineStr"/>
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
-      <c r="BG16" t="inlineStr"/>
+      <c r="BG16" t="n">
+        <v>2057900</v>
+      </c>
       <c r="BH16" t="inlineStr"/>
       <c r="BI16" t="inlineStr"/>
       <c r="BJ16" t="inlineStr"/>
@@ -3202,8 +3218,12 @@
       <c r="BL16" t="inlineStr"/>
       <c r="BM16" t="inlineStr"/>
       <c r="BN16" t="inlineStr"/>
-      <c r="BO16" t="inlineStr"/>
-      <c r="BP16" t="inlineStr"/>
+      <c r="BO16" t="n">
+        <v>2057900</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>2105307200</v>
+      </c>
       <c r="BQ16" t="inlineStr"/>
       <c r="BR16" t="inlineStr"/>
       <c r="BS16" t="inlineStr"/>
@@ -3211,24 +3231,26 @@
       <c r="BU16" t="inlineStr"/>
       <c r="BV16" t="inlineStr"/>
       <c r="BW16" t="inlineStr"/>
-      <c r="BX16" t="inlineStr"/>
+      <c r="BX16" t="n">
+        <v>2105307200</v>
+      </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
       <c r="CA16" t="inlineStr"/>
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3291,9 @@
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>25200</v>
+      </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -3320,13 +3344,13 @@
       <c r="BE17" t="inlineStr"/>
       <c r="BF17" t="inlineStr"/>
       <c r="BG17" t="n">
-        <v>300</v>
+        <v>266.6666666666667</v>
       </c>
       <c r="BH17" t="n">
-        <v>475</v>
+        <v>440</v>
       </c>
       <c r="BI17" t="n">
-        <v>925</v>
+        <v>875</v>
       </c>
       <c r="BJ17" t="n">
         <v>100</v>
@@ -3335,43 +3359,43 @@
         <v>450</v>
       </c>
       <c r="BL17" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="BM17" t="n">
-        <v>300</v>
+        <v>166.6666666666667</v>
       </c>
       <c r="BN17" t="n">
         <v>250</v>
       </c>
       <c r="BO17" t="n">
-        <v>300</v>
+        <v>266.6666666666667</v>
       </c>
       <c r="BP17" t="n">
-        <v>7372000</v>
+        <v>6588333.333333333</v>
       </c>
       <c r="BQ17" t="n">
-        <v>12469250</v>
+        <v>11565600</v>
       </c>
       <c r="BR17" t="n">
-        <v>25063500</v>
+        <v>23735750</v>
       </c>
       <c r="BS17" t="n">
-        <v>2645000</v>
+        <v>2650000</v>
       </c>
       <c r="BT17" t="n">
         <v>11285000</v>
       </c>
       <c r="BU17" t="n">
-        <v>4993250</v>
+        <v>7486400</v>
       </c>
       <c r="BV17" t="n">
-        <v>7443250</v>
+        <v>4104666.666666667</v>
       </c>
       <c r="BW17" t="n">
         <v>6260000</v>
       </c>
       <c r="BX17" t="n">
-        <v>7372000</v>
+        <v>6588333.333333333</v>
       </c>
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
@@ -3379,17 +3403,17 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>
@@ -3515,58 +3539,58 @@
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="n">
-        <v>1913806.6</v>
+        <v>1960023.6</v>
       </c>
       <c r="BH18" t="n">
-        <v>3353161.6</v>
+        <v>4774465.6</v>
       </c>
       <c r="BI18" t="n">
-        <v>12912269</v>
+        <v>13931419.2</v>
       </c>
       <c r="BJ18" t="n">
-        <v>7299611.6</v>
+        <v>5104435.2</v>
       </c>
       <c r="BK18" t="n">
-        <v>2742294</v>
+        <v>3130213.4</v>
       </c>
       <c r="BL18" t="n">
-        <v>3912781</v>
+        <v>3424175.2</v>
       </c>
       <c r="BM18" t="n">
-        <v>4714386.8</v>
+        <v>4747035.2</v>
       </c>
       <c r="BN18" t="n">
-        <v>2238110.2</v>
+        <v>1966370.8</v>
       </c>
       <c r="BO18" t="n">
-        <v>1913806.6</v>
+        <v>1960023.6</v>
       </c>
       <c r="BP18" t="n">
-        <v>52170691.2</v>
+        <v>52706922.8</v>
       </c>
       <c r="BQ18" t="n">
-        <v>134552872</v>
+        <v>170454411.4</v>
       </c>
       <c r="BR18" t="n">
-        <v>314646947.2</v>
+        <v>356289258</v>
       </c>
       <c r="BS18" t="n">
-        <v>226772440</v>
+        <v>147240261</v>
       </c>
       <c r="BT18" t="n">
-        <v>69693452.8</v>
+        <v>83366454.8</v>
       </c>
       <c r="BU18" t="n">
-        <v>114743178.6</v>
+        <v>100089101.6</v>
       </c>
       <c r="BV18" t="n">
-        <v>148128099</v>
+        <v>150288273.6</v>
       </c>
       <c r="BW18" t="n">
-        <v>67164683.59999999</v>
+        <v>58329980.2</v>
       </c>
       <c r="BX18" t="n">
-        <v>52170691.2</v>
+        <v>52706922.8</v>
       </c>
       <c r="BY18" t="inlineStr"/>
       <c r="BZ18" t="inlineStr"/>
@@ -3574,17 +3598,17 @@
       <c r="CB18" t="inlineStr"/>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>20260405-190048</t>
+          <t>20260406-190042</t>
         </is>
       </c>
       <c r="CD18" t="inlineStr">
         <is>
-          <t>2026-04-05T10:00:48+00:00</t>
+          <t>2026-04-06T10:00:42+00:00</t>
         </is>
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>2026-04-05T19:00:48+09:00</t>
+          <t>2026-04-06T19:00:42+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-07
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE18"/>
+  <dimension ref="A1:CE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -909,7 +909,7 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>43000</v>
+        <v>31000</v>
       </c>
       <c r="AF2" t="n">
         <v>17000</v>
@@ -932,7 +932,9 @@
       <c r="AL2" t="n">
         <v>43000</v>
       </c>
-      <c r="AM2" t="inlineStr"/>
+      <c r="AM2" t="n">
+        <v>31000</v>
+      </c>
       <c r="AN2" t="n">
         <v>0</v>
       </c>
@@ -954,7 +956,9 @@
       <c r="AT2" t="n">
         <v>0</v>
       </c>
-      <c r="AU2" t="inlineStr"/>
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
@@ -967,58 +971,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>25400</v>
+        <v>26400</v>
       </c>
       <c r="BH2" t="n">
-        <v>15400</v>
+        <v>17600</v>
       </c>
       <c r="BI2" t="n">
-        <v>10400</v>
+        <v>9600</v>
       </c>
       <c r="BJ2" t="n">
-        <v>15400</v>
+        <v>16200</v>
       </c>
       <c r="BK2" t="n">
-        <v>11000</v>
+        <v>22400</v>
       </c>
       <c r="BL2" t="n">
-        <v>25800</v>
+        <v>14200</v>
       </c>
       <c r="BM2" t="n">
-        <v>15800</v>
+        <v>14000</v>
       </c>
       <c r="BN2" t="n">
-        <v>14200</v>
+        <v>16000</v>
       </c>
       <c r="BO2" t="n">
-        <v>25400</v>
+        <v>26400</v>
       </c>
       <c r="BP2" t="n">
-        <v>1778000</v>
+        <v>1869600</v>
       </c>
       <c r="BQ2" t="n">
-        <v>1231800</v>
+        <v>1401800</v>
       </c>
       <c r="BR2" t="n">
-        <v>831600</v>
+        <v>772000</v>
       </c>
       <c r="BS2" t="n">
-        <v>1212800</v>
+        <v>1272800</v>
       </c>
       <c r="BT2" t="n">
-        <v>852400</v>
+        <v>1628000</v>
       </c>
       <c r="BU2" t="n">
-        <v>1810200</v>
+        <v>993800</v>
       </c>
       <c r="BV2" t="n">
-        <v>1101600</v>
+        <v>979400</v>
       </c>
       <c r="BW2" t="n">
-        <v>955400</v>
+        <v>1072200</v>
       </c>
       <c r="BX2" t="n">
-        <v>1778000</v>
+        <v>1869600</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1026,17 +1030,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1082,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2413</v>
+        <v>2454</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1101,10 +1105,10 @@
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="n">
-        <v>227300</v>
+        <v>236100</v>
       </c>
       <c r="AE3" t="n">
-        <v>3235400</v>
+        <v>3149100</v>
       </c>
       <c r="AF3" t="n">
         <v>3576100</v>
@@ -1127,7 +1131,9 @@
       <c r="AL3" t="n">
         <v>3235400</v>
       </c>
-      <c r="AM3" t="inlineStr"/>
+      <c r="AM3" t="n">
+        <v>3149100</v>
+      </c>
       <c r="AN3" t="n">
         <v>762600</v>
       </c>
@@ -1149,7 +1155,9 @@
       <c r="AT3" t="n">
         <v>227300</v>
       </c>
-      <c r="AU3" t="inlineStr"/>
+      <c r="AU3" t="n">
+        <v>236100</v>
+      </c>
       <c r="AV3" t="inlineStr">
         <is>
           <t>モルガン・スタンレーMUFG証券株式会社、Nomura International plc</t>
@@ -1186,58 +1194,58 @@
         <v>362132</v>
       </c>
       <c r="BG3" t="n">
-        <v>2349540</v>
+        <v>2399940</v>
       </c>
       <c r="BH3" t="n">
-        <v>1946920</v>
+        <v>1829140</v>
       </c>
       <c r="BI3" t="n">
-        <v>1159980</v>
+        <v>1128420</v>
       </c>
       <c r="BJ3" t="n">
-        <v>2018340</v>
+        <v>2249300</v>
       </c>
       <c r="BK3" t="n">
-        <v>2095360</v>
+        <v>2068040</v>
       </c>
       <c r="BL3" t="n">
-        <v>1645340</v>
+        <v>1558240</v>
       </c>
       <c r="BM3" t="n">
-        <v>3224160</v>
+        <v>3241660</v>
       </c>
       <c r="BN3" t="n">
-        <v>2021360</v>
+        <v>2032180</v>
       </c>
       <c r="BO3" t="n">
-        <v>2349540</v>
+        <v>2399940</v>
       </c>
       <c r="BP3" t="n">
-        <v>5396505260</v>
+        <v>5654626740</v>
       </c>
       <c r="BQ3" t="n">
-        <v>3963348740</v>
+        <v>3725834940</v>
       </c>
       <c r="BR3" t="n">
-        <v>2343385220</v>
+        <v>2306432200</v>
       </c>
       <c r="BS3" t="n">
-        <v>4290307920</v>
+        <v>4869925960</v>
       </c>
       <c r="BT3" t="n">
-        <v>4517672440</v>
+        <v>4302787140</v>
       </c>
       <c r="BU3" t="n">
-        <v>3430335160</v>
+        <v>3372377580</v>
       </c>
       <c r="BV3" t="n">
-        <v>7888006660</v>
+        <v>7930500380</v>
       </c>
       <c r="BW3" t="n">
-        <v>4656243060</v>
+        <v>4614806860</v>
       </c>
       <c r="BX3" t="n">
-        <v>5396505260</v>
+        <v>5654626740</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1245,17 +1253,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1297,7 +1305,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1323,7 +1331,7 @@
         <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>76600</v>
+        <v>76800</v>
       </c>
       <c r="AF4" t="n">
         <v>58100</v>
@@ -1346,7 +1354,9 @@
       <c r="AL4" t="n">
         <v>76600</v>
       </c>
-      <c r="AM4" t="inlineStr"/>
+      <c r="AM4" t="n">
+        <v>76800</v>
+      </c>
       <c r="AN4" t="n">
         <v>0</v>
       </c>
@@ -1368,7 +1378,9 @@
       <c r="AT4" t="n">
         <v>0</v>
       </c>
-      <c r="AU4" t="inlineStr"/>
+      <c r="AU4" t="n">
+        <v>0</v>
+      </c>
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="inlineStr"/>
@@ -1381,58 +1393,58 @@
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="n">
-        <v>16280</v>
+        <v>13980</v>
       </c>
       <c r="BH4" t="n">
-        <v>64680</v>
+        <v>82560</v>
       </c>
       <c r="BI4" t="n">
-        <v>75940</v>
+        <v>64700</v>
       </c>
       <c r="BJ4" t="n">
-        <v>63460</v>
+        <v>59380</v>
       </c>
       <c r="BK4" t="n">
-        <v>68420</v>
+        <v>77740</v>
       </c>
       <c r="BL4" t="n">
-        <v>58460</v>
+        <v>48480</v>
       </c>
       <c r="BM4" t="n">
-        <v>101700</v>
+        <v>103840</v>
       </c>
       <c r="BN4" t="n">
-        <v>40220</v>
+        <v>33720</v>
       </c>
       <c r="BO4" t="n">
-        <v>16280</v>
+        <v>13980</v>
       </c>
       <c r="BP4" t="n">
-        <v>3639380</v>
+        <v>3137240</v>
       </c>
       <c r="BQ4" t="n">
-        <v>17128720</v>
+        <v>21765620</v>
       </c>
       <c r="BR4" t="n">
-        <v>19566000</v>
+        <v>16438180</v>
       </c>
       <c r="BS4" t="n">
-        <v>15580660</v>
+        <v>14522900</v>
       </c>
       <c r="BT4" t="n">
-        <v>15720080</v>
+        <v>17546800</v>
       </c>
       <c r="BU4" t="n">
-        <v>13031980</v>
+        <v>10831060</v>
       </c>
       <c r="BV4" t="n">
-        <v>23672580</v>
+        <v>24264960</v>
       </c>
       <c r="BW4" t="n">
-        <v>9151220</v>
+        <v>7616900</v>
       </c>
       <c r="BX4" t="n">
-        <v>3639380</v>
+        <v>3137240</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1440,17 +1452,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1504,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>813</v>
+        <v>842</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1515,10 +1527,10 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>227900</v>
+        <v>234400</v>
       </c>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
@@ -1537,7 +1549,9 @@
       <c r="AL5" t="n">
         <v>227900</v>
       </c>
-      <c r="AM5" t="inlineStr"/>
+      <c r="AM5" t="n">
+        <v>234400</v>
+      </c>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="n">
@@ -1555,7 +1569,9 @@
       <c r="AT5" t="n">
         <v>400</v>
       </c>
-      <c r="AU5" t="inlineStr"/>
+      <c r="AU5" t="n">
+        <v>0</v>
+      </c>
       <c r="AV5" t="inlineStr">
         <is>
           <t>野村證券株式会社</t>
@@ -1588,50 +1604,50 @@
         <v>0</v>
       </c>
       <c r="BG5" t="n">
-        <v>61860</v>
+        <v>54260</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="n">
-        <v>1096975</v>
+        <v>971220</v>
       </c>
       <c r="BK5" t="n">
-        <v>229200</v>
+        <v>162400</v>
       </c>
       <c r="BL5" t="n">
-        <v>104900</v>
+        <v>94040</v>
       </c>
       <c r="BM5" t="n">
-        <v>127240</v>
+        <v>125360</v>
       </c>
       <c r="BN5" t="n">
-        <v>82900</v>
+        <v>86440</v>
       </c>
       <c r="BO5" t="n">
-        <v>61860</v>
+        <v>54260</v>
       </c>
       <c r="BP5" t="n">
-        <v>50250980</v>
+        <v>44134900</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="inlineStr"/>
       <c r="BS5" t="n">
-        <v>1152932450</v>
+        <v>1018630620</v>
       </c>
       <c r="BT5" t="n">
-        <v>238575980</v>
+        <v>168932740</v>
       </c>
       <c r="BU5" t="n">
-        <v>108578560</v>
+        <v>98665760</v>
       </c>
       <c r="BV5" t="n">
-        <v>123609800</v>
+        <v>119082120</v>
       </c>
       <c r="BW5" t="n">
-        <v>70208720</v>
+        <v>72462920</v>
       </c>
       <c r="BX5" t="n">
-        <v>50250980</v>
+        <v>44134900</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1639,17 +1655,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1733,7 @@
         <v>0</v>
       </c>
       <c r="AE6" t="n">
-        <v>200400</v>
+        <v>183000</v>
       </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
@@ -1736,7 +1752,9 @@
       <c r="AL6" t="n">
         <v>200400</v>
       </c>
-      <c r="AM6" t="inlineStr"/>
+      <c r="AM6" t="n">
+        <v>183000</v>
+      </c>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="n">
@@ -1754,7 +1772,9 @@
       <c r="AT6" t="n">
         <v>0</v>
       </c>
-      <c r="AU6" t="inlineStr"/>
+      <c r="AU6" t="n">
+        <v>0</v>
+      </c>
       <c r="AV6" t="inlineStr">
         <is>
           <t>野村證券株式会社</t>
@@ -1785,50 +1805,50 @@
         <v>0</v>
       </c>
       <c r="BG6" t="n">
-        <v>31640</v>
+        <v>28820</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="n">
-        <v>1061600</v>
+        <v>663400</v>
       </c>
       <c r="BK6" t="n">
-        <v>190460</v>
+        <v>155060</v>
       </c>
       <c r="BL6" t="n">
-        <v>54580</v>
+        <v>46960</v>
       </c>
       <c r="BM6" t="n">
-        <v>50760</v>
+        <v>46160</v>
       </c>
       <c r="BN6" t="n">
-        <v>37240</v>
+        <v>37800</v>
       </c>
       <c r="BO6" t="n">
-        <v>31640</v>
+        <v>28820</v>
       </c>
       <c r="BP6" t="n">
-        <v>40719960</v>
+        <v>37297620</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="n">
-        <v>1824386500</v>
+        <v>1125348550</v>
       </c>
       <c r="BT6" t="n">
-        <v>283021740</v>
+        <v>222315800</v>
       </c>
       <c r="BU6" t="n">
-        <v>76531300</v>
+        <v>65570020</v>
       </c>
       <c r="BV6" t="n">
-        <v>66217080</v>
+        <v>59230440</v>
       </c>
       <c r="BW6" t="n">
-        <v>46786260</v>
+        <v>47679980</v>
       </c>
       <c r="BX6" t="n">
-        <v>40719960</v>
+        <v>37297620</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1836,17 +1856,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1888,7 +1908,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>675</v>
+        <v>685</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1914,7 +1934,7 @@
         <v>0</v>
       </c>
       <c r="AE7" t="n">
-        <v>49900</v>
+        <v>56200</v>
       </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
@@ -1925,7 +1945,9 @@
       <c r="AL7" t="n">
         <v>49900</v>
       </c>
-      <c r="AM7" t="inlineStr"/>
+      <c r="AM7" t="n">
+        <v>56200</v>
+      </c>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
@@ -1935,7 +1957,9 @@
       <c r="AT7" t="n">
         <v>0</v>
       </c>
-      <c r="AU7" t="inlineStr"/>
+      <c r="AU7" t="n">
+        <v>0</v>
+      </c>
       <c r="AV7" t="inlineStr"/>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
@@ -1948,7 +1972,7 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>30900</v>
+        <v>28760</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1957,13 +1981,13 @@
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="inlineStr"/>
       <c r="BN7" t="n">
-        <v>318525</v>
+        <v>262360</v>
       </c>
       <c r="BO7" t="n">
-        <v>30900</v>
+        <v>28760</v>
       </c>
       <c r="BP7" t="n">
-        <v>21013720</v>
+        <v>19548000</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
@@ -1972,10 +1996,10 @@
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="n">
-        <v>247000550</v>
+        <v>202733020</v>
       </c>
       <c r="BX7" t="n">
-        <v>21013720</v>
+        <v>19548000</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -1983,17 +2007,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2059,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>665</v>
+        <v>678</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2058,10 +2082,10 @@
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="AE8" t="n">
-        <v>70700</v>
+        <v>106000</v>
       </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
@@ -2072,7 +2096,9 @@
       <c r="AL8" t="n">
         <v>70700</v>
       </c>
-      <c r="AM8" t="inlineStr"/>
+      <c r="AM8" t="n">
+        <v>106000</v>
+      </c>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
@@ -2082,7 +2108,9 @@
       <c r="AT8" t="n">
         <v>1000</v>
       </c>
-      <c r="AU8" t="inlineStr"/>
+      <c r="AU8" t="n">
+        <v>0</v>
+      </c>
       <c r="AV8" t="inlineStr"/>
       <c r="AW8" t="inlineStr"/>
       <c r="AX8" t="inlineStr"/>
@@ -2095,7 +2123,7 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
-        <v>140100</v>
+        <v>96860</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
@@ -2104,13 +2132,13 @@
       <c r="BL8" t="inlineStr"/>
       <c r="BM8" t="inlineStr"/>
       <c r="BN8" t="n">
-        <v>540325</v>
+        <v>484140</v>
       </c>
       <c r="BO8" t="n">
-        <v>140100</v>
+        <v>96860</v>
       </c>
       <c r="BP8" t="n">
-        <v>98474520</v>
+        <v>66866560</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
@@ -2119,10 +2147,10 @@
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="inlineStr"/>
       <c r="BW8" t="n">
-        <v>389225050</v>
+        <v>348791500</v>
       </c>
       <c r="BX8" t="n">
-        <v>98474520</v>
+        <v>66866560</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2130,17 +2158,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2210,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1362</v>
+        <v>1450</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2208,7 +2236,7 @@
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>408200</v>
+        <v>634100</v>
       </c>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
@@ -2219,7 +2247,9 @@
       <c r="AL9" t="n">
         <v>408200</v>
       </c>
-      <c r="AM9" t="inlineStr"/>
+      <c r="AM9" t="n">
+        <v>634100</v>
+      </c>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
@@ -2229,10 +2259,20 @@
       <c r="AT9" t="n">
         <v>0</v>
       </c>
-      <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr"/>
-      <c r="AW9" t="inlineStr"/>
-      <c r="AX9" t="inlineStr"/>
+      <c r="AU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>Jump Trading Pacific Pte Ltd</t>
+        </is>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>97000</v>
+      </c>
       <c r="AY9" t="inlineStr"/>
       <c r="AZ9" t="inlineStr"/>
       <c r="BA9" t="inlineStr"/>
@@ -2242,7 +2282,7 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>2620900</v>
+        <v>1377460</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
@@ -2251,13 +2291,13 @@
       <c r="BL9" t="inlineStr"/>
       <c r="BM9" t="inlineStr"/>
       <c r="BN9" t="n">
-        <v>7535550</v>
+        <v>7379033.333333333</v>
       </c>
       <c r="BO9" t="n">
-        <v>2620900</v>
+        <v>1377460</v>
       </c>
       <c r="BP9" t="n">
-        <v>3937584140</v>
+        <v>2064326120</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
@@ -2266,10 +2306,10 @@
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="inlineStr"/>
       <c r="BW9" t="n">
-        <v>11342836750</v>
+        <v>11088886866.66667</v>
       </c>
       <c r="BX9" t="n">
-        <v>3937584140</v>
+        <v>2064326120</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2277,17 +2317,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2369,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1184</v>
+        <v>1105</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2351,8 +2391,12 @@
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="inlineStr"/>
+      <c r="AD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>135800</v>
+      </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr"/>
@@ -2360,7 +2404,9 @@
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
+      <c r="AM10" t="n">
+        <v>135800</v>
+      </c>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
@@ -2368,7 +2414,9 @@
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="inlineStr"/>
-      <c r="AU10" t="inlineStr"/>
+      <c r="AU10" t="n">
+        <v>0</v>
+      </c>
       <c r="AV10" t="inlineStr"/>
       <c r="AW10" t="inlineStr"/>
       <c r="AX10" t="inlineStr"/>
@@ -2381,7 +2429,7 @@
       <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="n">
-        <v>675266.6666666666</v>
+        <v>590450</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2391,10 +2439,10 @@
       <c r="BM10" t="inlineStr"/>
       <c r="BN10" t="inlineStr"/>
       <c r="BO10" t="n">
-        <v>675266.6666666666</v>
+        <v>590450</v>
       </c>
       <c r="BP10" t="n">
-        <v>873361533.3333334</v>
+        <v>749783650</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2404,7 +2452,7 @@
       <c r="BV10" t="inlineStr"/>
       <c r="BW10" t="inlineStr"/>
       <c r="BX10" t="n">
-        <v>873361533.3333334</v>
+        <v>749783650</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2412,17 +2460,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2512,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>475</v>
+        <v>441</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2486,8 +2534,12 @@
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="inlineStr"/>
+      <c r="AD11" t="n">
+        <v>673100</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>3478500</v>
+      </c>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
@@ -2495,7 +2547,9 @@
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="inlineStr"/>
+      <c r="AM11" t="n">
+        <v>3478500</v>
+      </c>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
@@ -2503,7 +2557,9 @@
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="inlineStr"/>
-      <c r="AU11" t="inlineStr"/>
+      <c r="AU11" t="n">
+        <v>673100</v>
+      </c>
       <c r="AV11" t="inlineStr"/>
       <c r="AW11" t="inlineStr"/>
       <c r="AX11" t="inlineStr"/>
@@ -2516,7 +2572,7 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>22304225</v>
+        <v>21773700</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2526,10 +2582,10 @@
       <c r="BM11" t="inlineStr"/>
       <c r="BN11" t="inlineStr"/>
       <c r="BO11" t="n">
-        <v>22304225</v>
+        <v>21773700</v>
       </c>
       <c r="BP11" t="n">
-        <v>10645521900</v>
+        <v>10269101440</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2539,7 +2595,7 @@
       <c r="BV11" t="inlineStr"/>
       <c r="BW11" t="inlineStr"/>
       <c r="BX11" t="n">
-        <v>10645521900</v>
+        <v>10269101440</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2547,17 +2603,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2621,8 +2677,12 @@
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
+      <c r="AD12" t="n">
+        <v>39200</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>126500</v>
+      </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr"/>
@@ -2630,7 +2690,9 @@
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
+      <c r="AM12" t="n">
+        <v>126500</v>
+      </c>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
       <c r="AP12" t="inlineStr"/>
@@ -2638,17 +2700,19 @@
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="inlineStr"/>
-      <c r="AU12" t="inlineStr"/>
+      <c r="AU12" t="n">
+        <v>39200</v>
+      </c>
       <c r="AV12" t="inlineStr">
         <is>
           <t>GOLDMAN SACHS INTERNATIONAL</t>
         </is>
       </c>
       <c r="AW12" t="n">
-        <v>0.0053</v>
+        <v>0.0048</v>
       </c>
       <c r="AX12" t="n">
-        <v>382685</v>
+        <v>345085</v>
       </c>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
@@ -2659,7 +2723,7 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>248475</v>
+        <v>240660</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2669,10 +2733,10 @@
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="inlineStr"/>
       <c r="BO12" t="n">
-        <v>248475</v>
+        <v>240660</v>
       </c>
       <c r="BP12" t="n">
-        <v>103489250</v>
+        <v>100115340</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2682,7 +2746,7 @@
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="inlineStr"/>
       <c r="BX12" t="n">
-        <v>103489250</v>
+        <v>100115340</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2690,17 +2754,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2806,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>932</v>
+        <v>914</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2764,8 +2828,12 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
+      <c r="AD13" t="n">
+        <v>2200</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>62800</v>
+      </c>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
@@ -2773,7 +2841,9 @@
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
       <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
+      <c r="AM13" t="n">
+        <v>62800</v>
+      </c>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
@@ -2781,7 +2851,9 @@
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="inlineStr"/>
+      <c r="AU13" t="n">
+        <v>2200</v>
+      </c>
       <c r="AV13" t="inlineStr"/>
       <c r="AW13" t="inlineStr"/>
       <c r="AX13" t="inlineStr"/>
@@ -2794,7 +2866,7 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="n">
-        <v>171850</v>
+        <v>167980</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2804,10 +2876,10 @@
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="inlineStr"/>
       <c r="BO13" t="n">
-        <v>171850</v>
+        <v>167980</v>
       </c>
       <c r="BP13" t="n">
-        <v>160315700</v>
+        <v>156119560</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2817,7 +2889,7 @@
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="inlineStr"/>
       <c r="BX13" t="n">
-        <v>160315700</v>
+        <v>156119560</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2825,17 +2897,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2949,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1861</v>
+        <v>1859</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -2899,8 +2971,12 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
+      <c r="AD14" t="n">
+        <v>6700</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>546000</v>
+      </c>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr"/>
@@ -2908,7 +2984,9 @@
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
       <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr"/>
+      <c r="AM14" t="n">
+        <v>546000</v>
+      </c>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
@@ -2916,7 +2994,9 @@
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="inlineStr"/>
-      <c r="AU14" t="inlineStr"/>
+      <c r="AU14" t="n">
+        <v>6700</v>
+      </c>
       <c r="AV14" t="inlineStr">
         <is>
           <t>GOLDMAN SACHS INTERNATIONAL</t>
@@ -2939,7 +3019,7 @@
         <v>194633</v>
       </c>
       <c r="BG14" t="n">
-        <v>201300</v>
+        <v>181100</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -2949,10 +3029,10 @@
       <c r="BM14" t="inlineStr"/>
       <c r="BN14" t="inlineStr"/>
       <c r="BO14" t="n">
-        <v>201300</v>
+        <v>181100</v>
       </c>
       <c r="BP14" t="n">
-        <v>366972875</v>
+        <v>330671340</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -2962,7 +3042,7 @@
       <c r="BV14" t="inlineStr"/>
       <c r="BW14" t="inlineStr"/>
       <c r="BX14" t="n">
-        <v>366972875</v>
+        <v>330671340</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -2970,17 +3050,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3102,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -3044,8 +3124,12 @@
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="inlineStr"/>
+      <c r="AD15" t="n">
+        <v>86900</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>11624300</v>
+      </c>
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
@@ -3053,7 +3137,9 @@
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
       <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="inlineStr"/>
+      <c r="AM15" t="n">
+        <v>11624300</v>
+      </c>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
       <c r="AP15" t="inlineStr"/>
@@ -3061,7 +3147,9 @@
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="inlineStr"/>
-      <c r="AU15" t="inlineStr"/>
+      <c r="AU15" t="n">
+        <v>86900</v>
+      </c>
       <c r="AV15" t="inlineStr"/>
       <c r="AW15" t="inlineStr"/>
       <c r="AX15" t="inlineStr"/>
@@ -3074,7 +3162,7 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>2140650</v>
+        <v>2009960</v>
       </c>
       <c r="BH15" t="inlineStr"/>
       <c r="BI15" t="inlineStr"/>
@@ -3084,10 +3172,10 @@
       <c r="BM15" t="inlineStr"/>
       <c r="BN15" t="inlineStr"/>
       <c r="BO15" t="n">
-        <v>2140650</v>
+        <v>2009960</v>
       </c>
       <c r="BP15" t="n">
-        <v>932730175</v>
+        <v>871040860</v>
       </c>
       <c r="BQ15" t="inlineStr"/>
       <c r="BR15" t="inlineStr"/>
@@ -3097,7 +3185,7 @@
       <c r="BV15" t="inlineStr"/>
       <c r="BW15" t="inlineStr"/>
       <c r="BX15" t="n">
-        <v>932730175</v>
+        <v>871040860</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3105,17 +3193,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -3157,7 +3245,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>951</v>
+        <v>1040</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3209,7 +3297,7 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>2057900</v>
+        <v>2754150</v>
       </c>
       <c r="BH16" t="inlineStr"/>
       <c r="BI16" t="inlineStr"/>
@@ -3219,10 +3307,10 @@
       <c r="BM16" t="inlineStr"/>
       <c r="BN16" t="inlineStr"/>
       <c r="BO16" t="n">
-        <v>2057900</v>
+        <v>2754150</v>
       </c>
       <c r="BP16" t="n">
-        <v>2105307200</v>
+        <v>2897407950</v>
       </c>
       <c r="BQ16" t="inlineStr"/>
       <c r="BR16" t="inlineStr"/>
@@ -3232,7 +3320,7 @@
       <c r="BV16" t="inlineStr"/>
       <c r="BW16" t="inlineStr"/>
       <c r="BX16" t="n">
-        <v>2105307200</v>
+        <v>2897407950</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3240,29 +3328,29 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>549A</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>日本銀行</t>
+          <t>ヒトトヒトホールディングス</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3272,12 +3360,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>銀行</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>銀行業</t>
+          <t>サービス業</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3292,7 +3380,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>25200</v>
+        <v>441</v>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -3344,58 +3432,30 @@
       <c r="BE17" t="inlineStr"/>
       <c r="BF17" t="inlineStr"/>
       <c r="BG17" t="n">
-        <v>266.6666666666667</v>
-      </c>
-      <c r="BH17" t="n">
-        <v>440</v>
-      </c>
-      <c r="BI17" t="n">
-        <v>875</v>
-      </c>
-      <c r="BJ17" t="n">
-        <v>100</v>
-      </c>
-      <c r="BK17" t="n">
-        <v>450</v>
-      </c>
-      <c r="BL17" t="n">
-        <v>300</v>
-      </c>
-      <c r="BM17" t="n">
-        <v>166.6666666666667</v>
-      </c>
-      <c r="BN17" t="n">
-        <v>250</v>
-      </c>
+        <v>5849500</v>
+      </c>
+      <c r="BH17" t="inlineStr"/>
+      <c r="BI17" t="inlineStr"/>
+      <c r="BJ17" t="inlineStr"/>
+      <c r="BK17" t="inlineStr"/>
+      <c r="BL17" t="inlineStr"/>
+      <c r="BM17" t="inlineStr"/>
+      <c r="BN17" t="inlineStr"/>
       <c r="BO17" t="n">
-        <v>266.6666666666667</v>
+        <v>5849500</v>
       </c>
       <c r="BP17" t="n">
-        <v>6588333.333333333</v>
-      </c>
-      <c r="BQ17" t="n">
-        <v>11565600</v>
-      </c>
-      <c r="BR17" t="n">
-        <v>23735750</v>
-      </c>
-      <c r="BS17" t="n">
-        <v>2650000</v>
-      </c>
-      <c r="BT17" t="n">
-        <v>11285000</v>
-      </c>
-      <c r="BU17" t="n">
-        <v>7486400</v>
-      </c>
-      <c r="BV17" t="n">
-        <v>4104666.666666667</v>
-      </c>
-      <c r="BW17" t="n">
-        <v>6260000</v>
-      </c>
+        <v>2571111900</v>
+      </c>
+      <c r="BQ17" t="inlineStr"/>
+      <c r="BR17" t="inlineStr"/>
+      <c r="BS17" t="inlineStr"/>
+      <c r="BT17" t="inlineStr"/>
+      <c r="BU17" t="inlineStr"/>
+      <c r="BV17" t="inlineStr"/>
+      <c r="BW17" t="inlineStr"/>
       <c r="BX17" t="n">
-        <v>6588333.333333333</v>
+        <v>2571111900</v>
       </c>
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
@@ -3403,29 +3463,29 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9399</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+          <t>日本銀行</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3435,12 +3495,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>銀行</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>銀行業</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3454,9 +3514,7 @@
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>26</v>
-      </c>
+      <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -3477,55 +3535,23 @@
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE18" t="n">
-        <v>96080</v>
-      </c>
-      <c r="AF18" t="n">
-        <v>202741</v>
-      </c>
-      <c r="AG18" t="n">
-        <v>204885</v>
-      </c>
-      <c r="AH18" t="n">
-        <v>97185</v>
-      </c>
-      <c r="AI18" t="n">
-        <v>93675</v>
-      </c>
-      <c r="AJ18" t="n">
-        <v>126528</v>
-      </c>
-      <c r="AK18" t="n">
-        <v>99264</v>
-      </c>
-      <c r="AL18" t="n">
-        <v>96080</v>
-      </c>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
       <c r="AM18" t="inlineStr"/>
-      <c r="AN18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT18" t="n">
-        <v>0</v>
-      </c>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
       <c r="AU18" t="inlineStr"/>
       <c r="AV18" t="inlineStr"/>
       <c r="AW18" t="inlineStr"/>
@@ -3539,58 +3565,58 @@
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="n">
-        <v>1960023.6</v>
+        <v>250</v>
       </c>
       <c r="BH18" t="n">
-        <v>4774465.6</v>
+        <v>700</v>
       </c>
       <c r="BI18" t="n">
-        <v>13931419.2</v>
+        <v>300</v>
       </c>
       <c r="BJ18" t="n">
-        <v>5104435.2</v>
+        <v>200</v>
       </c>
       <c r="BK18" t="n">
-        <v>3130213.4</v>
+        <v>500</v>
       </c>
       <c r="BL18" t="n">
-        <v>3424175.2</v>
+        <v>260</v>
       </c>
       <c r="BM18" t="n">
-        <v>4747035.2</v>
+        <v>233.3333333333333</v>
       </c>
       <c r="BN18" t="n">
-        <v>1966370.8</v>
+        <v>250</v>
       </c>
       <c r="BO18" t="n">
-        <v>1960023.6</v>
+        <v>250</v>
       </c>
       <c r="BP18" t="n">
-        <v>52706922.8</v>
+        <v>6186000</v>
       </c>
       <c r="BQ18" t="n">
-        <v>170454411.4</v>
+        <v>18946800</v>
       </c>
       <c r="BR18" t="n">
-        <v>356289258</v>
+        <v>7920750</v>
       </c>
       <c r="BS18" t="n">
-        <v>147240261</v>
+        <v>5100000</v>
       </c>
       <c r="BT18" t="n">
-        <v>83366454.8</v>
+        <v>12464000</v>
       </c>
       <c r="BU18" t="n">
-        <v>100089101.6</v>
+        <v>6487600</v>
       </c>
       <c r="BV18" t="n">
-        <v>150288273.6</v>
+        <v>5785000</v>
       </c>
       <c r="BW18" t="n">
-        <v>58329980.2</v>
+        <v>6204000</v>
       </c>
       <c r="BX18" t="n">
-        <v>52706922.8</v>
+        <v>6186000</v>
       </c>
       <c r="BY18" t="inlineStr"/>
       <c r="BZ18" t="inlineStr"/>
@@ -3598,17 +3624,216 @@
       <c r="CB18" t="inlineStr"/>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>20260407-001522</t>
+          <t>20260407-190052</t>
         </is>
       </c>
       <c r="CD18" t="inlineStr">
         <is>
-          <t>2026-04-06T15:15:22+00:00</t>
+          <t>2026-04-07T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>2026-04-07T00:15:22+09:00</t>
+          <t>2026-04-07T19:00:52+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>9399</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>スタンダード</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>情報通信・サービスその他</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>情報･通信業</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>26</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>122230</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>202741</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>204885</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>97185</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>93675</v>
+      </c>
+      <c r="AJ19" t="n">
+        <v>126528</v>
+      </c>
+      <c r="AK19" t="n">
+        <v>99264</v>
+      </c>
+      <c r="AL19" t="n">
+        <v>96080</v>
+      </c>
+      <c r="AM19" t="n">
+        <v>122230</v>
+      </c>
+      <c r="AN19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="n">
+        <v>2038676.2</v>
+      </c>
+      <c r="BH19" t="n">
+        <v>6430472.2</v>
+      </c>
+      <c r="BI19" t="n">
+        <v>13641653.6</v>
+      </c>
+      <c r="BJ19" t="n">
+        <v>4141412.2</v>
+      </c>
+      <c r="BK19" t="n">
+        <v>3244477</v>
+      </c>
+      <c r="BL19" t="n">
+        <v>3121484.8</v>
+      </c>
+      <c r="BM19" t="n">
+        <v>4791179.2</v>
+      </c>
+      <c r="BN19" t="n">
+        <v>1602701</v>
+      </c>
+      <c r="BO19" t="n">
+        <v>2038676.2</v>
+      </c>
+      <c r="BP19" t="n">
+        <v>54470723.6</v>
+      </c>
+      <c r="BQ19" t="n">
+        <v>204969357.4</v>
+      </c>
+      <c r="BR19" t="n">
+        <v>361089200</v>
+      </c>
+      <c r="BS19" t="n">
+        <v>112574536.8</v>
+      </c>
+      <c r="BT19" t="n">
+        <v>89198367.8</v>
+      </c>
+      <c r="BU19" t="n">
+        <v>91308870.59999999</v>
+      </c>
+      <c r="BV19" t="n">
+        <v>152865029.4</v>
+      </c>
+      <c r="BW19" t="n">
+        <v>47100971.4</v>
+      </c>
+      <c r="BX19" t="n">
+        <v>54470723.6</v>
+      </c>
+      <c r="BY19" t="inlineStr"/>
+      <c r="BZ19" t="inlineStr"/>
+      <c r="CA19" t="inlineStr"/>
+      <c r="CB19" t="inlineStr"/>
+      <c r="CC19" t="inlineStr">
+        <is>
+          <t>20260407-190052</t>
+        </is>
+      </c>
+      <c r="CD19" t="inlineStr">
+        <is>
+          <t>2026-04-07T10:00:52+00:00</t>
+        </is>
+      </c>
+      <c r="CE19" t="inlineStr">
+        <is>
+          <t>2026-04-07T19:00:52+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-08
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -971,58 +971,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>26400</v>
+        <v>34400</v>
       </c>
       <c r="BH2" t="n">
-        <v>17600</v>
+        <v>14000</v>
       </c>
       <c r="BI2" t="n">
-        <v>9600</v>
+        <v>9200</v>
       </c>
       <c r="BJ2" t="n">
-        <v>16200</v>
+        <v>17800</v>
       </c>
       <c r="BK2" t="n">
-        <v>22400</v>
+        <v>21800</v>
       </c>
       <c r="BL2" t="n">
-        <v>14200</v>
+        <v>13200</v>
       </c>
       <c r="BM2" t="n">
-        <v>14000</v>
+        <v>14800</v>
       </c>
       <c r="BN2" t="n">
-        <v>16000</v>
+        <v>14600</v>
       </c>
       <c r="BO2" t="n">
-        <v>26400</v>
+        <v>34400</v>
       </c>
       <c r="BP2" t="n">
-        <v>1869600</v>
+        <v>2473200</v>
       </c>
       <c r="BQ2" t="n">
-        <v>1401800</v>
+        <v>1110800</v>
       </c>
       <c r="BR2" t="n">
-        <v>772000</v>
+        <v>742000</v>
       </c>
       <c r="BS2" t="n">
-        <v>1272800</v>
+        <v>1394000</v>
       </c>
       <c r="BT2" t="n">
-        <v>1628000</v>
+        <v>1567400</v>
       </c>
       <c r="BU2" t="n">
-        <v>993800</v>
+        <v>921000</v>
       </c>
       <c r="BV2" t="n">
-        <v>979400</v>
+        <v>1033200</v>
       </c>
       <c r="BW2" t="n">
-        <v>1072200</v>
+        <v>975800</v>
       </c>
       <c r="BX2" t="n">
-        <v>1869600</v>
+        <v>2473200</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1030,17 +1030,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2454</v>
+        <v>2702</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1194,58 +1194,58 @@
         <v>362132</v>
       </c>
       <c r="BG3" t="n">
-        <v>2399940</v>
+        <v>2882260</v>
       </c>
       <c r="BH3" t="n">
-        <v>1829140</v>
+        <v>1696600</v>
       </c>
       <c r="BI3" t="n">
-        <v>1128420</v>
+        <v>1586800</v>
       </c>
       <c r="BJ3" t="n">
-        <v>2249300</v>
+        <v>1915440</v>
       </c>
       <c r="BK3" t="n">
-        <v>2068040</v>
+        <v>1947500</v>
       </c>
       <c r="BL3" t="n">
-        <v>1558240</v>
+        <v>1697500</v>
       </c>
       <c r="BM3" t="n">
-        <v>3241660</v>
+        <v>3319560</v>
       </c>
       <c r="BN3" t="n">
-        <v>2032180</v>
+        <v>1890100</v>
       </c>
       <c r="BO3" t="n">
-        <v>2399940</v>
+        <v>2882260</v>
       </c>
       <c r="BP3" t="n">
-        <v>5654626740</v>
+        <v>7053615520</v>
       </c>
       <c r="BQ3" t="n">
-        <v>3725834940</v>
+        <v>3461498820</v>
       </c>
       <c r="BR3" t="n">
-        <v>2306432200</v>
+        <v>3311761960</v>
       </c>
       <c r="BS3" t="n">
-        <v>4869925960</v>
+        <v>4198538840</v>
       </c>
       <c r="BT3" t="n">
-        <v>4302787140</v>
+        <v>3985863960</v>
       </c>
       <c r="BU3" t="n">
-        <v>3372377580</v>
+        <v>3756858500</v>
       </c>
       <c r="BV3" t="n">
-        <v>7930500380</v>
+        <v>8162734480</v>
       </c>
       <c r="BW3" t="n">
-        <v>4614806860</v>
+        <v>4201238040</v>
       </c>
       <c r="BX3" t="n">
-        <v>5654626740</v>
+        <v>7053615520</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1253,17 +1253,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1393,58 +1393,58 @@
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="n">
-        <v>13980</v>
+        <v>19560</v>
       </c>
       <c r="BH4" t="n">
-        <v>82560</v>
+        <v>73760</v>
       </c>
       <c r="BI4" t="n">
-        <v>64700</v>
+        <v>66220</v>
       </c>
       <c r="BJ4" t="n">
-        <v>59380</v>
+        <v>65160</v>
       </c>
       <c r="BK4" t="n">
-        <v>77740</v>
+        <v>71700</v>
       </c>
       <c r="BL4" t="n">
-        <v>48480</v>
+        <v>76300</v>
       </c>
       <c r="BM4" t="n">
-        <v>103840</v>
+        <v>71860</v>
       </c>
       <c r="BN4" t="n">
-        <v>33720</v>
+        <v>28740</v>
       </c>
       <c r="BO4" t="n">
-        <v>13980</v>
+        <v>19560</v>
       </c>
       <c r="BP4" t="n">
-        <v>3137240</v>
+        <v>4404040</v>
       </c>
       <c r="BQ4" t="n">
-        <v>21765620</v>
+        <v>19529100</v>
       </c>
       <c r="BR4" t="n">
-        <v>16438180</v>
+        <v>16615420</v>
       </c>
       <c r="BS4" t="n">
-        <v>14522900</v>
+        <v>15752240</v>
       </c>
       <c r="BT4" t="n">
-        <v>17546800</v>
+        <v>16048700</v>
       </c>
       <c r="BU4" t="n">
-        <v>10831060</v>
+        <v>17525360</v>
       </c>
       <c r="BV4" t="n">
-        <v>24264960</v>
+        <v>16693620</v>
       </c>
       <c r="BW4" t="n">
-        <v>7616900</v>
+        <v>6423760</v>
       </c>
       <c r="BX4" t="n">
-        <v>3137240</v>
+        <v>4404040</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1452,17 +1452,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1604,50 +1604,54 @@
         <v>0</v>
       </c>
       <c r="BG5" t="n">
-        <v>54260</v>
+        <v>49560</v>
       </c>
       <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="inlineStr"/>
+      <c r="BI5" t="n">
+        <v>2819200</v>
+      </c>
       <c r="BJ5" t="n">
-        <v>971220</v>
+        <v>469840</v>
       </c>
       <c r="BK5" t="n">
-        <v>162400</v>
+        <v>119060</v>
       </c>
       <c r="BL5" t="n">
-        <v>94040</v>
+        <v>101440</v>
       </c>
       <c r="BM5" t="n">
-        <v>125360</v>
+        <v>110180</v>
       </c>
       <c r="BN5" t="n">
-        <v>86440</v>
+        <v>96620</v>
       </c>
       <c r="BO5" t="n">
-        <v>54260</v>
+        <v>49560</v>
       </c>
       <c r="BP5" t="n">
-        <v>44134900</v>
+        <v>41043140</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
-      <c r="BR5" t="inlineStr"/>
+      <c r="BR5" t="n">
+        <v>3093295700</v>
+      </c>
       <c r="BS5" t="n">
-        <v>1018630620</v>
+        <v>467821240</v>
       </c>
       <c r="BT5" t="n">
-        <v>168932740</v>
+        <v>120823060</v>
       </c>
       <c r="BU5" t="n">
-        <v>98665760</v>
+        <v>106038140</v>
       </c>
       <c r="BV5" t="n">
-        <v>119082120</v>
+        <v>101965460</v>
       </c>
       <c r="BW5" t="n">
-        <v>72462920</v>
+        <v>79752720</v>
       </c>
       <c r="BX5" t="n">
-        <v>44134900</v>
+        <v>41043140</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1655,17 +1659,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1711,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1295</v>
+        <v>1315</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1805,50 +1809,50 @@
         <v>0</v>
       </c>
       <c r="BG6" t="n">
-        <v>28820</v>
+        <v>38880</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="n">
-        <v>663400</v>
+        <v>521300</v>
       </c>
       <c r="BK6" t="n">
-        <v>155060</v>
+        <v>115100</v>
       </c>
       <c r="BL6" t="n">
-        <v>46960</v>
+        <v>50100</v>
       </c>
       <c r="BM6" t="n">
-        <v>46160</v>
+        <v>44220</v>
       </c>
       <c r="BN6" t="n">
-        <v>37800</v>
+        <v>38260</v>
       </c>
       <c r="BO6" t="n">
-        <v>28820</v>
+        <v>38880</v>
       </c>
       <c r="BP6" t="n">
-        <v>37297620</v>
+        <v>50626400</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="n">
-        <v>1125348550</v>
+        <v>870049733.3333334</v>
       </c>
       <c r="BT6" t="n">
-        <v>222315800</v>
+        <v>161032720</v>
       </c>
       <c r="BU6" t="n">
-        <v>65570020</v>
+        <v>69102560</v>
       </c>
       <c r="BV6" t="n">
-        <v>59230440</v>
+        <v>56122460</v>
       </c>
       <c r="BW6" t="n">
-        <v>47679980</v>
+        <v>48400700</v>
       </c>
       <c r="BX6" t="n">
-        <v>37297620</v>
+        <v>50626400</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1856,17 +1860,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1912,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>685</v>
+        <v>696</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1972,34 +1976,38 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>28760</v>
+        <v>19780</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
       <c r="BJ7" t="inlineStr"/>
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="inlineStr"/>
+      <c r="BM7" t="n">
+        <v>800000</v>
+      </c>
       <c r="BN7" t="n">
-        <v>262360</v>
+        <v>116000</v>
       </c>
       <c r="BO7" t="n">
-        <v>28760</v>
+        <v>19780</v>
       </c>
       <c r="BP7" t="n">
-        <v>19548000</v>
+        <v>13478760</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
-      <c r="BV7" t="inlineStr"/>
+      <c r="BV7" t="n">
+        <v>643551400</v>
+      </c>
       <c r="BW7" t="n">
-        <v>202733020</v>
+        <v>83306260</v>
       </c>
       <c r="BX7" t="n">
-        <v>19548000</v>
+        <v>13478760</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -2007,17 +2015,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2067,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2123,34 +2131,38 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
-        <v>96860</v>
+        <v>80500</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
       <c r="BJ8" t="inlineStr"/>
       <c r="BK8" t="inlineStr"/>
       <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="inlineStr"/>
+      <c r="BM8" t="n">
+        <v>989300</v>
+      </c>
       <c r="BN8" t="n">
-        <v>484140</v>
+        <v>313140</v>
       </c>
       <c r="BO8" t="n">
-        <v>96860</v>
+        <v>80500</v>
       </c>
       <c r="BP8" t="n">
-        <v>66866560</v>
+        <v>54726680</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
       <c r="BS8" t="inlineStr"/>
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
-      <c r="BV8" t="inlineStr"/>
+      <c r="BV8" t="n">
+        <v>737786900</v>
+      </c>
       <c r="BW8" t="n">
-        <v>348791500</v>
+        <v>220473800</v>
       </c>
       <c r="BX8" t="n">
-        <v>66866560</v>
+        <v>54726680</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2158,17 +2170,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2222,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1450</v>
+        <v>1470</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2282,7 +2294,7 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>1377460</v>
+        <v>790120</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
@@ -2291,13 +2303,13 @@
       <c r="BL9" t="inlineStr"/>
       <c r="BM9" t="inlineStr"/>
       <c r="BN9" t="n">
-        <v>7379033.333333333</v>
+        <v>6388500</v>
       </c>
       <c r="BO9" t="n">
-        <v>1377460</v>
+        <v>790120</v>
       </c>
       <c r="BP9" t="n">
-        <v>2064326120</v>
+        <v>1134294660</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
@@ -2306,10 +2318,10 @@
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="inlineStr"/>
       <c r="BW9" t="n">
-        <v>11088886866.66667</v>
+        <v>9658056125</v>
       </c>
       <c r="BX9" t="n">
-        <v>2064326120</v>
+        <v>1134294660</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2317,17 +2329,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2381,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1105</v>
+        <v>1110</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2429,7 +2441,7 @@
       <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="n">
-        <v>590450</v>
+        <v>498160</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2439,10 +2451,10 @@
       <c r="BM10" t="inlineStr"/>
       <c r="BN10" t="inlineStr"/>
       <c r="BO10" t="n">
-        <v>590450</v>
+        <v>498160</v>
       </c>
       <c r="BP10" t="n">
-        <v>749783650</v>
+        <v>628596580</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2452,7 +2464,7 @@
       <c r="BV10" t="inlineStr"/>
       <c r="BW10" t="inlineStr"/>
       <c r="BX10" t="n">
-        <v>749783650</v>
+        <v>628596580</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2460,17 +2472,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2524,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>441</v>
+        <v>432</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2572,7 +2584,7 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>21773700</v>
+        <v>23838300</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2580,12 +2592,14 @@
       <c r="BK11" t="inlineStr"/>
       <c r="BL11" t="inlineStr"/>
       <c r="BM11" t="inlineStr"/>
-      <c r="BN11" t="inlineStr"/>
+      <c r="BN11" t="n">
+        <v>10246600</v>
+      </c>
       <c r="BO11" t="n">
-        <v>21773700</v>
+        <v>23838300</v>
       </c>
       <c r="BP11" t="n">
-        <v>10269101440</v>
+        <v>11182826880</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2593,9 +2607,11 @@
       <c r="BT11" t="inlineStr"/>
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="inlineStr"/>
-      <c r="BW11" t="inlineStr"/>
+      <c r="BW11" t="n">
+        <v>4296843900</v>
+      </c>
       <c r="BX11" t="n">
-        <v>10269101440</v>
+        <v>11182826880</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2603,17 +2619,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2671,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2709,10 +2725,10 @@
         </is>
       </c>
       <c r="AW12" t="n">
-        <v>0.0048</v>
+        <v>0.0053</v>
       </c>
       <c r="AX12" t="n">
-        <v>345085</v>
+        <v>379285</v>
       </c>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
@@ -2723,7 +2739,7 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>240660</v>
+        <v>222760</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2731,12 +2747,14 @@
       <c r="BK12" t="inlineStr"/>
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
-      <c r="BN12" t="inlineStr"/>
+      <c r="BN12" t="n">
+        <v>244800</v>
+      </c>
       <c r="BO12" t="n">
-        <v>240660</v>
+        <v>222760</v>
       </c>
       <c r="BP12" t="n">
-        <v>100115340</v>
+        <v>92551780</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2744,9 +2762,11 @@
       <c r="BT12" t="inlineStr"/>
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
-      <c r="BW12" t="inlineStr"/>
+      <c r="BW12" t="n">
+        <v>102953000</v>
+      </c>
       <c r="BX12" t="n">
-        <v>100115340</v>
+        <v>92551780</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2754,17 +2774,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2826,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>914</v>
+        <v>944</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2866,7 +2886,7 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="n">
-        <v>167980</v>
+        <v>177860</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2874,12 +2894,14 @@
       <c r="BK13" t="inlineStr"/>
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
-      <c r="BN13" t="inlineStr"/>
+      <c r="BN13" t="n">
+        <v>91400</v>
+      </c>
       <c r="BO13" t="n">
-        <v>167980</v>
+        <v>177860</v>
       </c>
       <c r="BP13" t="n">
-        <v>156119560</v>
+        <v>166188720</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2887,9 +2909,11 @@
       <c r="BT13" t="inlineStr"/>
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
-      <c r="BW13" t="inlineStr"/>
+      <c r="BW13" t="n">
+        <v>81195700</v>
+      </c>
       <c r="BX13" t="n">
-        <v>156119560</v>
+        <v>166188720</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2897,17 +2921,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2973,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1859</v>
+        <v>1909</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -3019,7 +3043,7 @@
         <v>194633</v>
       </c>
       <c r="BG14" t="n">
-        <v>181100</v>
+        <v>199220</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -3027,12 +3051,14 @@
       <c r="BK14" t="inlineStr"/>
       <c r="BL14" t="inlineStr"/>
       <c r="BM14" t="inlineStr"/>
-      <c r="BN14" t="inlineStr"/>
+      <c r="BN14" t="n">
+        <v>157200</v>
+      </c>
       <c r="BO14" t="n">
-        <v>181100</v>
+        <v>199220</v>
       </c>
       <c r="BP14" t="n">
-        <v>330671340</v>
+        <v>369146580</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -3040,9 +3066,11 @@
       <c r="BT14" t="inlineStr"/>
       <c r="BU14" t="inlineStr"/>
       <c r="BV14" t="inlineStr"/>
-      <c r="BW14" t="inlineStr"/>
+      <c r="BW14" t="n">
+        <v>278865400</v>
+      </c>
       <c r="BX14" t="n">
-        <v>330671340</v>
+        <v>369146580</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -3050,17 +3078,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3130,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>421</v>
+        <v>441</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -3162,7 +3190,7 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>2009960</v>
+        <v>1942060</v>
       </c>
       <c r="BH15" t="inlineStr"/>
       <c r="BI15" t="inlineStr"/>
@@ -3170,12 +3198,14 @@
       <c r="BK15" t="inlineStr"/>
       <c r="BL15" t="inlineStr"/>
       <c r="BM15" t="inlineStr"/>
-      <c r="BN15" t="inlineStr"/>
+      <c r="BN15" t="n">
+        <v>2383200</v>
+      </c>
       <c r="BO15" t="n">
-        <v>2009960</v>
+        <v>1942060</v>
       </c>
       <c r="BP15" t="n">
-        <v>871040860</v>
+        <v>837295120</v>
       </c>
       <c r="BQ15" t="inlineStr"/>
       <c r="BR15" t="inlineStr"/>
@@ -3183,9 +3213,11 @@
       <c r="BT15" t="inlineStr"/>
       <c r="BU15" t="inlineStr"/>
       <c r="BV15" t="inlineStr"/>
-      <c r="BW15" t="inlineStr"/>
+      <c r="BW15" t="n">
+        <v>1069834200</v>
+      </c>
       <c r="BX15" t="n">
-        <v>871040860</v>
+        <v>837295120</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3193,17 +3225,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3277,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>1040</v>
+        <v>1060</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3297,7 +3329,7 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>2754150</v>
+        <v>3354300</v>
       </c>
       <c r="BH16" t="inlineStr"/>
       <c r="BI16" t="inlineStr"/>
@@ -3307,10 +3339,10 @@
       <c r="BM16" t="inlineStr"/>
       <c r="BN16" t="inlineStr"/>
       <c r="BO16" t="n">
-        <v>2754150</v>
+        <v>3354300</v>
       </c>
       <c r="BP16" t="n">
-        <v>2897407950</v>
+        <v>3606050766.666667</v>
       </c>
       <c r="BQ16" t="inlineStr"/>
       <c r="BR16" t="inlineStr"/>
@@ -3320,7 +3352,7 @@
       <c r="BV16" t="inlineStr"/>
       <c r="BW16" t="inlineStr"/>
       <c r="BX16" t="n">
-        <v>2897407950</v>
+        <v>3606050766.666667</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3328,17 +3360,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -3380,7 +3412,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>441</v>
+        <v>521</v>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -3420,9 +3452,17 @@
       <c r="AS17" t="inlineStr"/>
       <c r="AT17" t="inlineStr"/>
       <c r="AU17" t="inlineStr"/>
-      <c r="AV17" t="inlineStr"/>
-      <c r="AW17" t="inlineStr"/>
-      <c r="AX17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>野村證券株式会社</t>
+        </is>
+      </c>
+      <c r="AW17" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="AX17" t="n">
+        <v>525000</v>
+      </c>
       <c r="AY17" t="inlineStr"/>
       <c r="AZ17" t="inlineStr"/>
       <c r="BA17" t="inlineStr"/>
@@ -3432,7 +3472,7 @@
       <c r="BE17" t="inlineStr"/>
       <c r="BF17" t="inlineStr"/>
       <c r="BG17" t="n">
-        <v>5849500</v>
+        <v>4432950</v>
       </c>
       <c r="BH17" t="inlineStr"/>
       <c r="BI17" t="inlineStr"/>
@@ -3442,10 +3482,10 @@
       <c r="BM17" t="inlineStr"/>
       <c r="BN17" t="inlineStr"/>
       <c r="BO17" t="n">
-        <v>5849500</v>
+        <v>4432950</v>
       </c>
       <c r="BP17" t="n">
-        <v>2571111900</v>
+        <v>2059503450</v>
       </c>
       <c r="BQ17" t="inlineStr"/>
       <c r="BR17" t="inlineStr"/>
@@ -3455,7 +3495,7 @@
       <c r="BV17" t="inlineStr"/>
       <c r="BW17" t="inlineStr"/>
       <c r="BX17" t="n">
-        <v>2571111900</v>
+        <v>2059503450</v>
       </c>
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
@@ -3463,17 +3503,17 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3554,9 @@
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>24800</v>
+      </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -3565,58 +3607,58 @@
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="BH18" t="n">
-        <v>700</v>
+        <v>860</v>
       </c>
       <c r="BI18" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="BJ18" t="n">
         <v>200</v>
       </c>
       <c r="BK18" t="n">
-        <v>500</v>
+        <v>366.6666666666667</v>
       </c>
       <c r="BL18" t="n">
-        <v>260</v>
+        <v>300</v>
       </c>
       <c r="BM18" t="n">
         <v>233.3333333333333</v>
       </c>
       <c r="BN18" t="n">
-        <v>250</v>
+        <v>266.6666666666667</v>
       </c>
       <c r="BO18" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="BP18" t="n">
-        <v>6186000</v>
+        <v>3750500</v>
       </c>
       <c r="BQ18" t="n">
-        <v>18946800</v>
+        <v>23184800</v>
       </c>
       <c r="BR18" t="n">
-        <v>7920750</v>
+        <v>2637666.666666667</v>
       </c>
       <c r="BS18" t="n">
         <v>5100000</v>
       </c>
       <c r="BT18" t="n">
-        <v>12464000</v>
+        <v>9128666.666666666</v>
       </c>
       <c r="BU18" t="n">
-        <v>6487600</v>
+        <v>7495000</v>
       </c>
       <c r="BV18" t="n">
         <v>5785000</v>
       </c>
       <c r="BW18" t="n">
-        <v>6204000</v>
+        <v>6586333.333333333</v>
       </c>
       <c r="BX18" t="n">
-        <v>6186000</v>
+        <v>3750500</v>
       </c>
       <c r="BY18" t="inlineStr"/>
       <c r="BZ18" t="inlineStr"/>
@@ -3624,17 +3666,17 @@
       <c r="CB18" t="inlineStr"/>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD18" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3718,7 @@
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
@@ -3764,58 +3806,58 @@
       <c r="BE19" t="inlineStr"/>
       <c r="BF19" t="inlineStr"/>
       <c r="BG19" t="n">
-        <v>2038676.2</v>
+        <v>2187308.8</v>
       </c>
       <c r="BH19" t="n">
-        <v>6430472.2</v>
+        <v>8023941.4</v>
       </c>
       <c r="BI19" t="n">
-        <v>13641653.6</v>
+        <v>12179098.2</v>
       </c>
       <c r="BJ19" t="n">
-        <v>4141412.2</v>
+        <v>3700743.4</v>
       </c>
       <c r="BK19" t="n">
-        <v>3244477</v>
+        <v>2944529.2</v>
       </c>
       <c r="BL19" t="n">
-        <v>3121484.8</v>
+        <v>3526709.6</v>
       </c>
       <c r="BM19" t="n">
-        <v>4791179.2</v>
+        <v>4273540.8</v>
       </c>
       <c r="BN19" t="n">
-        <v>1602701</v>
+        <v>1520583.8</v>
       </c>
       <c r="BO19" t="n">
-        <v>2038676.2</v>
+        <v>2187308.8</v>
       </c>
       <c r="BP19" t="n">
-        <v>54470723.6</v>
+        <v>58501407.4</v>
       </c>
       <c r="BQ19" t="n">
-        <v>204969357.4</v>
+        <v>216155375.6</v>
       </c>
       <c r="BR19" t="n">
-        <v>361089200</v>
+        <v>342936198.6</v>
       </c>
       <c r="BS19" t="n">
-        <v>112574536.8</v>
+        <v>97185042.40000001</v>
       </c>
       <c r="BT19" t="n">
-        <v>89198367.8</v>
+        <v>82702191</v>
       </c>
       <c r="BU19" t="n">
-        <v>91308870.59999999</v>
+        <v>103461676.8</v>
       </c>
       <c r="BV19" t="n">
-        <v>152865029.4</v>
+        <v>138019536.4</v>
       </c>
       <c r="BW19" t="n">
-        <v>47100971.4</v>
+        <v>43926478</v>
       </c>
       <c r="BX19" t="n">
-        <v>54470723.6</v>
+        <v>58501407.4</v>
       </c>
       <c r="BY19" t="inlineStr"/>
       <c r="BZ19" t="inlineStr"/>
@@ -3823,17 +3865,17 @@
       <c r="CB19" t="inlineStr"/>
       <c r="CC19" t="inlineStr">
         <is>
-          <t>20260407-210937</t>
+          <t>20260408-190054</t>
         </is>
       </c>
       <c r="CD19" t="inlineStr">
         <is>
-          <t>2026-04-07T12:09:37+00:00</t>
+          <t>2026-04-08T10:00:54+00:00</t>
         </is>
       </c>
       <c r="CE19" t="inlineStr">
         <is>
-          <t>2026-04-07T21:09:37+09:00</t>
+          <t>2026-04-08T19:00:54+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-09
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE19"/>
+  <dimension ref="A1:CE20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -971,58 +971,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>34400</v>
+        <v>29400</v>
       </c>
       <c r="BH2" t="n">
-        <v>14000</v>
+        <v>13800</v>
       </c>
       <c r="BI2" t="n">
-        <v>9200</v>
+        <v>12200</v>
       </c>
       <c r="BJ2" t="n">
-        <v>17800</v>
+        <v>14800</v>
       </c>
       <c r="BK2" t="n">
-        <v>21800</v>
+        <v>22000</v>
       </c>
       <c r="BL2" t="n">
-        <v>13200</v>
+        <v>14600</v>
       </c>
       <c r="BM2" t="n">
-        <v>14800</v>
+        <v>12600</v>
       </c>
       <c r="BN2" t="n">
-        <v>14600</v>
+        <v>19600</v>
       </c>
       <c r="BO2" t="n">
-        <v>34400</v>
+        <v>29400</v>
       </c>
       <c r="BP2" t="n">
-        <v>2473200</v>
+        <v>2134200</v>
       </c>
       <c r="BQ2" t="n">
-        <v>1110800</v>
+        <v>1093400</v>
       </c>
       <c r="BR2" t="n">
-        <v>742000</v>
+        <v>979000</v>
       </c>
       <c r="BS2" t="n">
-        <v>1394000</v>
+        <v>1153000</v>
       </c>
       <c r="BT2" t="n">
-        <v>1567400</v>
+        <v>1572800</v>
       </c>
       <c r="BU2" t="n">
-        <v>921000</v>
+        <v>1021400</v>
       </c>
       <c r="BV2" t="n">
-        <v>1033200</v>
+        <v>873200</v>
       </c>
       <c r="BW2" t="n">
-        <v>975800</v>
+        <v>1322400</v>
       </c>
       <c r="BX2" t="n">
-        <v>2473200</v>
+        <v>2134200</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1030,17 +1030,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2702</v>
+        <v>2593</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1194,58 +1194,58 @@
         <v>362132</v>
       </c>
       <c r="BG3" t="n">
-        <v>2882260</v>
+        <v>2576640</v>
       </c>
       <c r="BH3" t="n">
-        <v>1696600</v>
+        <v>1510060</v>
       </c>
       <c r="BI3" t="n">
-        <v>1586800</v>
+        <v>1600640</v>
       </c>
       <c r="BJ3" t="n">
-        <v>1915440</v>
+        <v>2243000</v>
       </c>
       <c r="BK3" t="n">
-        <v>1947500</v>
+        <v>1591980</v>
       </c>
       <c r="BL3" t="n">
-        <v>1697500</v>
+        <v>2497980</v>
       </c>
       <c r="BM3" t="n">
-        <v>3319560</v>
+        <v>2639900</v>
       </c>
       <c r="BN3" t="n">
-        <v>1890100</v>
+        <v>2330460</v>
       </c>
       <c r="BO3" t="n">
-        <v>2882260</v>
+        <v>2576640</v>
       </c>
       <c r="BP3" t="n">
-        <v>7053615520</v>
+        <v>6470640660</v>
       </c>
       <c r="BQ3" t="n">
-        <v>3461498820</v>
+        <v>3071635760</v>
       </c>
       <c r="BR3" t="n">
-        <v>3311761960</v>
+        <v>3348515080</v>
       </c>
       <c r="BS3" t="n">
-        <v>4198538840</v>
+        <v>4886821540</v>
       </c>
       <c r="BT3" t="n">
-        <v>3985863960</v>
+        <v>3260416720</v>
       </c>
       <c r="BU3" t="n">
-        <v>3756858500</v>
+        <v>5867370100</v>
       </c>
       <c r="BV3" t="n">
-        <v>8162734480</v>
+        <v>6411712660</v>
       </c>
       <c r="BW3" t="n">
-        <v>4201238040</v>
+        <v>5221066100</v>
       </c>
       <c r="BX3" t="n">
-        <v>7053615520</v>
+        <v>6470640660</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1253,17 +1253,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1393,58 +1393,58 @@
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="n">
-        <v>19560</v>
+        <v>17240</v>
       </c>
       <c r="BH4" t="n">
-        <v>73760</v>
+        <v>72740</v>
       </c>
       <c r="BI4" t="n">
-        <v>66220</v>
+        <v>68220</v>
       </c>
       <c r="BJ4" t="n">
-        <v>65160</v>
+        <v>72660</v>
       </c>
       <c r="BK4" t="n">
-        <v>71700</v>
+        <v>54760</v>
       </c>
       <c r="BL4" t="n">
-        <v>76300</v>
+        <v>79640</v>
       </c>
       <c r="BM4" t="n">
-        <v>71860</v>
+        <v>65180</v>
       </c>
       <c r="BN4" t="n">
-        <v>28740</v>
+        <v>28680</v>
       </c>
       <c r="BO4" t="n">
-        <v>19560</v>
+        <v>17240</v>
       </c>
       <c r="BP4" t="n">
-        <v>4404040</v>
+        <v>3875160</v>
       </c>
       <c r="BQ4" t="n">
-        <v>19529100</v>
+        <v>19193580</v>
       </c>
       <c r="BR4" t="n">
-        <v>16615420</v>
+        <v>16851020</v>
       </c>
       <c r="BS4" t="n">
-        <v>15752240</v>
+        <v>17113740</v>
       </c>
       <c r="BT4" t="n">
-        <v>16048700</v>
+        <v>12314000</v>
       </c>
       <c r="BU4" t="n">
-        <v>17525360</v>
+        <v>18335000</v>
       </c>
       <c r="BV4" t="n">
-        <v>16693620</v>
+        <v>15121560</v>
       </c>
       <c r="BW4" t="n">
-        <v>6423760</v>
+        <v>6394280</v>
       </c>
       <c r="BX4" t="n">
-        <v>4404040</v>
+        <v>3875160</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1452,17 +1452,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>845</v>
+        <v>780</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1604,54 +1604,54 @@
         <v>0</v>
       </c>
       <c r="BG5" t="n">
-        <v>49560</v>
+        <v>59880</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="n">
-        <v>2819200</v>
+        <v>1685750</v>
       </c>
       <c r="BJ5" t="n">
-        <v>469840</v>
+        <v>386680</v>
       </c>
       <c r="BK5" t="n">
-        <v>119060</v>
+        <v>112920</v>
       </c>
       <c r="BL5" t="n">
-        <v>101440</v>
+        <v>103520</v>
       </c>
       <c r="BM5" t="n">
-        <v>110180</v>
+        <v>101680</v>
       </c>
       <c r="BN5" t="n">
-        <v>96620</v>
+        <v>93360</v>
       </c>
       <c r="BO5" t="n">
-        <v>49560</v>
+        <v>59880</v>
       </c>
       <c r="BP5" t="n">
-        <v>41043140</v>
+        <v>48844340</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="n">
-        <v>3093295700</v>
+        <v>1822441950</v>
       </c>
       <c r="BS5" t="n">
-        <v>467821240</v>
+        <v>385590560</v>
       </c>
       <c r="BT5" t="n">
-        <v>120823060</v>
+        <v>114817520</v>
       </c>
       <c r="BU5" t="n">
-        <v>106038140</v>
+        <v>107356060</v>
       </c>
       <c r="BV5" t="n">
-        <v>101965460</v>
+        <v>91259340</v>
       </c>
       <c r="BW5" t="n">
-        <v>79752720</v>
+        <v>76451260</v>
       </c>
       <c r="BX5" t="n">
-        <v>41043140</v>
+        <v>48844340</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1659,17 +1659,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1315</v>
+        <v>1289</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1809,50 +1809,50 @@
         <v>0</v>
       </c>
       <c r="BG6" t="n">
-        <v>38880</v>
+        <v>41680</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="n">
-        <v>521300</v>
+        <v>451025</v>
       </c>
       <c r="BK6" t="n">
-        <v>115100</v>
+        <v>77680</v>
       </c>
       <c r="BL6" t="n">
-        <v>50100</v>
+        <v>46300</v>
       </c>
       <c r="BM6" t="n">
-        <v>44220</v>
+        <v>46820</v>
       </c>
       <c r="BN6" t="n">
-        <v>38260</v>
+        <v>34480</v>
       </c>
       <c r="BO6" t="n">
-        <v>38880</v>
+        <v>41680</v>
       </c>
       <c r="BP6" t="n">
-        <v>50626400</v>
+        <v>54262900</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="n">
-        <v>870049733.3333334</v>
+        <v>735964400</v>
       </c>
       <c r="BT6" t="n">
-        <v>161032720</v>
+        <v>109410200</v>
       </c>
       <c r="BU6" t="n">
-        <v>69102560</v>
+        <v>63034360</v>
       </c>
       <c r="BV6" t="n">
-        <v>56122460</v>
+        <v>59037820</v>
       </c>
       <c r="BW6" t="n">
-        <v>48400700</v>
+        <v>43737780</v>
       </c>
       <c r="BX6" t="n">
-        <v>50626400</v>
+        <v>54262900</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1860,17 +1860,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>696</v>
+        <v>688</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1976,7 +1976,7 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>19780</v>
+        <v>19340</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1984,16 +1984,16 @@
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="n">
-        <v>800000</v>
+        <v>494650</v>
       </c>
       <c r="BN7" t="n">
-        <v>116000</v>
+        <v>81840</v>
       </c>
       <c r="BO7" t="n">
-        <v>19780</v>
+        <v>19340</v>
       </c>
       <c r="BP7" t="n">
-        <v>13478760</v>
+        <v>13185240</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
@@ -2001,13 +2001,13 @@
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="n">
-        <v>643551400</v>
+        <v>394376800</v>
       </c>
       <c r="BW7" t="n">
-        <v>83306260</v>
+        <v>56793080</v>
       </c>
       <c r="BX7" t="n">
-        <v>13478760</v>
+        <v>13185240</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -2015,17 +2015,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>680</v>
+        <v>670</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2131,7 +2131,7 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
-        <v>80500</v>
+        <v>63160</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
@@ -2139,16 +2139,16 @@
       <c r="BK8" t="inlineStr"/>
       <c r="BL8" t="inlineStr"/>
       <c r="BM8" t="n">
-        <v>989300</v>
+        <v>662250</v>
       </c>
       <c r="BN8" t="n">
-        <v>313140</v>
+        <v>268820</v>
       </c>
       <c r="BO8" t="n">
-        <v>80500</v>
+        <v>63160</v>
       </c>
       <c r="BP8" t="n">
-        <v>54726680</v>
+        <v>42663760</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
@@ -2156,13 +2156,13 @@
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="n">
-        <v>737786900</v>
+        <v>486764000</v>
       </c>
       <c r="BW8" t="n">
-        <v>220473800</v>
+        <v>189029760</v>
       </c>
       <c r="BX8" t="n">
-        <v>54726680</v>
+        <v>42663760</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2170,17 +2170,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1470</v>
+        <v>1540</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2294,7 +2294,7 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>790120</v>
+        <v>726440</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
@@ -2303,13 +2303,13 @@
       <c r="BL9" t="inlineStr"/>
       <c r="BM9" t="inlineStr"/>
       <c r="BN9" t="n">
-        <v>6388500</v>
+        <v>5316140</v>
       </c>
       <c r="BO9" t="n">
-        <v>790120</v>
+        <v>726440</v>
       </c>
       <c r="BP9" t="n">
-        <v>1134294660</v>
+        <v>1050813620</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
@@ -2318,10 +2318,10 @@
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="inlineStr"/>
       <c r="BW9" t="n">
-        <v>9658056125</v>
+        <v>8028731360</v>
       </c>
       <c r="BX9" t="n">
-        <v>1134294660</v>
+        <v>1050813620</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2329,17 +2329,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1110</v>
+        <v>1136</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2429,9 +2429,17 @@
       <c r="AU10" t="n">
         <v>0</v>
       </c>
-      <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
-      <c r="AX10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>Morgan Stanley &amp; Co. International plc</t>
+        </is>
+      </c>
+      <c r="AW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0</v>
+      </c>
       <c r="AY10" t="inlineStr"/>
       <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="inlineStr"/>
@@ -2441,7 +2449,7 @@
       <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="n">
-        <v>498160</v>
+        <v>211840</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2449,12 +2457,14 @@
       <c r="BK10" t="inlineStr"/>
       <c r="BL10" t="inlineStr"/>
       <c r="BM10" t="inlineStr"/>
-      <c r="BN10" t="inlineStr"/>
+      <c r="BN10" t="n">
+        <v>1505100</v>
+      </c>
       <c r="BO10" t="n">
-        <v>498160</v>
+        <v>211840</v>
       </c>
       <c r="BP10" t="n">
-        <v>628596580</v>
+        <v>247418060</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2462,9 +2472,11 @@
       <c r="BT10" t="inlineStr"/>
       <c r="BU10" t="inlineStr"/>
       <c r="BV10" t="inlineStr"/>
-      <c r="BW10" t="inlineStr"/>
+      <c r="BW10" t="n">
+        <v>1988927000</v>
+      </c>
       <c r="BX10" t="n">
-        <v>628596580</v>
+        <v>247418060</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2472,17 +2484,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2536,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>432</v>
+        <v>412</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2584,7 +2596,7 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>23838300</v>
+        <v>24024360</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2593,13 +2605,13 @@
       <c r="BL11" t="inlineStr"/>
       <c r="BM11" t="inlineStr"/>
       <c r="BN11" t="n">
-        <v>10246600</v>
+        <v>10922450</v>
       </c>
       <c r="BO11" t="n">
-        <v>23838300</v>
+        <v>24024360</v>
       </c>
       <c r="BP11" t="n">
-        <v>11182826880</v>
+        <v>11174434740</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2608,10 +2620,10 @@
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="inlineStr"/>
       <c r="BW11" t="n">
-        <v>4296843900</v>
+        <v>4758047550</v>
       </c>
       <c r="BX11" t="n">
-        <v>11182826880</v>
+        <v>11174434740</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2619,17 +2631,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2683,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2739,7 +2751,7 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>222760</v>
+        <v>201040</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2748,13 +2760,13 @@
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="n">
-        <v>244800</v>
+        <v>247150</v>
       </c>
       <c r="BO12" t="n">
-        <v>222760</v>
+        <v>201040</v>
       </c>
       <c r="BP12" t="n">
-        <v>92551780</v>
+        <v>83837520</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2763,10 +2775,10 @@
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="n">
-        <v>102953000</v>
+        <v>102748250</v>
       </c>
       <c r="BX12" t="n">
-        <v>92551780</v>
+        <v>83837520</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2774,17 +2786,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2838,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>944</v>
+        <v>949</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2886,7 +2898,7 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="n">
-        <v>177860</v>
+        <v>150280</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2895,13 +2907,13 @@
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="n">
-        <v>91400</v>
+        <v>155450</v>
       </c>
       <c r="BO13" t="n">
-        <v>177860</v>
+        <v>150280</v>
       </c>
       <c r="BP13" t="n">
-        <v>166188720</v>
+        <v>140007220</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2910,10 +2922,10 @@
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="n">
-        <v>81195700</v>
+        <v>144927050</v>
       </c>
       <c r="BX13" t="n">
-        <v>166188720</v>
+        <v>140007220</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2921,17 +2933,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2985,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1909</v>
+        <v>1863</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -3043,7 +3055,7 @@
         <v>194633</v>
       </c>
       <c r="BG14" t="n">
-        <v>199220</v>
+        <v>184180</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -3052,13 +3064,13 @@
       <c r="BL14" t="inlineStr"/>
       <c r="BM14" t="inlineStr"/>
       <c r="BN14" t="n">
-        <v>157200</v>
+        <v>195250</v>
       </c>
       <c r="BO14" t="n">
-        <v>199220</v>
+        <v>184180</v>
       </c>
       <c r="BP14" t="n">
-        <v>369146580</v>
+        <v>343918960</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -3067,10 +3079,10 @@
       <c r="BU14" t="inlineStr"/>
       <c r="BV14" t="inlineStr"/>
       <c r="BW14" t="n">
-        <v>278865400</v>
+        <v>351530650</v>
       </c>
       <c r="BX14" t="n">
-        <v>369146580</v>
+        <v>343918960</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -3078,17 +3090,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3142,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>441</v>
+        <v>430</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -3190,7 +3202,7 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>1942060</v>
+        <v>1845660</v>
       </c>
       <c r="BH15" t="inlineStr"/>
       <c r="BI15" t="inlineStr"/>
@@ -3199,13 +3211,13 @@
       <c r="BL15" t="inlineStr"/>
       <c r="BM15" t="inlineStr"/>
       <c r="BN15" t="n">
-        <v>2383200</v>
+        <v>2210850</v>
       </c>
       <c r="BO15" t="n">
-        <v>1942060</v>
+        <v>1845660</v>
       </c>
       <c r="BP15" t="n">
-        <v>837295120</v>
+        <v>791971060</v>
       </c>
       <c r="BQ15" t="inlineStr"/>
       <c r="BR15" t="inlineStr"/>
@@ -3214,10 +3226,10 @@
       <c r="BU15" t="inlineStr"/>
       <c r="BV15" t="inlineStr"/>
       <c r="BW15" t="n">
-        <v>1069834200</v>
+        <v>984957200</v>
       </c>
       <c r="BX15" t="n">
-        <v>837295120</v>
+        <v>791971060</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3225,17 +3237,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3289,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>1060</v>
+        <v>1020</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3329,7 +3341,7 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>3354300</v>
+        <v>2872425</v>
       </c>
       <c r="BH16" t="inlineStr"/>
       <c r="BI16" t="inlineStr"/>
@@ -3339,10 +3351,10 @@
       <c r="BM16" t="inlineStr"/>
       <c r="BN16" t="inlineStr"/>
       <c r="BO16" t="n">
-        <v>3354300</v>
+        <v>2872425</v>
       </c>
       <c r="BP16" t="n">
-        <v>3606050766.666667</v>
+        <v>3084106450</v>
       </c>
       <c r="BQ16" t="inlineStr"/>
       <c r="BR16" t="inlineStr"/>
@@ -3352,7 +3364,7 @@
       <c r="BV16" t="inlineStr"/>
       <c r="BW16" t="inlineStr"/>
       <c r="BX16" t="n">
-        <v>3606050766.666667</v>
+        <v>3084106450</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3360,17 +3372,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3424,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>521</v>
+        <v>621</v>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -3472,7 +3484,7 @@
       <c r="BE17" t="inlineStr"/>
       <c r="BF17" t="inlineStr"/>
       <c r="BG17" t="n">
-        <v>4432950</v>
+        <v>3251933.333333333</v>
       </c>
       <c r="BH17" t="inlineStr"/>
       <c r="BI17" t="inlineStr"/>
@@ -3482,10 +3494,10 @@
       <c r="BM17" t="inlineStr"/>
       <c r="BN17" t="inlineStr"/>
       <c r="BO17" t="n">
-        <v>4432950</v>
+        <v>3251933.333333333</v>
       </c>
       <c r="BP17" t="n">
-        <v>2059503450</v>
+        <v>1553883300</v>
       </c>
       <c r="BQ17" t="inlineStr"/>
       <c r="BR17" t="inlineStr"/>
@@ -3495,7 +3507,7 @@
       <c r="BV17" t="inlineStr"/>
       <c r="BW17" t="inlineStr"/>
       <c r="BX17" t="n">
-        <v>2059503450</v>
+        <v>1553883300</v>
       </c>
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
@@ -3503,29 +3515,29 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>550A</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>日本銀行</t>
+          <t>ソフトテックス</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3535,12 +3547,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>銀行</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>銀行業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3555,7 +3567,7 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>24800</v>
+        <v>2613</v>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
@@ -3607,58 +3619,30 @@
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="n">
-        <v>150</v>
-      </c>
-      <c r="BH18" t="n">
-        <v>860</v>
-      </c>
-      <c r="BI18" t="n">
-        <v>100</v>
-      </c>
-      <c r="BJ18" t="n">
-        <v>200</v>
-      </c>
-      <c r="BK18" t="n">
-        <v>366.6666666666667</v>
-      </c>
-      <c r="BL18" t="n">
-        <v>300</v>
-      </c>
-      <c r="BM18" t="n">
-        <v>233.3333333333333</v>
-      </c>
-      <c r="BN18" t="n">
-        <v>266.6666666666667</v>
-      </c>
+        <v>1185300</v>
+      </c>
+      <c r="BH18" t="inlineStr"/>
+      <c r="BI18" t="inlineStr"/>
+      <c r="BJ18" t="inlineStr"/>
+      <c r="BK18" t="inlineStr"/>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="inlineStr"/>
+      <c r="BN18" t="inlineStr"/>
       <c r="BO18" t="n">
-        <v>150</v>
+        <v>1185300</v>
       </c>
       <c r="BP18" t="n">
-        <v>3750500</v>
-      </c>
-      <c r="BQ18" t="n">
-        <v>23184800</v>
-      </c>
-      <c r="BR18" t="n">
-        <v>2637666.666666667</v>
-      </c>
-      <c r="BS18" t="n">
-        <v>5100000</v>
-      </c>
-      <c r="BT18" t="n">
-        <v>9128666.666666666</v>
-      </c>
-      <c r="BU18" t="n">
-        <v>7495000</v>
-      </c>
-      <c r="BV18" t="n">
-        <v>5785000</v>
-      </c>
-      <c r="BW18" t="n">
-        <v>6586333.333333333</v>
-      </c>
+        <v>3532839500</v>
+      </c>
+      <c r="BQ18" t="inlineStr"/>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr"/>
+      <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="inlineStr"/>
       <c r="BX18" t="n">
-        <v>3750500</v>
+        <v>3532839500</v>
       </c>
       <c r="BY18" t="inlineStr"/>
       <c r="BZ18" t="inlineStr"/>
@@ -3666,29 +3650,29 @@
       <c r="CB18" t="inlineStr"/>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD18" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9399</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+          <t>日本銀行</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3698,12 +3682,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>銀行</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>銀行業</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3717,9 +3701,7 @@
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>27</v>
-      </c>
+      <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -3740,60 +3722,24 @@
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE19" t="n">
-        <v>122230</v>
-      </c>
-      <c r="AF19" t="n">
-        <v>202741</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>204885</v>
-      </c>
-      <c r="AH19" t="n">
-        <v>97185</v>
-      </c>
-      <c r="AI19" t="n">
-        <v>93675</v>
-      </c>
-      <c r="AJ19" t="n">
-        <v>126528</v>
-      </c>
-      <c r="AK19" t="n">
-        <v>99264</v>
-      </c>
-      <c r="AL19" t="n">
-        <v>96080</v>
-      </c>
-      <c r="AM19" t="n">
-        <v>122230</v>
-      </c>
-      <c r="AN19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU19" t="n">
-        <v>0</v>
-      </c>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
       <c r="AV19" t="inlineStr"/>
       <c r="AW19" t="inlineStr"/>
       <c r="AX19" t="inlineStr"/>
@@ -3806,58 +3752,58 @@
       <c r="BE19" t="inlineStr"/>
       <c r="BF19" t="inlineStr"/>
       <c r="BG19" t="n">
-        <v>2187308.8</v>
+        <v>150</v>
       </c>
       <c r="BH19" t="n">
-        <v>8023941.4</v>
+        <v>780</v>
       </c>
       <c r="BI19" t="n">
-        <v>12179098.2</v>
+        <v>100</v>
       </c>
       <c r="BJ19" t="n">
-        <v>3700743.4</v>
+        <v>450</v>
       </c>
       <c r="BK19" t="n">
-        <v>2944529.2</v>
+        <v>166.6666666666667</v>
       </c>
       <c r="BL19" t="n">
-        <v>3526709.6</v>
+        <v>325</v>
       </c>
       <c r="BM19" t="n">
-        <v>4273540.8</v>
+        <v>233.3333333333333</v>
       </c>
       <c r="BN19" t="n">
-        <v>1520583.8</v>
+        <v>300</v>
       </c>
       <c r="BO19" t="n">
-        <v>2187308.8</v>
+        <v>150</v>
       </c>
       <c r="BP19" t="n">
-        <v>58501407.4</v>
+        <v>3750500</v>
       </c>
       <c r="BQ19" t="n">
-        <v>216155375.6</v>
+        <v>21083400</v>
       </c>
       <c r="BR19" t="n">
-        <v>342936198.6</v>
+        <v>2645000</v>
       </c>
       <c r="BS19" t="n">
-        <v>97185042.40000001</v>
+        <v>11285000</v>
       </c>
       <c r="BT19" t="n">
-        <v>82702191</v>
+        <v>4161000</v>
       </c>
       <c r="BU19" t="n">
-        <v>103461676.8</v>
+        <v>8085750</v>
       </c>
       <c r="BV19" t="n">
-        <v>138019536.4</v>
+        <v>5813333.333333333</v>
       </c>
       <c r="BW19" t="n">
-        <v>43926478</v>
+        <v>7372000</v>
       </c>
       <c r="BX19" t="n">
-        <v>58501407.4</v>
+        <v>3750500</v>
       </c>
       <c r="BY19" t="inlineStr"/>
       <c r="BZ19" t="inlineStr"/>
@@ -3865,17 +3811,216 @@
       <c r="CB19" t="inlineStr"/>
       <c r="CC19" t="inlineStr">
         <is>
-          <t>20260408-210915</t>
+          <t>20260409-190052</t>
         </is>
       </c>
       <c r="CD19" t="inlineStr">
         <is>
-          <t>2026-04-08T12:09:15+00:00</t>
+          <t>2026-04-09T10:00:52+00:00</t>
         </is>
       </c>
       <c r="CE19" t="inlineStr">
         <is>
-          <t>2026-04-08T21:09:15+09:00</t>
+          <t>2026-04-09T19:00:52+09:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>9399</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>スタンダード</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>情報通信・サービスその他</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>情報･通信業</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>fins_summary_api_fail</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>RuntimeError: empty /fins/summary</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>27</v>
+      </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>122230</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>202741</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>204885</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>97185</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>93675</v>
+      </c>
+      <c r="AJ20" t="n">
+        <v>126528</v>
+      </c>
+      <c r="AK20" t="n">
+        <v>99264</v>
+      </c>
+      <c r="AL20" t="n">
+        <v>96080</v>
+      </c>
+      <c r="AM20" t="n">
+        <v>122230</v>
+      </c>
+      <c r="AN20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
+      <c r="BA20" t="inlineStr"/>
+      <c r="BB20" t="inlineStr"/>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+      <c r="BE20" t="inlineStr"/>
+      <c r="BF20" t="inlineStr"/>
+      <c r="BG20" t="n">
+        <v>1690468.6</v>
+      </c>
+      <c r="BH20" t="n">
+        <v>11028008.4</v>
+      </c>
+      <c r="BI20" t="n">
+        <v>9570452.800000001</v>
+      </c>
+      <c r="BJ20" t="n">
+        <v>3267717.4</v>
+      </c>
+      <c r="BK20" t="n">
+        <v>3674551.2</v>
+      </c>
+      <c r="BL20" t="n">
+        <v>4241035.4</v>
+      </c>
+      <c r="BM20" t="n">
+        <v>3010975.8</v>
+      </c>
+      <c r="BN20" t="n">
+        <v>1764609.6</v>
+      </c>
+      <c r="BO20" t="n">
+        <v>1690468.6</v>
+      </c>
+      <c r="BP20" t="n">
+        <v>45282081.2</v>
+      </c>
+      <c r="BQ20" t="n">
+        <v>272405338.6</v>
+      </c>
+      <c r="BR20" t="n">
+        <v>292344615.4</v>
+      </c>
+      <c r="BS20" t="n">
+        <v>83737882</v>
+      </c>
+      <c r="BT20" t="n">
+        <v>107086813.6</v>
+      </c>
+      <c r="BU20" t="n">
+        <v>131265781.6</v>
+      </c>
+      <c r="BV20" t="n">
+        <v>92793402.59999999</v>
+      </c>
+      <c r="BW20" t="n">
+        <v>48812478.4</v>
+      </c>
+      <c r="BX20" t="n">
+        <v>45282081.2</v>
+      </c>
+      <c r="BY20" t="inlineStr"/>
+      <c r="BZ20" t="inlineStr"/>
+      <c r="CA20" t="inlineStr"/>
+      <c r="CB20" t="inlineStr"/>
+      <c r="CC20" t="inlineStr">
+        <is>
+          <t>20260409-190052</t>
+        </is>
+      </c>
+      <c r="CD20" t="inlineStr">
+        <is>
+          <t>2026-04-09T10:00:52+00:00</t>
+        </is>
+      </c>
+      <c r="CE20" t="inlineStr">
+        <is>
+          <t>2026-04-09T19:00:52+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-10
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -912,29 +912,27 @@
         <v>31000</v>
       </c>
       <c r="AF2" t="n">
-        <v>17000</v>
+        <v>15000</v>
       </c>
       <c r="AG2" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="AH2" t="n">
-        <v>16000</v>
+        <v>33000</v>
       </c>
       <c r="AI2" t="n">
-        <v>33000</v>
+        <v>45000</v>
       </c>
       <c r="AJ2" t="n">
-        <v>45000</v>
+        <v>46000</v>
       </c>
       <c r="AK2" t="n">
-        <v>46000</v>
+        <v>43000</v>
       </c>
       <c r="AL2" t="n">
-        <v>43000</v>
-      </c>
-      <c r="AM2" t="n">
         <v>31000</v>
       </c>
+      <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="n">
         <v>0</v>
       </c>
@@ -956,9 +954,7 @@
       <c r="AT2" t="n">
         <v>0</v>
       </c>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU2" t="inlineStr"/>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
@@ -971,58 +967,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>29400</v>
+        <v>19600</v>
       </c>
       <c r="BH2" t="n">
-        <v>13800</v>
+        <v>8600</v>
       </c>
       <c r="BI2" t="n">
-        <v>12200</v>
+        <v>13400</v>
       </c>
       <c r="BJ2" t="n">
         <v>14800</v>
       </c>
       <c r="BK2" t="n">
-        <v>22000</v>
+        <v>22800</v>
       </c>
       <c r="BL2" t="n">
-        <v>14600</v>
+        <v>14000</v>
       </c>
       <c r="BM2" t="n">
-        <v>12600</v>
+        <v>13800</v>
       </c>
       <c r="BN2" t="n">
+        <v>27200</v>
+      </c>
+      <c r="BO2" t="n">
         <v>19600</v>
       </c>
-      <c r="BO2" t="n">
-        <v>29400</v>
-      </c>
       <c r="BP2" t="n">
-        <v>2134200</v>
+        <v>1452600</v>
       </c>
       <c r="BQ2" t="n">
-        <v>1093400</v>
+        <v>677000</v>
       </c>
       <c r="BR2" t="n">
-        <v>979000</v>
+        <v>1074800</v>
       </c>
       <c r="BS2" t="n">
-        <v>1153000</v>
+        <v>1151800</v>
       </c>
       <c r="BT2" t="n">
-        <v>1572800</v>
+        <v>1615200</v>
       </c>
       <c r="BU2" t="n">
-        <v>1021400</v>
+        <v>981400</v>
       </c>
       <c r="BV2" t="n">
-        <v>873200</v>
+        <v>947600</v>
       </c>
       <c r="BW2" t="n">
-        <v>1322400</v>
+        <v>1862000</v>
       </c>
       <c r="BX2" t="n">
-        <v>2134200</v>
+        <v>1452600</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1030,17 +1026,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1078,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2593</v>
+        <v>2832</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1111,53 +1107,49 @@
         <v>3149100</v>
       </c>
       <c r="AF3" t="n">
-        <v>3576100</v>
+        <v>3398500</v>
       </c>
       <c r="AG3" t="n">
-        <v>3398500</v>
+        <v>3082900</v>
       </c>
       <c r="AH3" t="n">
-        <v>3082900</v>
+        <v>3002100</v>
       </c>
       <c r="AI3" t="n">
-        <v>3002100</v>
+        <v>2859200</v>
       </c>
       <c r="AJ3" t="n">
-        <v>2859200</v>
+        <v>2911500</v>
       </c>
       <c r="AK3" t="n">
-        <v>2911500</v>
+        <v>3235400</v>
       </c>
       <c r="AL3" t="n">
-        <v>3235400</v>
-      </c>
-      <c r="AM3" t="n">
         <v>3149100</v>
       </c>
+      <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="n">
-        <v>762600</v>
+        <v>619800</v>
       </c>
       <c r="AO3" t="n">
-        <v>619800</v>
+        <v>650000</v>
       </c>
       <c r="AP3" t="n">
-        <v>650000</v>
+        <v>269900</v>
       </c>
       <c r="AQ3" t="n">
-        <v>269900</v>
+        <v>275900</v>
       </c>
       <c r="AR3" t="n">
-        <v>275900</v>
+        <v>283300</v>
       </c>
       <c r="AS3" t="n">
-        <v>283300</v>
+        <v>227300</v>
       </c>
       <c r="AT3" t="n">
-        <v>227300</v>
-      </c>
-      <c r="AU3" t="n">
         <v>236100</v>
       </c>
+      <c r="AU3" t="inlineStr"/>
       <c r="AV3" t="inlineStr">
         <is>
           <t>モルガン・スタンレーMUFG証券株式会社、Nomura International plc</t>
@@ -1194,58 +1186,58 @@
         <v>362132</v>
       </c>
       <c r="BG3" t="n">
-        <v>2576640</v>
+        <v>3191940</v>
       </c>
       <c r="BH3" t="n">
-        <v>1510060</v>
+        <v>1374680</v>
       </c>
       <c r="BI3" t="n">
-        <v>1600640</v>
+        <v>1707980</v>
       </c>
       <c r="BJ3" t="n">
-        <v>2243000</v>
+        <v>2332920</v>
       </c>
       <c r="BK3" t="n">
-        <v>1591980</v>
+        <v>1349720</v>
       </c>
       <c r="BL3" t="n">
-        <v>2497980</v>
+        <v>3208240</v>
       </c>
       <c r="BM3" t="n">
-        <v>2639900</v>
+        <v>2079840</v>
       </c>
       <c r="BN3" t="n">
-        <v>2330460</v>
+        <v>2432780</v>
       </c>
       <c r="BO3" t="n">
-        <v>2576640</v>
+        <v>3191940</v>
       </c>
       <c r="BP3" t="n">
-        <v>6470640660</v>
+        <v>8388170740</v>
       </c>
       <c r="BQ3" t="n">
-        <v>3071635760</v>
+        <v>2781072700</v>
       </c>
       <c r="BR3" t="n">
-        <v>3348515080</v>
+        <v>3574143180</v>
       </c>
       <c r="BS3" t="n">
-        <v>4886821540</v>
+        <v>5081670080</v>
       </c>
       <c r="BT3" t="n">
-        <v>3260416720</v>
+        <v>2747044860</v>
       </c>
       <c r="BU3" t="n">
-        <v>5867370100</v>
+        <v>7781799320</v>
       </c>
       <c r="BV3" t="n">
-        <v>6411712660</v>
+        <v>4889458760</v>
       </c>
       <c r="BW3" t="n">
-        <v>5221066100</v>
+        <v>5462913800</v>
       </c>
       <c r="BX3" t="n">
-        <v>6470640660</v>
+        <v>8388170740</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1253,17 +1245,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1297,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1334,29 +1326,27 @@
         <v>76800</v>
       </c>
       <c r="AF4" t="n">
-        <v>58100</v>
+        <v>57400</v>
       </c>
       <c r="AG4" t="n">
-        <v>57400</v>
+        <v>57100</v>
       </c>
       <c r="AH4" t="n">
-        <v>57100</v>
+        <v>57700</v>
       </c>
       <c r="AI4" t="n">
-        <v>57700</v>
+        <v>78800</v>
       </c>
       <c r="AJ4" t="n">
-        <v>78800</v>
+        <v>80100</v>
       </c>
       <c r="AK4" t="n">
-        <v>80100</v>
+        <v>76600</v>
       </c>
       <c r="AL4" t="n">
-        <v>76600</v>
-      </c>
-      <c r="AM4" t="n">
         <v>76800</v>
       </c>
+      <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="n">
         <v>0</v>
       </c>
@@ -1378,9 +1368,7 @@
       <c r="AT4" t="n">
         <v>0</v>
       </c>
-      <c r="AU4" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="inlineStr"/>
@@ -1393,58 +1381,58 @@
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="n">
-        <v>17240</v>
+        <v>18480</v>
       </c>
       <c r="BH4" t="n">
-        <v>72740</v>
+        <v>79860</v>
       </c>
       <c r="BI4" t="n">
-        <v>68220</v>
+        <v>59380</v>
       </c>
       <c r="BJ4" t="n">
-        <v>72660</v>
+        <v>68320</v>
       </c>
       <c r="BK4" t="n">
-        <v>54760</v>
+        <v>58860</v>
       </c>
       <c r="BL4" t="n">
-        <v>79640</v>
+        <v>79320</v>
       </c>
       <c r="BM4" t="n">
-        <v>65180</v>
+        <v>63700</v>
       </c>
       <c r="BN4" t="n">
-        <v>28680</v>
+        <v>26220</v>
       </c>
       <c r="BO4" t="n">
-        <v>17240</v>
+        <v>18480</v>
       </c>
       <c r="BP4" t="n">
-        <v>3875160</v>
+        <v>4174480</v>
       </c>
       <c r="BQ4" t="n">
-        <v>19193580</v>
+        <v>20766940</v>
       </c>
       <c r="BR4" t="n">
-        <v>16851020</v>
+        <v>14569660</v>
       </c>
       <c r="BS4" t="n">
-        <v>17113740</v>
+        <v>15978460</v>
       </c>
       <c r="BT4" t="n">
-        <v>12314000</v>
+        <v>13221880</v>
       </c>
       <c r="BU4" t="n">
-        <v>18335000</v>
+        <v>18258940</v>
       </c>
       <c r="BV4" t="n">
-        <v>15121560</v>
+        <v>14797380</v>
       </c>
       <c r="BW4" t="n">
-        <v>6394280</v>
+        <v>5820080</v>
       </c>
       <c r="BX4" t="n">
-        <v>3875160</v>
+        <v>4174480</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1452,17 +1440,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1492,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>780</v>
+        <v>743</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1533,27 +1521,29 @@
         <v>234400</v>
       </c>
       <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
+      <c r="AG5" t="n">
+        <v>222300</v>
+      </c>
       <c r="AH5" t="n">
-        <v>222300</v>
+        <v>216400</v>
       </c>
       <c r="AI5" t="n">
-        <v>216400</v>
+        <v>204600</v>
       </c>
       <c r="AJ5" t="n">
-        <v>204600</v>
+        <v>212600</v>
       </c>
       <c r="AK5" t="n">
-        <v>212600</v>
+        <v>227900</v>
       </c>
       <c r="AL5" t="n">
-        <v>227900</v>
-      </c>
-      <c r="AM5" t="n">
         <v>234400</v>
       </c>
+      <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
+      <c r="AO5" t="n">
+        <v>0</v>
+      </c>
       <c r="AP5" t="n">
         <v>0</v>
       </c>
@@ -1564,14 +1554,12 @@
         <v>0</v>
       </c>
       <c r="AS5" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="AT5" t="n">
-        <v>400</v>
-      </c>
-      <c r="AU5" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr">
         <is>
           <t>野村證券株式会社</t>
@@ -1584,18 +1572,20 @@
         <v>0</v>
       </c>
       <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
+      <c r="AZ5" t="n">
+        <v>2482900</v>
+      </c>
       <c r="BA5" t="n">
-        <v>2482900</v>
+        <v>1080200</v>
       </c>
       <c r="BB5" t="n">
         <v>1080200</v>
       </c>
       <c r="BC5" t="n">
-        <v>1080200</v>
+        <v>1041600</v>
       </c>
       <c r="BD5" t="n">
-        <v>1041600</v>
+        <v>0</v>
       </c>
       <c r="BE5" t="n">
         <v>0</v>
@@ -1604,54 +1594,54 @@
         <v>0</v>
       </c>
       <c r="BG5" t="n">
-        <v>59880</v>
+        <v>76980</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="n">
-        <v>1685750</v>
+        <v>1302366.666666667</v>
       </c>
       <c r="BJ5" t="n">
-        <v>386680</v>
+        <v>300260</v>
       </c>
       <c r="BK5" t="n">
-        <v>112920</v>
+        <v>111260</v>
       </c>
       <c r="BL5" t="n">
-        <v>103520</v>
+        <v>117620</v>
       </c>
       <c r="BM5" t="n">
-        <v>101680</v>
+        <v>86180</v>
       </c>
       <c r="BN5" t="n">
-        <v>93360</v>
+        <v>82320</v>
       </c>
       <c r="BO5" t="n">
-        <v>59880</v>
+        <v>76980</v>
       </c>
       <c r="BP5" t="n">
-        <v>48844340</v>
+        <v>61452380</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="n">
-        <v>1822441950</v>
+        <v>1383993266.666667</v>
       </c>
       <c r="BS5" t="n">
-        <v>385590560</v>
+        <v>305469720</v>
       </c>
       <c r="BT5" t="n">
-        <v>114817520</v>
+        <v>113793920</v>
       </c>
       <c r="BU5" t="n">
-        <v>107356060</v>
+        <v>118662180</v>
       </c>
       <c r="BV5" t="n">
-        <v>91259340</v>
+        <v>74449720</v>
       </c>
       <c r="BW5" t="n">
-        <v>76451260</v>
+        <v>67033160</v>
       </c>
       <c r="BX5" t="n">
-        <v>48844340</v>
+        <v>61452380</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1659,17 +1649,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1701,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1289</v>
+        <v>1279</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1740,27 +1730,29 @@
         <v>183000</v>
       </c>
       <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="inlineStr"/>
+      <c r="AG6" t="n">
+        <v>101900</v>
+      </c>
       <c r="AH6" t="n">
-        <v>101900</v>
+        <v>201600</v>
       </c>
       <c r="AI6" t="n">
-        <v>201600</v>
+        <v>200600</v>
       </c>
       <c r="AJ6" t="n">
-        <v>200600</v>
+        <v>183800</v>
       </c>
       <c r="AK6" t="n">
-        <v>183800</v>
+        <v>200400</v>
       </c>
       <c r="AL6" t="n">
-        <v>200400</v>
-      </c>
-      <c r="AM6" t="n">
         <v>183000</v>
       </c>
+      <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
+      <c r="AO6" t="n">
+        <v>0</v>
+      </c>
       <c r="AP6" t="n">
         <v>0</v>
       </c>
@@ -1776,9 +1768,7 @@
       <c r="AT6" t="n">
         <v>0</v>
       </c>
-      <c r="AU6" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU6" t="inlineStr"/>
       <c r="AV6" t="inlineStr">
         <is>
           <t>野村證券株式会社</t>
@@ -1792,15 +1782,17 @@
       </c>
       <c r="AY6" t="inlineStr"/>
       <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
+      <c r="BA6" t="n">
+        <v>160600</v>
+      </c>
       <c r="BB6" t="n">
-        <v>160600</v>
+        <v>151600</v>
       </c>
       <c r="BC6" t="n">
-        <v>151600</v>
+        <v>127100</v>
       </c>
       <c r="BD6" t="n">
-        <v>127100</v>
+        <v>0</v>
       </c>
       <c r="BE6" t="n">
         <v>0</v>
@@ -1809,50 +1801,50 @@
         <v>0</v>
       </c>
       <c r="BG6" t="n">
-        <v>41680</v>
+        <v>46940</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="n">
-        <v>451025</v>
+        <v>387740</v>
       </c>
       <c r="BK6" t="n">
-        <v>77680</v>
+        <v>57680</v>
       </c>
       <c r="BL6" t="n">
-        <v>46300</v>
+        <v>51540</v>
       </c>
       <c r="BM6" t="n">
-        <v>46820</v>
+        <v>40660</v>
       </c>
       <c r="BN6" t="n">
-        <v>34480</v>
+        <v>32720</v>
       </c>
       <c r="BO6" t="n">
-        <v>41680</v>
+        <v>46940</v>
       </c>
       <c r="BP6" t="n">
-        <v>54262900</v>
+        <v>60955240</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="n">
-        <v>735964400</v>
+        <v>626504680</v>
       </c>
       <c r="BT6" t="n">
-        <v>109410200</v>
+        <v>81473640</v>
       </c>
       <c r="BU6" t="n">
-        <v>63034360</v>
+        <v>69089120</v>
       </c>
       <c r="BV6" t="n">
-        <v>59037820</v>
+        <v>50832820</v>
       </c>
       <c r="BW6" t="n">
-        <v>43737780</v>
+        <v>41588180</v>
       </c>
       <c r="BX6" t="n">
-        <v>54262900</v>
+        <v>60955240</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1860,17 +1852,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1904,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>688</v>
+        <v>682</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1945,25 +1937,25 @@
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+      <c r="AK7" t="n">
+        <v>49900</v>
+      </c>
       <c r="AL7" t="n">
-        <v>49900</v>
-      </c>
-      <c r="AM7" t="n">
         <v>56200</v>
       </c>
+      <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
       <c r="AT7" t="n">
         <v>0</v>
       </c>
-      <c r="AU7" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU7" t="inlineStr"/>
       <c r="AV7" t="inlineStr"/>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
@@ -1976,7 +1968,7 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>19340</v>
+        <v>20400</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1984,16 +1976,16 @@
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="n">
-        <v>494650</v>
+        <v>406400</v>
       </c>
       <c r="BN7" t="n">
-        <v>81840</v>
+        <v>38440</v>
       </c>
       <c r="BO7" t="n">
-        <v>19340</v>
+        <v>20400</v>
       </c>
       <c r="BP7" t="n">
-        <v>13185240</v>
+        <v>13911860</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
@@ -2001,13 +1993,13 @@
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="n">
-        <v>394376800</v>
+        <v>316942333.3333333</v>
       </c>
       <c r="BW7" t="n">
-        <v>56793080</v>
+        <v>26133940</v>
       </c>
       <c r="BX7" t="n">
-        <v>13185240</v>
+        <v>13911860</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -2015,17 +2007,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2059,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>670</v>
+        <v>664</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2100,25 +2092,25 @@
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+      <c r="AK8" t="n">
+        <v>70700</v>
+      </c>
       <c r="AL8" t="n">
-        <v>70700</v>
-      </c>
-      <c r="AM8" t="n">
         <v>106000</v>
       </c>
+      <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
+      <c r="AS8" t="n">
+        <v>1000</v>
+      </c>
       <c r="AT8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AU8" t="inlineStr"/>
       <c r="AV8" t="inlineStr"/>
       <c r="AW8" t="inlineStr"/>
       <c r="AX8" t="inlineStr"/>
@@ -2131,7 +2123,7 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
-        <v>63160</v>
+        <v>54260</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
@@ -2139,16 +2131,16 @@
       <c r="BK8" t="inlineStr"/>
       <c r="BL8" t="inlineStr"/>
       <c r="BM8" t="n">
-        <v>662250</v>
+        <v>608533.3333333334</v>
       </c>
       <c r="BN8" t="n">
-        <v>268820</v>
+        <v>187780</v>
       </c>
       <c r="BO8" t="n">
-        <v>63160</v>
+        <v>54260</v>
       </c>
       <c r="BP8" t="n">
-        <v>42663760</v>
+        <v>36525580</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
@@ -2156,13 +2148,13 @@
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="n">
-        <v>486764000</v>
+        <v>445297133.3333333</v>
       </c>
       <c r="BW8" t="n">
-        <v>189029760</v>
+        <v>129544760</v>
       </c>
       <c r="BX8" t="n">
-        <v>42663760</v>
+        <v>36525580</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2170,17 +2162,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2214,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1540</v>
+        <v>1502</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2255,25 +2247,25 @@
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
+      <c r="AK9" t="n">
+        <v>408200</v>
+      </c>
       <c r="AL9" t="n">
-        <v>408200</v>
-      </c>
-      <c r="AM9" t="n">
         <v>634100</v>
       </c>
+      <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr"/>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
       <c r="AT9" t="n">
         <v>0</v>
       </c>
-      <c r="AU9" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU9" t="inlineStr"/>
       <c r="AV9" t="inlineStr">
         <is>
           <t>Jump Trading Pacific Pte Ltd</t>
@@ -2292,36 +2284,42 @@
       <c r="BC9" t="inlineStr"/>
       <c r="BD9" t="inlineStr"/>
       <c r="BE9" t="inlineStr"/>
-      <c r="BF9" t="inlineStr"/>
+      <c r="BF9" t="n">
+        <v>97000</v>
+      </c>
       <c r="BG9" t="n">
-        <v>726440</v>
+        <v>650480</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
       <c r="BJ9" t="inlineStr"/>
       <c r="BK9" t="inlineStr"/>
       <c r="BL9" t="inlineStr"/>
-      <c r="BM9" t="inlineStr"/>
+      <c r="BM9" t="n">
+        <v>7132800</v>
+      </c>
       <c r="BN9" t="n">
-        <v>5316140</v>
+        <v>4071720</v>
       </c>
       <c r="BO9" t="n">
-        <v>726440</v>
+        <v>650480</v>
       </c>
       <c r="BP9" t="n">
-        <v>1050813620</v>
+        <v>958065200</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
       <c r="BS9" t="inlineStr"/>
       <c r="BT9" t="inlineStr"/>
       <c r="BU9" t="inlineStr"/>
-      <c r="BV9" t="inlineStr"/>
+      <c r="BV9" t="n">
+        <v>9710768600</v>
+      </c>
       <c r="BW9" t="n">
-        <v>8028731360</v>
+        <v>6341660460</v>
       </c>
       <c r="BX9" t="n">
-        <v>1050813620</v>
+        <v>958065200</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2329,17 +2327,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2379,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1136</v>
+        <v>1168</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2415,20 +2413,20 @@
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="n">
+      <c r="AL10" t="n">
         <v>135800</v>
       </c>
+      <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
       <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
-      <c r="AT10" t="inlineStr"/>
-      <c r="AU10" t="n">
-        <v>0</v>
-      </c>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="inlineStr"/>
       <c r="AV10" t="inlineStr">
         <is>
           <t>Morgan Stanley &amp; Co. International plc</t>
@@ -2447,9 +2445,11 @@
       <c r="BC10" t="inlineStr"/>
       <c r="BD10" t="inlineStr"/>
       <c r="BE10" t="inlineStr"/>
-      <c r="BF10" t="inlineStr"/>
+      <c r="BF10" t="n">
+        <v>0</v>
+      </c>
       <c r="BG10" t="n">
-        <v>211840</v>
+        <v>156960</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2458,13 +2458,13 @@
       <c r="BL10" t="inlineStr"/>
       <c r="BM10" t="inlineStr"/>
       <c r="BN10" t="n">
-        <v>1505100</v>
+        <v>917800</v>
       </c>
       <c r="BO10" t="n">
-        <v>211840</v>
+        <v>156960</v>
       </c>
       <c r="BP10" t="n">
-        <v>247418060</v>
+        <v>178777700</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2473,10 +2473,10 @@
       <c r="BU10" t="inlineStr"/>
       <c r="BV10" t="inlineStr"/>
       <c r="BW10" t="n">
-        <v>1988927000</v>
+        <v>1198242850</v>
       </c>
       <c r="BX10" t="n">
-        <v>247418060</v>
+        <v>178777700</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2484,17 +2484,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2570,20 +2570,20 @@
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
-      <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="n">
+      <c r="AL11" t="n">
         <v>3478500</v>
       </c>
+      <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="inlineStr"/>
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
-      <c r="AT11" t="inlineStr"/>
-      <c r="AU11" t="n">
+      <c r="AT11" t="n">
         <v>673100</v>
       </c>
+      <c r="AU11" t="inlineStr"/>
       <c r="AV11" t="inlineStr"/>
       <c r="AW11" t="inlineStr"/>
       <c r="AX11" t="inlineStr"/>
@@ -2596,7 +2596,7 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>24024360</v>
+        <v>21291380</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2605,13 +2605,13 @@
       <c r="BL11" t="inlineStr"/>
       <c r="BM11" t="inlineStr"/>
       <c r="BN11" t="n">
-        <v>10922450</v>
+        <v>15476400</v>
       </c>
       <c r="BO11" t="n">
-        <v>24024360</v>
+        <v>21291380</v>
       </c>
       <c r="BP11" t="n">
-        <v>11174434740</v>
+        <v>9604040680</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2620,10 +2620,10 @@
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="inlineStr"/>
       <c r="BW11" t="n">
-        <v>4758047550</v>
+        <v>7270849000</v>
       </c>
       <c r="BX11" t="n">
-        <v>11174434740</v>
+        <v>9604040680</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2631,17 +2631,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2683,7 +2683,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2717,20 +2717,20 @@
       <c r="AI12" t="inlineStr"/>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="n">
+      <c r="AL12" t="n">
         <v>126500</v>
       </c>
+      <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
       <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="inlineStr"/>
-      <c r="AU12" t="n">
+      <c r="AT12" t="n">
         <v>39200</v>
       </c>
+      <c r="AU12" t="inlineStr"/>
       <c r="AV12" t="inlineStr">
         <is>
           <t>GOLDMAN SACHS INTERNATIONAL</t>
@@ -2749,9 +2749,11 @@
       <c r="BC12" t="inlineStr"/>
       <c r="BD12" t="inlineStr"/>
       <c r="BE12" t="inlineStr"/>
-      <c r="BF12" t="inlineStr"/>
+      <c r="BF12" t="n">
+        <v>379285</v>
+      </c>
       <c r="BG12" t="n">
-        <v>201040</v>
+        <v>192000</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2760,13 +2762,13 @@
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="n">
-        <v>247150</v>
+        <v>245833.3333333333</v>
       </c>
       <c r="BO12" t="n">
-        <v>201040</v>
+        <v>192000</v>
       </c>
       <c r="BP12" t="n">
-        <v>83837520</v>
+        <v>79708300</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2775,10 +2777,10 @@
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="n">
-        <v>102748250</v>
+        <v>102468266.6666667</v>
       </c>
       <c r="BX12" t="n">
-        <v>83837520</v>
+        <v>79708300</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2786,17 +2788,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2840,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2872,20 +2874,20 @@
       <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="n">
+      <c r="AL13" t="n">
         <v>62800</v>
       </c>
+      <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="n">
+      <c r="AT13" t="n">
         <v>2200</v>
       </c>
+      <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr"/>
       <c r="AW13" t="inlineStr"/>
       <c r="AX13" t="inlineStr"/>
@@ -2898,7 +2900,7 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="n">
-        <v>150280</v>
+        <v>103320</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2907,13 +2909,13 @@
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="n">
-        <v>155450</v>
+        <v>198733.3333333333</v>
       </c>
       <c r="BO13" t="n">
-        <v>150280</v>
+        <v>103320</v>
       </c>
       <c r="BP13" t="n">
-        <v>140007220</v>
+        <v>96350860</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2922,10 +2924,10 @@
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="n">
-        <v>144927050</v>
+        <v>185306366.6666667</v>
       </c>
       <c r="BX13" t="n">
-        <v>140007220</v>
+        <v>96350860</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2933,17 +2935,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2987,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1863</v>
+        <v>1861</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -3019,30 +3021,30 @@
       <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="n">
+      <c r="AL14" t="n">
         <v>546000</v>
       </c>
+      <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr"/>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
-      <c r="AT14" t="inlineStr"/>
-      <c r="AU14" t="n">
+      <c r="AT14" t="n">
         <v>6700</v>
       </c>
+      <c r="AU14" t="inlineStr"/>
       <c r="AV14" t="inlineStr">
         <is>
           <t>GOLDMAN SACHS INTERNATIONAL</t>
         </is>
       </c>
       <c r="AW14" t="n">
-        <v>0.0054</v>
+        <v>0.0041</v>
       </c>
       <c r="AX14" t="n">
-        <v>194633</v>
+        <v>146386</v>
       </c>
       <c r="AY14" t="inlineStr"/>
       <c r="AZ14" t="inlineStr"/>
@@ -3050,12 +3052,14 @@
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
       <c r="BD14" t="inlineStr"/>
-      <c r="BE14" t="inlineStr"/>
+      <c r="BE14" t="n">
+        <v>194633</v>
+      </c>
       <c r="BF14" t="n">
-        <v>194633</v>
+        <v>146386</v>
       </c>
       <c r="BG14" t="n">
-        <v>184180</v>
+        <v>167780</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -3064,13 +3068,13 @@
       <c r="BL14" t="inlineStr"/>
       <c r="BM14" t="inlineStr"/>
       <c r="BN14" t="n">
-        <v>195250</v>
+        <v>206866.6666666667</v>
       </c>
       <c r="BO14" t="n">
-        <v>184180</v>
+        <v>167780</v>
       </c>
       <c r="BP14" t="n">
-        <v>343918960</v>
+        <v>314505480</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -3079,10 +3083,10 @@
       <c r="BU14" t="inlineStr"/>
       <c r="BV14" t="inlineStr"/>
       <c r="BW14" t="n">
-        <v>351530650</v>
+        <v>375613033.3333333</v>
       </c>
       <c r="BX14" t="n">
-        <v>343918960</v>
+        <v>314505480</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -3090,17 +3094,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3146,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>430</v>
+        <v>413</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -3176,20 +3180,20 @@
       <c r="AI15" t="inlineStr"/>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="inlineStr"/>
-      <c r="AM15" t="n">
+      <c r="AL15" t="n">
         <v>11624300</v>
       </c>
+      <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
       <c r="AP15" t="inlineStr"/>
       <c r="AQ15" t="inlineStr"/>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
-      <c r="AT15" t="inlineStr"/>
-      <c r="AU15" t="n">
+      <c r="AT15" t="n">
         <v>86900</v>
       </c>
+      <c r="AU15" t="inlineStr"/>
       <c r="AV15" t="inlineStr"/>
       <c r="AW15" t="inlineStr"/>
       <c r="AX15" t="inlineStr"/>
@@ -3202,7 +3206,7 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>1845660</v>
+        <v>2157100</v>
       </c>
       <c r="BH15" t="inlineStr"/>
       <c r="BI15" t="inlineStr"/>
@@ -3211,13 +3215,13 @@
       <c r="BL15" t="inlineStr"/>
       <c r="BM15" t="inlineStr"/>
       <c r="BN15" t="n">
-        <v>2210850</v>
+        <v>2252600</v>
       </c>
       <c r="BO15" t="n">
-        <v>1845660</v>
+        <v>2157100</v>
       </c>
       <c r="BP15" t="n">
-        <v>791971060</v>
+        <v>920704780</v>
       </c>
       <c r="BQ15" t="inlineStr"/>
       <c r="BR15" t="inlineStr"/>
@@ -3226,10 +3230,10 @@
       <c r="BU15" t="inlineStr"/>
       <c r="BV15" t="inlineStr"/>
       <c r="BW15" t="n">
-        <v>984957200</v>
+        <v>988981966.6666666</v>
       </c>
       <c r="BX15" t="n">
-        <v>791971060</v>
+        <v>920704780</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3237,17 +3241,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3293,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>1020</v>
+        <v>966</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3341,7 +3345,7 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>2872425</v>
+        <v>2510860</v>
       </c>
       <c r="BH16" t="inlineStr"/>
       <c r="BI16" t="inlineStr"/>
@@ -3351,10 +3355,10 @@
       <c r="BM16" t="inlineStr"/>
       <c r="BN16" t="inlineStr"/>
       <c r="BO16" t="n">
-        <v>2872425</v>
+        <v>2510860</v>
       </c>
       <c r="BP16" t="n">
-        <v>3084106450</v>
+        <v>2679272900</v>
       </c>
       <c r="BQ16" t="inlineStr"/>
       <c r="BR16" t="inlineStr"/>
@@ -3364,7 +3368,7 @@
       <c r="BV16" t="inlineStr"/>
       <c r="BW16" t="inlineStr"/>
       <c r="BX16" t="n">
-        <v>3084106450</v>
+        <v>2679272900</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3372,17 +3376,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3424,7 +3428,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>621</v>
+        <v>593</v>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -3482,9 +3486,11 @@
       <c r="BC17" t="inlineStr"/>
       <c r="BD17" t="inlineStr"/>
       <c r="BE17" t="inlineStr"/>
-      <c r="BF17" t="inlineStr"/>
+      <c r="BF17" t="n">
+        <v>525000</v>
+      </c>
       <c r="BG17" t="n">
-        <v>3251933.333333333</v>
+        <v>6937850</v>
       </c>
       <c r="BH17" t="inlineStr"/>
       <c r="BI17" t="inlineStr"/>
@@ -3494,10 +3500,10 @@
       <c r="BM17" t="inlineStr"/>
       <c r="BN17" t="inlineStr"/>
       <c r="BO17" t="n">
-        <v>3251933.333333333</v>
+        <v>6937850</v>
       </c>
       <c r="BP17" t="n">
-        <v>1553883300</v>
+        <v>3931852700</v>
       </c>
       <c r="BQ17" t="inlineStr"/>
       <c r="BR17" t="inlineStr"/>
@@ -3507,7 +3513,7 @@
       <c r="BV17" t="inlineStr"/>
       <c r="BW17" t="inlineStr"/>
       <c r="BX17" t="n">
-        <v>1553883300</v>
+        <v>3931852700</v>
       </c>
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
@@ -3515,17 +3521,17 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3573,7 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>2613</v>
+        <v>3115</v>
       </c>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
@@ -3619,7 +3625,7 @@
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="n">
-        <v>1185300</v>
+        <v>818800</v>
       </c>
       <c r="BH18" t="inlineStr"/>
       <c r="BI18" t="inlineStr"/>
@@ -3629,10 +3635,10 @@
       <c r="BM18" t="inlineStr"/>
       <c r="BN18" t="inlineStr"/>
       <c r="BO18" t="n">
-        <v>1185300</v>
+        <v>818800</v>
       </c>
       <c r="BP18" t="n">
-        <v>3532839500</v>
+        <v>2428380250</v>
       </c>
       <c r="BQ18" t="inlineStr"/>
       <c r="BR18" t="inlineStr"/>
@@ -3642,7 +3648,7 @@
       <c r="BV18" t="inlineStr"/>
       <c r="BW18" t="inlineStr"/>
       <c r="BX18" t="n">
-        <v>3532839500</v>
+        <v>2428380250</v>
       </c>
       <c r="BY18" t="inlineStr"/>
       <c r="BZ18" t="inlineStr"/>
@@ -3650,17 +3656,17 @@
       <c r="CB18" t="inlineStr"/>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD18" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3707,9 @@
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>25000</v>
+      </c>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -3752,10 +3760,10 @@
       <c r="BE19" t="inlineStr"/>
       <c r="BF19" t="inlineStr"/>
       <c r="BG19" t="n">
-        <v>150</v>
+        <v>133.3333333333333</v>
       </c>
       <c r="BH19" t="n">
-        <v>780</v>
+        <v>925</v>
       </c>
       <c r="BI19" t="n">
         <v>100</v>
@@ -3764,25 +3772,25 @@
         <v>450</v>
       </c>
       <c r="BK19" t="n">
-        <v>166.6666666666667</v>
+        <v>200</v>
       </c>
       <c r="BL19" t="n">
-        <v>325</v>
+        <v>300</v>
       </c>
       <c r="BM19" t="n">
-        <v>233.3333333333333</v>
+        <v>250</v>
       </c>
       <c r="BN19" t="n">
         <v>300</v>
       </c>
       <c r="BO19" t="n">
-        <v>150</v>
+        <v>133.3333333333333</v>
       </c>
       <c r="BP19" t="n">
-        <v>3750500</v>
+        <v>3333666.666666667</v>
       </c>
       <c r="BQ19" t="n">
-        <v>21083400</v>
+        <v>25063500</v>
       </c>
       <c r="BR19" t="n">
         <v>2645000</v>
@@ -3791,19 +3799,19 @@
         <v>11285000</v>
       </c>
       <c r="BT19" t="n">
-        <v>4161000</v>
+        <v>4993250</v>
       </c>
       <c r="BU19" t="n">
-        <v>8085750</v>
+        <v>7443250</v>
       </c>
       <c r="BV19" t="n">
-        <v>5813333.333333333</v>
+        <v>6260000</v>
       </c>
       <c r="BW19" t="n">
         <v>7372000</v>
       </c>
       <c r="BX19" t="n">
-        <v>3750500</v>
+        <v>3333666.666666667</v>
       </c>
       <c r="BY19" t="inlineStr"/>
       <c r="BZ19" t="inlineStr"/>
@@ -3811,17 +3819,17 @@
       <c r="CB19" t="inlineStr"/>
       <c r="CC19" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD19" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE19" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3871,7 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -3892,29 +3900,27 @@
         <v>122230</v>
       </c>
       <c r="AF20" t="n">
-        <v>202741</v>
+        <v>204885</v>
       </c>
       <c r="AG20" t="n">
-        <v>204885</v>
+        <v>97185</v>
       </c>
       <c r="AH20" t="n">
-        <v>97185</v>
+        <v>93675</v>
       </c>
       <c r="AI20" t="n">
-        <v>93675</v>
+        <v>126528</v>
       </c>
       <c r="AJ20" t="n">
-        <v>126528</v>
+        <v>99264</v>
       </c>
       <c r="AK20" t="n">
-        <v>99264</v>
+        <v>96080</v>
       </c>
       <c r="AL20" t="n">
-        <v>96080</v>
-      </c>
-      <c r="AM20" t="n">
         <v>122230</v>
       </c>
+      <c r="AM20" t="inlineStr"/>
       <c r="AN20" t="n">
         <v>0</v>
       </c>
@@ -3936,9 +3942,7 @@
       <c r="AT20" t="n">
         <v>0</v>
       </c>
-      <c r="AU20" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU20" t="inlineStr"/>
       <c r="AV20" t="inlineStr"/>
       <c r="AW20" t="inlineStr"/>
       <c r="AX20" t="inlineStr"/>
@@ -3951,58 +3955,58 @@
       <c r="BE20" t="inlineStr"/>
       <c r="BF20" t="inlineStr"/>
       <c r="BG20" t="n">
-        <v>1690468.6</v>
+        <v>3083292.6</v>
       </c>
       <c r="BH20" t="n">
-        <v>11028008.4</v>
+        <v>12912269</v>
       </c>
       <c r="BI20" t="n">
-        <v>9570452.800000001</v>
+        <v>7299611.6</v>
       </c>
       <c r="BJ20" t="n">
-        <v>3267717.4</v>
+        <v>2742294</v>
       </c>
       <c r="BK20" t="n">
-        <v>3674551.2</v>
+        <v>3912781</v>
       </c>
       <c r="BL20" t="n">
-        <v>4241035.4</v>
+        <v>4714386.8</v>
       </c>
       <c r="BM20" t="n">
-        <v>3010975.8</v>
+        <v>2238110.2</v>
       </c>
       <c r="BN20" t="n">
-        <v>1764609.6</v>
+        <v>1913806.6</v>
       </c>
       <c r="BO20" t="n">
-        <v>1690468.6</v>
+        <v>3083292.6</v>
       </c>
       <c r="BP20" t="n">
-        <v>45282081.2</v>
+        <v>88928311</v>
       </c>
       <c r="BQ20" t="n">
-        <v>272405338.6</v>
+        <v>314646947.2</v>
       </c>
       <c r="BR20" t="n">
-        <v>292344615.4</v>
+        <v>226772440</v>
       </c>
       <c r="BS20" t="n">
-        <v>83737882</v>
+        <v>69693452.8</v>
       </c>
       <c r="BT20" t="n">
-        <v>107086813.6</v>
+        <v>114743178.6</v>
       </c>
       <c r="BU20" t="n">
-        <v>131265781.6</v>
+        <v>148128099</v>
       </c>
       <c r="BV20" t="n">
-        <v>92793402.59999999</v>
+        <v>67164683.59999999</v>
       </c>
       <c r="BW20" t="n">
-        <v>48812478.4</v>
+        <v>52170691.2</v>
       </c>
       <c r="BX20" t="n">
-        <v>45282081.2</v>
+        <v>88928311</v>
       </c>
       <c r="BY20" t="inlineStr"/>
       <c r="BZ20" t="inlineStr"/>
@@ -4010,17 +4014,17 @@
       <c r="CB20" t="inlineStr"/>
       <c r="CC20" t="inlineStr">
         <is>
-          <t>20260409-211147</t>
+          <t>20260410-190048</t>
         </is>
       </c>
       <c r="CD20" t="inlineStr">
         <is>
-          <t>2026-04-09T12:11:47+00:00</t>
+          <t>2026-04-10T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE20" t="inlineStr">
         <is>
-          <t>2026-04-09T21:11:47+09:00</t>
+          <t>2026-04-10T19:00:48+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-11
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -1026,17 +1026,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1245,17 +1245,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1440,17 +1440,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1649,17 +1649,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1852,17 +1852,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2007,17 +2007,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2162,17 +2162,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2327,17 +2327,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2484,17 +2484,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2631,17 +2631,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2788,17 +2788,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2935,17 +2935,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3094,17 +3094,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3241,17 +3241,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3376,17 +3376,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3521,17 +3521,17 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3656,17 +3656,17 @@
       <c r="CB18" t="inlineStr"/>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD18" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3819,17 +3819,17 @@
       <c r="CB19" t="inlineStr"/>
       <c r="CC19" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD19" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE19" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -4014,17 +4014,17 @@
       <c r="CB20" t="inlineStr"/>
       <c r="CC20" t="inlineStr">
         <is>
-          <t>20260410-210616</t>
+          <t>20260411-190049</t>
         </is>
       </c>
       <c r="CD20" t="inlineStr">
         <is>
-          <t>2026-04-10T12:06:16+00:00</t>
+          <t>2026-04-11T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE20" t="inlineStr">
         <is>
-          <t>2026-04-10T21:06:16+09:00</t>
+          <t>2026-04-11T19:00:49+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-12
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -1026,17 +1026,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1245,17 +1245,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1440,17 +1440,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1649,17 +1649,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -1852,17 +1852,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2007,17 +2007,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2162,17 +2162,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2327,17 +2327,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2484,17 +2484,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2631,17 +2631,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2788,17 +2788,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -2935,17 +2935,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3094,17 +3094,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3241,17 +3241,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3376,17 +3376,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3521,17 +3521,17 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3656,17 +3656,17 @@
       <c r="CB18" t="inlineStr"/>
       <c r="CC18" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD18" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE18" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -3819,17 +3819,17 @@
       <c r="CB19" t="inlineStr"/>
       <c r="CC19" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD19" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE19" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>
@@ -4014,17 +4014,17 @@
       <c r="CB20" t="inlineStr"/>
       <c r="CC20" t="inlineStr">
         <is>
-          <t>20260411-190049</t>
+          <t>20260412-190048</t>
         </is>
       </c>
       <c r="CD20" t="inlineStr">
         <is>
-          <t>2026-04-11T10:00:49+00:00</t>
+          <t>2026-04-12T10:00:48+00:00</t>
         </is>
       </c>
       <c r="CE20" t="inlineStr">
         <is>
-          <t>2026-04-11T19:00:49+09:00</t>
+          <t>2026-04-12T19:00:48+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-13
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE20"/>
+  <dimension ref="A1:CE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -967,58 +967,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>19600</v>
+        <v>16200</v>
       </c>
       <c r="BH2" t="n">
-        <v>8600</v>
+        <v>10400</v>
       </c>
       <c r="BI2" t="n">
-        <v>13400</v>
+        <v>15400</v>
       </c>
       <c r="BJ2" t="n">
-        <v>14800</v>
+        <v>11000</v>
       </c>
       <c r="BK2" t="n">
-        <v>22800</v>
+        <v>25800</v>
       </c>
       <c r="BL2" t="n">
-        <v>14000</v>
+        <v>15800</v>
       </c>
       <c r="BM2" t="n">
-        <v>13800</v>
+        <v>14200</v>
       </c>
       <c r="BN2" t="n">
-        <v>27200</v>
+        <v>25400</v>
       </c>
       <c r="BO2" t="n">
-        <v>19600</v>
+        <v>16200</v>
       </c>
       <c r="BP2" t="n">
-        <v>1452600</v>
+        <v>1214600</v>
       </c>
       <c r="BQ2" t="n">
-        <v>677000</v>
+        <v>831600</v>
       </c>
       <c r="BR2" t="n">
-        <v>1074800</v>
+        <v>1212800</v>
       </c>
       <c r="BS2" t="n">
-        <v>1151800</v>
+        <v>852400</v>
       </c>
       <c r="BT2" t="n">
-        <v>1615200</v>
+        <v>1810200</v>
       </c>
       <c r="BU2" t="n">
-        <v>981400</v>
+        <v>1101600</v>
       </c>
       <c r="BV2" t="n">
-        <v>947600</v>
+        <v>955400</v>
       </c>
       <c r="BW2" t="n">
-        <v>1862000</v>
+        <v>1778000</v>
       </c>
       <c r="BX2" t="n">
-        <v>1452600</v>
+        <v>1214600</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1026,44 +1026,44 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>464A</t>
+          <t>4875</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ＱＰＳホールディングス</t>
+          <t>メディシノバ・インク</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>グロース</t>
+          <t>スタンダード</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>医薬品</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>医薬品</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>2832</v>
+        <v>233</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1101,143 +1101,119 @@
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="n">
-        <v>236100</v>
+        <v>0</v>
       </c>
       <c r="AE3" t="n">
-        <v>3149100</v>
+        <v>76800</v>
       </c>
       <c r="AF3" t="n">
-        <v>3398500</v>
+        <v>57400</v>
       </c>
       <c r="AG3" t="n">
-        <v>3082900</v>
+        <v>57100</v>
       </c>
       <c r="AH3" t="n">
-        <v>3002100</v>
+        <v>57700</v>
       </c>
       <c r="AI3" t="n">
-        <v>2859200</v>
+        <v>78800</v>
       </c>
       <c r="AJ3" t="n">
-        <v>2911500</v>
+        <v>80100</v>
       </c>
       <c r="AK3" t="n">
-        <v>3235400</v>
+        <v>76600</v>
       </c>
       <c r="AL3" t="n">
-        <v>3149100</v>
+        <v>76800</v>
       </c>
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="n">
-        <v>619800</v>
+        <v>0</v>
       </c>
       <c r="AO3" t="n">
-        <v>650000</v>
+        <v>0</v>
       </c>
       <c r="AP3" t="n">
-        <v>269900</v>
+        <v>0</v>
       </c>
       <c r="AQ3" t="n">
-        <v>275900</v>
+        <v>0</v>
       </c>
       <c r="AR3" t="n">
-        <v>283300</v>
+        <v>0</v>
       </c>
       <c r="AS3" t="n">
-        <v>227300</v>
+        <v>0</v>
       </c>
       <c r="AT3" t="n">
-        <v>236100</v>
+        <v>0</v>
       </c>
       <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr">
-        <is>
-          <t>モルガン・スタンレーMUFG証券株式会社、Nomura International plc</t>
-        </is>
-      </c>
-      <c r="AW3" t="n">
-        <v>0.0046</v>
-      </c>
-      <c r="AX3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="AY3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="AZ3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="BA3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="BB3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="BC3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="BD3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>362132</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>362132</v>
-      </c>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="n">
-        <v>3191940</v>
+        <v>36680</v>
       </c>
       <c r="BH3" t="n">
-        <v>1374680</v>
+        <v>75940</v>
       </c>
       <c r="BI3" t="n">
-        <v>1707980</v>
+        <v>63460</v>
       </c>
       <c r="BJ3" t="n">
-        <v>2332920</v>
+        <v>68420</v>
       </c>
       <c r="BK3" t="n">
-        <v>1349720</v>
+        <v>58460</v>
       </c>
       <c r="BL3" t="n">
-        <v>3208240</v>
+        <v>101700</v>
       </c>
       <c r="BM3" t="n">
-        <v>2079840</v>
+        <v>40220</v>
       </c>
       <c r="BN3" t="n">
-        <v>2432780</v>
+        <v>16280</v>
       </c>
       <c r="BO3" t="n">
-        <v>3191940</v>
+        <v>36680</v>
       </c>
       <c r="BP3" t="n">
-        <v>8388170740</v>
+        <v>8475240</v>
       </c>
       <c r="BQ3" t="n">
-        <v>2781072700</v>
+        <v>19566000</v>
       </c>
       <c r="BR3" t="n">
-        <v>3574143180</v>
+        <v>15580660</v>
       </c>
       <c r="BS3" t="n">
-        <v>5081670080</v>
+        <v>15720080</v>
       </c>
       <c r="BT3" t="n">
-        <v>2747044860</v>
+        <v>13031980</v>
       </c>
       <c r="BU3" t="n">
-        <v>7781799320</v>
+        <v>23672580</v>
       </c>
       <c r="BV3" t="n">
-        <v>4889458760</v>
+        <v>9151220</v>
       </c>
       <c r="BW3" t="n">
-        <v>5462913800</v>
+        <v>3639380</v>
       </c>
       <c r="BX3" t="n">
-        <v>8388170740</v>
+        <v>8475240</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1245,34 +1221,34 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4875</t>
+          <t>504A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>メディシノバ・インク</t>
+          <t>イノバセル</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>スタンダード</t>
+          <t>グロース</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1297,7 +1273,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>230</v>
+        <v>750</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1323,33 +1299,29 @@
         <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>76800</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>57400</v>
-      </c>
+        <v>234400</v>
+      </c>
+      <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
-        <v>57100</v>
+        <v>222300</v>
       </c>
       <c r="AH4" t="n">
-        <v>57700</v>
+        <v>216400</v>
       </c>
       <c r="AI4" t="n">
-        <v>78800</v>
+        <v>204600</v>
       </c>
       <c r="AJ4" t="n">
-        <v>80100</v>
+        <v>212600</v>
       </c>
       <c r="AK4" t="n">
-        <v>76600</v>
+        <v>227900</v>
       </c>
       <c r="AL4" t="n">
-        <v>76800</v>
+        <v>234400</v>
       </c>
       <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="n">
-        <v>0</v>
-      </c>
+      <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="n">
         <v>0</v>
       </c>
@@ -1363,76 +1335,94 @@
         <v>0</v>
       </c>
       <c r="AS4" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="AT4" t="n">
         <v>0</v>
       </c>
       <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>野村證券株式会社</t>
+        </is>
+      </c>
+      <c r="AW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>0</v>
+      </c>
       <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
-      <c r="BB4" t="inlineStr"/>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
+      <c r="AZ4" t="n">
+        <v>2482900</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>1080200</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>1080200</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>1041600</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0</v>
+      </c>
       <c r="BG4" t="n">
-        <v>18480</v>
-      </c>
-      <c r="BH4" t="n">
-        <v>79860</v>
-      </c>
+        <v>86180</v>
+      </c>
+      <c r="BH4" t="inlineStr"/>
       <c r="BI4" t="n">
-        <v>59380</v>
+        <v>1096975</v>
       </c>
       <c r="BJ4" t="n">
-        <v>68320</v>
+        <v>229200</v>
       </c>
       <c r="BK4" t="n">
-        <v>58860</v>
+        <v>104900</v>
       </c>
       <c r="BL4" t="n">
-        <v>79320</v>
+        <v>127240</v>
       </c>
       <c r="BM4" t="n">
-        <v>63700</v>
+        <v>82900</v>
       </c>
       <c r="BN4" t="n">
-        <v>26220</v>
+        <v>61860</v>
       </c>
       <c r="BO4" t="n">
-        <v>18480</v>
+        <v>86180</v>
       </c>
       <c r="BP4" t="n">
-        <v>4174480</v>
-      </c>
-      <c r="BQ4" t="n">
-        <v>20766940</v>
-      </c>
+        <v>67974940</v>
+      </c>
+      <c r="BQ4" t="inlineStr"/>
       <c r="BR4" t="n">
-        <v>14569660</v>
+        <v>1152932450</v>
       </c>
       <c r="BS4" t="n">
-        <v>15978460</v>
+        <v>238575980</v>
       </c>
       <c r="BT4" t="n">
-        <v>13221880</v>
+        <v>108578560</v>
       </c>
       <c r="BU4" t="n">
-        <v>18258940</v>
+        <v>123609800</v>
       </c>
       <c r="BV4" t="n">
-        <v>14797380</v>
+        <v>70208720</v>
       </c>
       <c r="BW4" t="n">
-        <v>5820080</v>
+        <v>50250980</v>
       </c>
       <c r="BX4" t="n">
-        <v>4174480</v>
+        <v>67974940</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1440,29 +1430,29 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>504A</t>
+          <t>519A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>イノバセル</t>
+          <t>ベーシック</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1472,12 +1462,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>医薬品</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>医薬品</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1492,7 +1482,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>743</v>
+        <v>692</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1518,130 +1508,76 @@
         <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>234400</v>
+        <v>56200</v>
       </c>
       <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="n">
-        <v>222300</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>216400</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>204600</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>212600</v>
-      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="n">
-        <v>227900</v>
+        <v>49900</v>
       </c>
       <c r="AL5" t="n">
-        <v>234400</v>
+        <v>56200</v>
       </c>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="n">
-        <v>0</v>
-      </c>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="AT5" t="n">
         <v>0</v>
       </c>
       <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t>野村證券株式会社</t>
-        </is>
-      </c>
-      <c r="AW5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX5" t="n">
-        <v>0</v>
-      </c>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
       <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="n">
-        <v>2482900</v>
-      </c>
-      <c r="BA5" t="n">
-        <v>1080200</v>
-      </c>
-      <c r="BB5" t="n">
-        <v>1080200</v>
-      </c>
-      <c r="BC5" t="n">
-        <v>1041600</v>
-      </c>
-      <c r="BD5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF5" t="n">
-        <v>0</v>
-      </c>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="n">
-        <v>76980</v>
+        <v>18880</v>
       </c>
       <c r="BH5" t="inlineStr"/>
-      <c r="BI5" t="n">
-        <v>1302366.666666667</v>
-      </c>
-      <c r="BJ5" t="n">
-        <v>300260</v>
-      </c>
-      <c r="BK5" t="n">
-        <v>111260</v>
-      </c>
-      <c r="BL5" t="n">
-        <v>117620</v>
-      </c>
+      <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
       <c r="BM5" t="n">
-        <v>86180</v>
+        <v>318525</v>
       </c>
       <c r="BN5" t="n">
-        <v>82320</v>
+        <v>30900</v>
       </c>
       <c r="BO5" t="n">
-        <v>76980</v>
+        <v>18880</v>
       </c>
       <c r="BP5" t="n">
-        <v>61452380</v>
+        <v>12917580</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
-      <c r="BR5" t="n">
-        <v>1383993266.666667</v>
-      </c>
-      <c r="BS5" t="n">
-        <v>305469720</v>
-      </c>
-      <c r="BT5" t="n">
-        <v>113793920</v>
-      </c>
-      <c r="BU5" t="n">
-        <v>118662180</v>
-      </c>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
       <c r="BV5" t="n">
-        <v>74449720</v>
+        <v>247000550</v>
       </c>
       <c r="BW5" t="n">
-        <v>67033160</v>
+        <v>21013720</v>
       </c>
       <c r="BX5" t="n">
-        <v>61452380</v>
+        <v>12917580</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1649,44 +1585,44 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>505A</t>
+          <t>520A</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ギークリー</t>
+          <t>ジェイファーマ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>スタンダード</t>
+          <t>グロース</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>医薬品</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>サービス業</t>
+          <t>医薬品</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1701,7 +1637,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>1279</v>
+        <v>668</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1727,124 +1663,76 @@
         <v>0</v>
       </c>
       <c r="AE6" t="n">
-        <v>183000</v>
+        <v>106000</v>
       </c>
       <c r="AF6" t="inlineStr"/>
-      <c r="AG6" t="n">
-        <v>101900</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>201600</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>200600</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>183800</v>
-      </c>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="n">
-        <v>200400</v>
+        <v>70700</v>
       </c>
       <c r="AL6" t="n">
-        <v>183000</v>
+        <v>106000</v>
       </c>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>0</v>
-      </c>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AT6" t="n">
         <v>0</v>
       </c>
       <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr">
-        <is>
-          <t>野村證券株式会社</t>
-        </is>
-      </c>
-      <c r="AW6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX6" t="n">
-        <v>0</v>
-      </c>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
       <c r="AY6" t="inlineStr"/>
       <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="n">
-        <v>160600</v>
-      </c>
-      <c r="BB6" t="n">
-        <v>151600</v>
-      </c>
-      <c r="BC6" t="n">
-        <v>127100</v>
-      </c>
-      <c r="BD6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF6" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="n">
-        <v>46940</v>
+        <v>40500</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
-      <c r="BJ6" t="n">
-        <v>387740</v>
-      </c>
-      <c r="BK6" t="n">
-        <v>57680</v>
-      </c>
-      <c r="BL6" t="n">
-        <v>51540</v>
-      </c>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
       <c r="BM6" t="n">
-        <v>40660</v>
+        <v>540325</v>
       </c>
       <c r="BN6" t="n">
-        <v>32720</v>
+        <v>140100</v>
       </c>
       <c r="BO6" t="n">
-        <v>46940</v>
+        <v>40500</v>
       </c>
       <c r="BP6" t="n">
-        <v>60955240</v>
+        <v>27184060</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
-      <c r="BS6" t="n">
-        <v>626504680</v>
-      </c>
-      <c r="BT6" t="n">
-        <v>81473640</v>
-      </c>
-      <c r="BU6" t="n">
-        <v>69089120</v>
-      </c>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
       <c r="BV6" t="n">
-        <v>50832820</v>
+        <v>389225050</v>
       </c>
       <c r="BW6" t="n">
-        <v>41588180</v>
+        <v>98474520</v>
       </c>
       <c r="BX6" t="n">
-        <v>60955240</v>
+        <v>27184060</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1852,29 +1740,29 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>519A</t>
+          <t>523A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ベーシック</t>
+          <t>セイワホールディングス</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1884,12 +1772,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>建設・資材</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>金属製品</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1904,7 +1792,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>682</v>
+        <v>1497</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1930,7 +1818,7 @@
         <v>0</v>
       </c>
       <c r="AE7" t="n">
-        <v>56200</v>
+        <v>634100</v>
       </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
@@ -1938,10 +1826,10 @@
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="n">
-        <v>49900</v>
+        <v>408200</v>
       </c>
       <c r="AL7" t="n">
-        <v>56200</v>
+        <v>634100</v>
       </c>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
@@ -1956,9 +1844,17 @@
         <v>0</v>
       </c>
       <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>Jump Trading Pacific Pte Ltd</t>
+        </is>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.0051</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>97000</v>
+      </c>
       <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="inlineStr"/>
@@ -1966,9 +1862,11 @@
       <c r="BC7" t="inlineStr"/>
       <c r="BD7" t="inlineStr"/>
       <c r="BE7" t="inlineStr"/>
-      <c r="BF7" t="inlineStr"/>
+      <c r="BF7" t="n">
+        <v>97000</v>
+      </c>
       <c r="BG7" t="n">
-        <v>20400</v>
+        <v>579780</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1976,16 +1874,16 @@
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="n">
-        <v>406400</v>
+        <v>7535550</v>
       </c>
       <c r="BN7" t="n">
-        <v>38440</v>
+        <v>2620900</v>
       </c>
       <c r="BO7" t="n">
-        <v>20400</v>
+        <v>579780</v>
       </c>
       <c r="BP7" t="n">
-        <v>13911860</v>
+        <v>866355580</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
@@ -1993,13 +1891,13 @@
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="n">
-        <v>316942333.3333333</v>
+        <v>11342836750</v>
       </c>
       <c r="BW7" t="n">
-        <v>26133940</v>
+        <v>3937584140</v>
       </c>
       <c r="BX7" t="n">
-        <v>13911860</v>
+        <v>866355580</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -2007,44 +1905,44 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>520A</t>
+          <t>543A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ジェイファーマ</t>
+          <t>ＡＲＣＨＩＯＮ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>グロース</t>
+          <t>プライム</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>医薬品</t>
+          <t>自動車・輸送機</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>医薬品</t>
+          <t>輸送用機器</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2059,7 +1957,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>664</v>
+        <v>428</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2082,21 +1980,19 @@
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>673100</v>
       </c>
       <c r="AE8" t="n">
-        <v>106000</v>
+        <v>3478500</v>
       </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="n">
-        <v>70700</v>
-      </c>
+      <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="n">
-        <v>106000</v>
+        <v>3478500</v>
       </c>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
@@ -2104,11 +2000,9 @@
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="n">
-        <v>1000</v>
-      </c>
+      <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="n">
-        <v>0</v>
+        <v>673100</v>
       </c>
       <c r="AU8" t="inlineStr"/>
       <c r="AV8" t="inlineStr"/>
@@ -2123,38 +2017,34 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="n">
-        <v>54260</v>
+        <v>14445560</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
       <c r="BJ8" t="inlineStr"/>
       <c r="BK8" t="inlineStr"/>
       <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="n">
-        <v>608533.3333333334</v>
-      </c>
+      <c r="BM8" t="inlineStr"/>
       <c r="BN8" t="n">
-        <v>187780</v>
+        <v>22304225</v>
       </c>
       <c r="BO8" t="n">
-        <v>54260</v>
+        <v>14445560</v>
       </c>
       <c r="BP8" t="n">
-        <v>36525580</v>
+        <v>6156474700</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
       <c r="BS8" t="inlineStr"/>
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
-      <c r="BV8" t="n">
-        <v>445297133.3333333</v>
-      </c>
+      <c r="BV8" t="inlineStr"/>
       <c r="BW8" t="n">
-        <v>129544760</v>
+        <v>10645521900</v>
       </c>
       <c r="BX8" t="n">
-        <v>36525580</v>
+        <v>6156474700</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2162,44 +2052,44 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>523A</t>
+          <t>544A</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>セイワホールディングス</t>
+          <t>ＧＭＳグループ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>グロース</t>
+          <t>プライム</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>建設・資材</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>金属製品</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2214,7 +2104,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>1502</v>
+        <v>410</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2237,21 +2127,19 @@
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
-        <v>0</v>
+        <v>39200</v>
       </c>
       <c r="AE9" t="n">
-        <v>634100</v>
+        <v>126500</v>
       </c>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="n">
-        <v>408200</v>
-      </c>
+      <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="n">
-        <v>634100</v>
+        <v>126500</v>
       </c>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
@@ -2259,23 +2147,21 @@
       <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="n">
-        <v>0</v>
-      </c>
+      <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>39200</v>
       </c>
       <c r="AU9" t="inlineStr"/>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>Jump Trading Pacific Pte Ltd</t>
+          <t>GOLDMAN SACHS INTERNATIONAL</t>
         </is>
       </c>
       <c r="AW9" t="n">
-        <v>0.0051</v>
+        <v>0.0053</v>
       </c>
       <c r="AX9" t="n">
-        <v>97000</v>
+        <v>379285</v>
       </c>
       <c r="AY9" t="inlineStr"/>
       <c r="AZ9" t="inlineStr"/>
@@ -2285,41 +2171,37 @@
       <c r="BD9" t="inlineStr"/>
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="n">
-        <v>97000</v>
+        <v>379285</v>
       </c>
       <c r="BG9" t="n">
-        <v>650480</v>
+        <v>173700</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
       <c r="BJ9" t="inlineStr"/>
       <c r="BK9" t="inlineStr"/>
       <c r="BL9" t="inlineStr"/>
-      <c r="BM9" t="n">
-        <v>7132800</v>
-      </c>
+      <c r="BM9" t="inlineStr"/>
       <c r="BN9" t="n">
-        <v>4071720</v>
+        <v>248475</v>
       </c>
       <c r="BO9" t="n">
-        <v>650480</v>
+        <v>173700</v>
       </c>
       <c r="BP9" t="n">
-        <v>958065200</v>
+        <v>72047820</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
       <c r="BS9" t="inlineStr"/>
       <c r="BT9" t="inlineStr"/>
       <c r="BU9" t="inlineStr"/>
-      <c r="BV9" t="n">
-        <v>9710768600</v>
-      </c>
+      <c r="BV9" t="inlineStr"/>
       <c r="BW9" t="n">
-        <v>6341660460</v>
+        <v>103489250</v>
       </c>
       <c r="BX9" t="n">
-        <v>958065200</v>
+        <v>72047820</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2327,44 +2209,44 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>542A</t>
+          <t>545A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ビタブリッドジャパン</t>
+          <t>トランヴィア</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>グロース</t>
+          <t>プライム</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>素材・化学</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>化学</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2379,7 +2261,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1168</v>
+        <v>940</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2402,10 +2284,10 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="AE10" t="n">
-        <v>135800</v>
+        <v>62800</v>
       </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
@@ -2414,7 +2296,7 @@
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="n">
-        <v>135800</v>
+        <v>62800</v>
       </c>
       <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
@@ -2424,20 +2306,12 @@
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="n">
-        <v>0</v>
+        <v>2200</v>
       </c>
       <c r="AU10" t="inlineStr"/>
-      <c r="AV10" t="inlineStr">
-        <is>
-          <t>Morgan Stanley &amp; Co. International plc</t>
-        </is>
-      </c>
-      <c r="AW10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX10" t="n">
-        <v>0</v>
-      </c>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
       <c r="AY10" t="inlineStr"/>
       <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="inlineStr"/>
@@ -2445,11 +2319,9 @@
       <c r="BC10" t="inlineStr"/>
       <c r="BD10" t="inlineStr"/>
       <c r="BE10" t="inlineStr"/>
-      <c r="BF10" t="n">
-        <v>0</v>
-      </c>
+      <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="n">
-        <v>156960</v>
+        <v>98700</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2458,13 +2330,13 @@
       <c r="BL10" t="inlineStr"/>
       <c r="BM10" t="inlineStr"/>
       <c r="BN10" t="n">
-        <v>917800</v>
+        <v>171850</v>
       </c>
       <c r="BO10" t="n">
-        <v>156960</v>
+        <v>98700</v>
       </c>
       <c r="BP10" t="n">
-        <v>178777700</v>
+        <v>92168220</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2473,10 +2345,10 @@
       <c r="BU10" t="inlineStr"/>
       <c r="BV10" t="inlineStr"/>
       <c r="BW10" t="n">
-        <v>1198242850</v>
+        <v>160315700</v>
       </c>
       <c r="BX10" t="n">
-        <v>178777700</v>
+        <v>92168220</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2484,29 +2356,29 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>543A</t>
+          <t>546A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ＡＲＣＨＩＯＮ</t>
+          <t>ＭＩＲＡＩＮＩホールディングス</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2516,12 +2388,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>自動車・輸送機</t>
+          <t>商社・卸売</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>輸送用機器</t>
+          <t>卸売業</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2536,7 +2408,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>398</v>
+        <v>1883</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2559,10 +2431,10 @@
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="n">
-        <v>673100</v>
+        <v>6700</v>
       </c>
       <c r="AE11" t="n">
-        <v>3478500</v>
+        <v>546000</v>
       </c>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
@@ -2571,7 +2443,7 @@
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="n">
-        <v>3478500</v>
+        <v>546000</v>
       </c>
       <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
@@ -2581,22 +2453,34 @@
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="n">
-        <v>673100</v>
+        <v>6700</v>
       </c>
       <c r="AU11" t="inlineStr"/>
-      <c r="AV11" t="inlineStr"/>
-      <c r="AW11" t="inlineStr"/>
-      <c r="AX11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>GOLDMAN SACHS INTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="AW11" t="n">
+        <v>0.0041</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>146386</v>
+      </c>
       <c r="AY11" t="inlineStr"/>
       <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="inlineStr"/>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
       <c r="BD11" t="inlineStr"/>
-      <c r="BE11" t="inlineStr"/>
-      <c r="BF11" t="inlineStr"/>
+      <c r="BE11" t="n">
+        <v>194633</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>146386</v>
+      </c>
       <c r="BG11" t="n">
-        <v>21291380</v>
+        <v>152960</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2605,13 +2489,13 @@
       <c r="BL11" t="inlineStr"/>
       <c r="BM11" t="inlineStr"/>
       <c r="BN11" t="n">
-        <v>15476400</v>
+        <v>201300</v>
       </c>
       <c r="BO11" t="n">
-        <v>21291380</v>
+        <v>152960</v>
       </c>
       <c r="BP11" t="n">
-        <v>9604040680</v>
+        <v>287691620</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2620,10 +2504,10 @@
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="inlineStr"/>
       <c r="BW11" t="n">
-        <v>7270849000</v>
+        <v>366972875</v>
       </c>
       <c r="BX11" t="n">
-        <v>9604040680</v>
+        <v>287691620</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2631,29 +2515,29 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>544A</t>
+          <t>547A</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ＧＭＳグループ</t>
+          <t>ムニノバホールディングス</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2663,12 +2547,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>機械</t>
+          <t>金融（除く銀行）</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>機械</t>
+          <t>その他金融業</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2683,7 +2567,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2706,10 +2590,10 @@
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="n">
-        <v>39200</v>
+        <v>86900</v>
       </c>
       <c r="AE12" t="n">
-        <v>126500</v>
+        <v>11624300</v>
       </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
@@ -2718,7 +2602,7 @@
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="n">
-        <v>126500</v>
+        <v>11624300</v>
       </c>
       <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
@@ -2728,20 +2612,12 @@
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="n">
-        <v>39200</v>
+        <v>86900</v>
       </c>
       <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr">
-        <is>
-          <t>GOLDMAN SACHS INTERNATIONAL</t>
-        </is>
-      </c>
-      <c r="AW12" t="n">
-        <v>0.0053</v>
-      </c>
-      <c r="AX12" t="n">
-        <v>379285</v>
-      </c>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
       <c r="BA12" t="inlineStr"/>
@@ -2749,11 +2625,9 @@
       <c r="BC12" t="inlineStr"/>
       <c r="BD12" t="inlineStr"/>
       <c r="BE12" t="inlineStr"/>
-      <c r="BF12" t="n">
-        <v>379285</v>
-      </c>
+      <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>192000</v>
+        <v>2212760</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2762,13 +2636,13 @@
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="n">
-        <v>245833.3333333333</v>
+        <v>2140650</v>
       </c>
       <c r="BO12" t="n">
-        <v>192000</v>
+        <v>2212760</v>
       </c>
       <c r="BP12" t="n">
-        <v>79708300</v>
+        <v>938631960</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2777,10 +2651,10 @@
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="n">
-        <v>102468266.6666667</v>
+        <v>932730175</v>
       </c>
       <c r="BX12" t="n">
-        <v>79708300</v>
+        <v>938631960</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2788,34 +2662,34 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>545A</t>
+          <t>548A</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>トランヴィア</t>
+          <t>システムエグゼ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>プライム</t>
+          <t>スタンダード</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2840,7 +2714,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>948</v>
+        <v>966</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2862,21 +2736,15 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="n">
-        <v>2200</v>
-      </c>
-      <c r="AE13" t="n">
-        <v>62800</v>
-      </c>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="n">
-        <v>62800</v>
-      </c>
+      <c r="AL13" t="inlineStr"/>
       <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
@@ -2884,13 +2752,19 @@
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="n">
-        <v>2200</v>
-      </c>
+      <c r="AT13" t="inlineStr"/>
       <c r="AU13" t="inlineStr"/>
-      <c r="AV13" t="inlineStr"/>
-      <c r="AW13" t="inlineStr"/>
-      <c r="AX13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>Nomura International plc、モルガン・スタンレーMUFG証券株式会社</t>
+        </is>
+      </c>
+      <c r="AW13" t="n">
+        <v>0.0077</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>72800</v>
+      </c>
       <c r="AY13" t="inlineStr"/>
       <c r="AZ13" t="inlineStr"/>
       <c r="BA13" t="inlineStr"/>
@@ -2900,7 +2774,7 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="n">
-        <v>103320</v>
+        <v>2177820</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2909,13 +2783,13 @@
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="n">
-        <v>198733.3333333333</v>
+        <v>2057900</v>
       </c>
       <c r="BO13" t="n">
-        <v>103320</v>
+        <v>2177820</v>
       </c>
       <c r="BP13" t="n">
-        <v>96350860</v>
+        <v>2332905800</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2924,10 +2798,10 @@
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="n">
-        <v>185306366.6666667</v>
+        <v>2105307200</v>
       </c>
       <c r="BX13" t="n">
-        <v>96350860</v>
+        <v>2332905800</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2935,44 +2809,44 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>546A</t>
+          <t>549A</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ＭＩＲＡＩＮＩホールディングス</t>
+          <t>ヒトトヒトホールディングス</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>プライム</t>
+          <t>スタンダード</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>商社・卸売</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>卸売業</t>
+          <t>サービス業</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2987,7 +2861,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>1861</v>
+        <v>596</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -3009,21 +2883,15 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="n">
-        <v>6700</v>
-      </c>
-      <c r="AE14" t="n">
-        <v>546000</v>
-      </c>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr"/>
       <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="n">
-        <v>546000</v>
-      </c>
+      <c r="AL14" t="inlineStr"/>
       <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
@@ -3031,20 +2899,18 @@
       <c r="AQ14" t="inlineStr"/>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
-      <c r="AT14" t="n">
-        <v>6700</v>
-      </c>
+      <c r="AT14" t="inlineStr"/>
       <c r="AU14" t="inlineStr"/>
       <c r="AV14" t="inlineStr">
         <is>
-          <t>GOLDMAN SACHS INTERNATIONAL</t>
+          <t>野村證券株式会社</t>
         </is>
       </c>
       <c r="AW14" t="n">
-        <v>0.0041</v>
+        <v>0.0375</v>
       </c>
       <c r="AX14" t="n">
-        <v>146386</v>
+        <v>525000</v>
       </c>
       <c r="AY14" t="inlineStr"/>
       <c r="AZ14" t="inlineStr"/>
@@ -3052,14 +2918,12 @@
       <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr"/>
       <c r="BD14" t="inlineStr"/>
-      <c r="BE14" t="n">
-        <v>194633</v>
-      </c>
+      <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="n">
-        <v>146386</v>
+        <v>525000</v>
       </c>
       <c r="BG14" t="n">
-        <v>167780</v>
+        <v>6291160</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -3067,14 +2931,12 @@
       <c r="BK14" t="inlineStr"/>
       <c r="BL14" t="inlineStr"/>
       <c r="BM14" t="inlineStr"/>
-      <c r="BN14" t="n">
-        <v>206866.6666666667</v>
-      </c>
+      <c r="BN14" t="inlineStr"/>
       <c r="BO14" t="n">
-        <v>167780</v>
+        <v>6291160</v>
       </c>
       <c r="BP14" t="n">
-        <v>314505480</v>
+        <v>3593526160</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -3082,11 +2944,9 @@
       <c r="BT14" t="inlineStr"/>
       <c r="BU14" t="inlineStr"/>
       <c r="BV14" t="inlineStr"/>
-      <c r="BW14" t="n">
-        <v>375613033.3333333</v>
-      </c>
+      <c r="BW14" t="inlineStr"/>
       <c r="BX14" t="n">
-        <v>314505480</v>
+        <v>3593526160</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -3094,44 +2954,44 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>547A</t>
+          <t>550A</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ムニノバホールディングス</t>
+          <t>ソフトテックス</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>プライム</t>
+          <t>スタンダード</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>金融（除く銀行）</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>その他金融業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3146,7 +3006,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>413</v>
+        <v>3815</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -3168,21 +3028,15 @@
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
-      <c r="AD15" t="n">
-        <v>86900</v>
-      </c>
-      <c r="AE15" t="n">
-        <v>11624300</v>
-      </c>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
       <c r="AF15" t="inlineStr"/>
       <c r="AG15" t="inlineStr"/>
       <c r="AH15" t="inlineStr"/>
       <c r="AI15" t="inlineStr"/>
       <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr"/>
-      <c r="AL15" t="n">
-        <v>11624300</v>
-      </c>
+      <c r="AL15" t="inlineStr"/>
       <c r="AM15" t="inlineStr"/>
       <c r="AN15" t="inlineStr"/>
       <c r="AO15" t="inlineStr"/>
@@ -3190,9 +3044,7 @@
       <c r="AQ15" t="inlineStr"/>
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
-      <c r="AT15" t="n">
-        <v>86900</v>
-      </c>
+      <c r="AT15" t="inlineStr"/>
       <c r="AU15" t="inlineStr"/>
       <c r="AV15" t="inlineStr"/>
       <c r="AW15" t="inlineStr"/>
@@ -3206,7 +3058,7 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>2157100</v>
+        <v>631566.6666666666</v>
       </c>
       <c r="BH15" t="inlineStr"/>
       <c r="BI15" t="inlineStr"/>
@@ -3214,14 +3066,12 @@
       <c r="BK15" t="inlineStr"/>
       <c r="BL15" t="inlineStr"/>
       <c r="BM15" t="inlineStr"/>
-      <c r="BN15" t="n">
-        <v>2252600</v>
-      </c>
+      <c r="BN15" t="inlineStr"/>
       <c r="BO15" t="n">
-        <v>2157100</v>
+        <v>631566.6666666666</v>
       </c>
       <c r="BP15" t="n">
-        <v>920704780</v>
+        <v>1921926166.666667</v>
       </c>
       <c r="BQ15" t="inlineStr"/>
       <c r="BR15" t="inlineStr"/>
@@ -3229,11 +3079,9 @@
       <c r="BT15" t="inlineStr"/>
       <c r="BU15" t="inlineStr"/>
       <c r="BV15" t="inlineStr"/>
-      <c r="BW15" t="n">
-        <v>988981966.6666666</v>
-      </c>
+      <c r="BW15" t="inlineStr"/>
       <c r="BX15" t="n">
-        <v>920704780</v>
+        <v>1921926166.666667</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3241,29 +3089,29 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>548A</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>システムエグゼ</t>
+          <t>日本銀行</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3273,12 +3121,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>銀行</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>銀行業</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3293,7 +3141,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>966</v>
+        <v>25000</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3345,30 +3193,58 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>2510860</v>
-      </c>
-      <c r="BH16" t="inlineStr"/>
-      <c r="BI16" t="inlineStr"/>
-      <c r="BJ16" t="inlineStr"/>
-      <c r="BK16" t="inlineStr"/>
-      <c r="BL16" t="inlineStr"/>
-      <c r="BM16" t="inlineStr"/>
-      <c r="BN16" t="inlineStr"/>
+        <v>166.6666666666667</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>875</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>100</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>450</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>300</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>166.6666666666667</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>250</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>266.6666666666667</v>
+      </c>
       <c r="BO16" t="n">
-        <v>2510860</v>
+        <v>166.6666666666667</v>
       </c>
       <c r="BP16" t="n">
-        <v>2679272900</v>
-      </c>
-      <c r="BQ16" t="inlineStr"/>
-      <c r="BR16" t="inlineStr"/>
-      <c r="BS16" t="inlineStr"/>
-      <c r="BT16" t="inlineStr"/>
-      <c r="BU16" t="inlineStr"/>
-      <c r="BV16" t="inlineStr"/>
-      <c r="BW16" t="inlineStr"/>
+        <v>4147000</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>23735750</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>2650000</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>11285000</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>7486400</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>4104666.666666667</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>6260000</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>6588333.333333333</v>
+      </c>
       <c r="BX16" t="n">
-        <v>2679272900</v>
+        <v>4147000</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3376,29 +3252,29 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>549A</t>
+          <t>9399</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ヒトトヒトホールディングス</t>
+          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3413,7 +3289,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>サービス業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3428,7 +3304,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>593</v>
+        <v>28</v>
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -3450,35 +3326,59 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
-      <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
-      <c r="AG17" t="inlineStr"/>
-      <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
-      <c r="AL17" t="inlineStr"/>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>122230</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>204885</v>
+      </c>
+      <c r="AG17" t="n">
+        <v>97185</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>93675</v>
+      </c>
+      <c r="AI17" t="n">
+        <v>126528</v>
+      </c>
+      <c r="AJ17" t="n">
+        <v>99264</v>
+      </c>
+      <c r="AK17" t="n">
+        <v>96080</v>
+      </c>
+      <c r="AL17" t="n">
+        <v>122230</v>
+      </c>
       <c r="AM17" t="inlineStr"/>
-      <c r="AN17" t="inlineStr"/>
-      <c r="AO17" t="inlineStr"/>
-      <c r="AP17" t="inlineStr"/>
-      <c r="AQ17" t="inlineStr"/>
-      <c r="AR17" t="inlineStr"/>
-      <c r="AS17" t="inlineStr"/>
-      <c r="AT17" t="inlineStr"/>
+      <c r="AN17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT17" t="n">
+        <v>0</v>
+      </c>
       <c r="AU17" t="inlineStr"/>
-      <c r="AV17" t="inlineStr">
-        <is>
-          <t>野村證券株式会社</t>
-        </is>
-      </c>
-      <c r="AW17" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="AX17" t="n">
-        <v>525000</v>
-      </c>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
       <c r="AY17" t="inlineStr"/>
       <c r="AZ17" t="inlineStr"/>
       <c r="BA17" t="inlineStr"/>
@@ -3486,34 +3386,60 @@
       <c r="BC17" t="inlineStr"/>
       <c r="BD17" t="inlineStr"/>
       <c r="BE17" t="inlineStr"/>
-      <c r="BF17" t="n">
-        <v>525000</v>
-      </c>
+      <c r="BF17" t="inlineStr"/>
       <c r="BG17" t="n">
-        <v>6937850</v>
-      </c>
-      <c r="BH17" t="inlineStr"/>
-      <c r="BI17" t="inlineStr"/>
-      <c r="BJ17" t="inlineStr"/>
-      <c r="BK17" t="inlineStr"/>
-      <c r="BL17" t="inlineStr"/>
-      <c r="BM17" t="inlineStr"/>
-      <c r="BN17" t="inlineStr"/>
+        <v>3463774</v>
+      </c>
+      <c r="BH17" t="n">
+        <v>13931419.2</v>
+      </c>
+      <c r="BI17" t="n">
+        <v>5104435.2</v>
+      </c>
+      <c r="BJ17" t="n">
+        <v>3130213.4</v>
+      </c>
+      <c r="BK17" t="n">
+        <v>3424175.2</v>
+      </c>
+      <c r="BL17" t="n">
+        <v>4747035.2</v>
+      </c>
+      <c r="BM17" t="n">
+        <v>1966370.8</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>1960023.6</v>
+      </c>
       <c r="BO17" t="n">
-        <v>6937850</v>
+        <v>3463774</v>
       </c>
       <c r="BP17" t="n">
-        <v>3931852700</v>
-      </c>
-      <c r="BQ17" t="inlineStr"/>
-      <c r="BR17" t="inlineStr"/>
-      <c r="BS17" t="inlineStr"/>
-      <c r="BT17" t="inlineStr"/>
-      <c r="BU17" t="inlineStr"/>
-      <c r="BV17" t="inlineStr"/>
-      <c r="BW17" t="inlineStr"/>
+        <v>100737881.8</v>
+      </c>
+      <c r="BQ17" t="n">
+        <v>356289258</v>
+      </c>
+      <c r="BR17" t="n">
+        <v>147240261</v>
+      </c>
+      <c r="BS17" t="n">
+        <v>83366454.8</v>
+      </c>
+      <c r="BT17" t="n">
+        <v>100089101.6</v>
+      </c>
+      <c r="BU17" t="n">
+        <v>150288273.6</v>
+      </c>
+      <c r="BV17" t="n">
+        <v>58329980.2</v>
+      </c>
+      <c r="BW17" t="n">
+        <v>52706922.8</v>
+      </c>
       <c r="BX17" t="n">
-        <v>3931852700</v>
+        <v>100737881.8</v>
       </c>
       <c r="BY17" t="inlineStr"/>
       <c r="BZ17" t="inlineStr"/>
@@ -3521,510 +3447,17 @@
       <c r="CB17" t="inlineStr"/>
       <c r="CC17" t="inlineStr">
         <is>
-          <t>20260412-190048</t>
+          <t>20260413-190053</t>
         </is>
       </c>
       <c r="CD17" t="inlineStr">
         <is>
-          <t>2026-04-12T10:00:48+00:00</t>
+          <t>2026-04-13T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE17" t="inlineStr">
         <is>
-          <t>2026-04-12T19:00:48+09:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>550A</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ソフトテックス</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>スタンダード</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>情報通信・サービスその他</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>情報･通信業</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>fins_summary_api_fail</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>RuntimeError: empty /fins/summary</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>3115</v>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
-      <c r="AF18" t="inlineStr"/>
-      <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
-      <c r="AK18" t="inlineStr"/>
-      <c r="AL18" t="inlineStr"/>
-      <c r="AM18" t="inlineStr"/>
-      <c r="AN18" t="inlineStr"/>
-      <c r="AO18" t="inlineStr"/>
-      <c r="AP18" t="inlineStr"/>
-      <c r="AQ18" t="inlineStr"/>
-      <c r="AR18" t="inlineStr"/>
-      <c r="AS18" t="inlineStr"/>
-      <c r="AT18" t="inlineStr"/>
-      <c r="AU18" t="inlineStr"/>
-      <c r="AV18" t="inlineStr"/>
-      <c r="AW18" t="inlineStr"/>
-      <c r="AX18" t="inlineStr"/>
-      <c r="AY18" t="inlineStr"/>
-      <c r="AZ18" t="inlineStr"/>
-      <c r="BA18" t="inlineStr"/>
-      <c r="BB18" t="inlineStr"/>
-      <c r="BC18" t="inlineStr"/>
-      <c r="BD18" t="inlineStr"/>
-      <c r="BE18" t="inlineStr"/>
-      <c r="BF18" t="inlineStr"/>
-      <c r="BG18" t="n">
-        <v>818800</v>
-      </c>
-      <c r="BH18" t="inlineStr"/>
-      <c r="BI18" t="inlineStr"/>
-      <c r="BJ18" t="inlineStr"/>
-      <c r="BK18" t="inlineStr"/>
-      <c r="BL18" t="inlineStr"/>
-      <c r="BM18" t="inlineStr"/>
-      <c r="BN18" t="inlineStr"/>
-      <c r="BO18" t="n">
-        <v>818800</v>
-      </c>
-      <c r="BP18" t="n">
-        <v>2428380250</v>
-      </c>
-      <c r="BQ18" t="inlineStr"/>
-      <c r="BR18" t="inlineStr"/>
-      <c r="BS18" t="inlineStr"/>
-      <c r="BT18" t="inlineStr"/>
-      <c r="BU18" t="inlineStr"/>
-      <c r="BV18" t="inlineStr"/>
-      <c r="BW18" t="inlineStr"/>
-      <c r="BX18" t="n">
-        <v>2428380250</v>
-      </c>
-      <c r="BY18" t="inlineStr"/>
-      <c r="BZ18" t="inlineStr"/>
-      <c r="CA18" t="inlineStr"/>
-      <c r="CB18" t="inlineStr"/>
-      <c r="CC18" t="inlineStr">
-        <is>
-          <t>20260412-190048</t>
-        </is>
-      </c>
-      <c r="CD18" t="inlineStr">
-        <is>
-          <t>2026-04-12T10:00:48+00:00</t>
-        </is>
-      </c>
-      <c r="CE18" t="inlineStr">
-        <is>
-          <t>2026-04-12T19:00:48+09:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>8301</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>日本銀行</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>スタンダード</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>銀行</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>銀行業</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>fins_summary_api_fail</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>RuntimeError: empty /fins/summary</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>25000</v>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
-      <c r="AB19" t="inlineStr"/>
-      <c r="AC19" t="inlineStr"/>
-      <c r="AD19" t="inlineStr"/>
-      <c r="AE19" t="inlineStr"/>
-      <c r="AF19" t="inlineStr"/>
-      <c r="AG19" t="inlineStr"/>
-      <c r="AH19" t="inlineStr"/>
-      <c r="AI19" t="inlineStr"/>
-      <c r="AJ19" t="inlineStr"/>
-      <c r="AK19" t="inlineStr"/>
-      <c r="AL19" t="inlineStr"/>
-      <c r="AM19" t="inlineStr"/>
-      <c r="AN19" t="inlineStr"/>
-      <c r="AO19" t="inlineStr"/>
-      <c r="AP19" t="inlineStr"/>
-      <c r="AQ19" t="inlineStr"/>
-      <c r="AR19" t="inlineStr"/>
-      <c r="AS19" t="inlineStr"/>
-      <c r="AT19" t="inlineStr"/>
-      <c r="AU19" t="inlineStr"/>
-      <c r="AV19" t="inlineStr"/>
-      <c r="AW19" t="inlineStr"/>
-      <c r="AX19" t="inlineStr"/>
-      <c r="AY19" t="inlineStr"/>
-      <c r="AZ19" t="inlineStr"/>
-      <c r="BA19" t="inlineStr"/>
-      <c r="BB19" t="inlineStr"/>
-      <c r="BC19" t="inlineStr"/>
-      <c r="BD19" t="inlineStr"/>
-      <c r="BE19" t="inlineStr"/>
-      <c r="BF19" t="inlineStr"/>
-      <c r="BG19" t="n">
-        <v>133.3333333333333</v>
-      </c>
-      <c r="BH19" t="n">
-        <v>925</v>
-      </c>
-      <c r="BI19" t="n">
-        <v>100</v>
-      </c>
-      <c r="BJ19" t="n">
-        <v>450</v>
-      </c>
-      <c r="BK19" t="n">
-        <v>200</v>
-      </c>
-      <c r="BL19" t="n">
-        <v>300</v>
-      </c>
-      <c r="BM19" t="n">
-        <v>250</v>
-      </c>
-      <c r="BN19" t="n">
-        <v>300</v>
-      </c>
-      <c r="BO19" t="n">
-        <v>133.3333333333333</v>
-      </c>
-      <c r="BP19" t="n">
-        <v>3333666.666666667</v>
-      </c>
-      <c r="BQ19" t="n">
-        <v>25063500</v>
-      </c>
-      <c r="BR19" t="n">
-        <v>2645000</v>
-      </c>
-      <c r="BS19" t="n">
-        <v>11285000</v>
-      </c>
-      <c r="BT19" t="n">
-        <v>4993250</v>
-      </c>
-      <c r="BU19" t="n">
-        <v>7443250</v>
-      </c>
-      <c r="BV19" t="n">
-        <v>6260000</v>
-      </c>
-      <c r="BW19" t="n">
-        <v>7372000</v>
-      </c>
-      <c r="BX19" t="n">
-        <v>3333666.666666667</v>
-      </c>
-      <c r="BY19" t="inlineStr"/>
-      <c r="BZ19" t="inlineStr"/>
-      <c r="CA19" t="inlineStr"/>
-      <c r="CB19" t="inlineStr"/>
-      <c r="CC19" t="inlineStr">
-        <is>
-          <t>20260412-190048</t>
-        </is>
-      </c>
-      <c r="CD19" t="inlineStr">
-        <is>
-          <t>2026-04-12T10:00:48+00:00</t>
-        </is>
-      </c>
-      <c r="CE19" t="inlineStr">
-        <is>
-          <t>2026-04-12T19:00:48+09:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>9399</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>スタンダード</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>情報通信・サービスその他</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>情報･通信業</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>fins_summary_api_fail</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>RuntimeError: empty /fins/summary</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>28</v>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
-      <c r="AB20" t="inlineStr"/>
-      <c r="AC20" t="inlineStr"/>
-      <c r="AD20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE20" t="n">
-        <v>122230</v>
-      </c>
-      <c r="AF20" t="n">
-        <v>204885</v>
-      </c>
-      <c r="AG20" t="n">
-        <v>97185</v>
-      </c>
-      <c r="AH20" t="n">
-        <v>93675</v>
-      </c>
-      <c r="AI20" t="n">
-        <v>126528</v>
-      </c>
-      <c r="AJ20" t="n">
-        <v>99264</v>
-      </c>
-      <c r="AK20" t="n">
-        <v>96080</v>
-      </c>
-      <c r="AL20" t="n">
-        <v>122230</v>
-      </c>
-      <c r="AM20" t="inlineStr"/>
-      <c r="AN20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT20" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU20" t="inlineStr"/>
-      <c r="AV20" t="inlineStr"/>
-      <c r="AW20" t="inlineStr"/>
-      <c r="AX20" t="inlineStr"/>
-      <c r="AY20" t="inlineStr"/>
-      <c r="AZ20" t="inlineStr"/>
-      <c r="BA20" t="inlineStr"/>
-      <c r="BB20" t="inlineStr"/>
-      <c r="BC20" t="inlineStr"/>
-      <c r="BD20" t="inlineStr"/>
-      <c r="BE20" t="inlineStr"/>
-      <c r="BF20" t="inlineStr"/>
-      <c r="BG20" t="n">
-        <v>3083292.6</v>
-      </c>
-      <c r="BH20" t="n">
-        <v>12912269</v>
-      </c>
-      <c r="BI20" t="n">
-        <v>7299611.6</v>
-      </c>
-      <c r="BJ20" t="n">
-        <v>2742294</v>
-      </c>
-      <c r="BK20" t="n">
-        <v>3912781</v>
-      </c>
-      <c r="BL20" t="n">
-        <v>4714386.8</v>
-      </c>
-      <c r="BM20" t="n">
-        <v>2238110.2</v>
-      </c>
-      <c r="BN20" t="n">
-        <v>1913806.6</v>
-      </c>
-      <c r="BO20" t="n">
-        <v>3083292.6</v>
-      </c>
-      <c r="BP20" t="n">
-        <v>88928311</v>
-      </c>
-      <c r="BQ20" t="n">
-        <v>314646947.2</v>
-      </c>
-      <c r="BR20" t="n">
-        <v>226772440</v>
-      </c>
-      <c r="BS20" t="n">
-        <v>69693452.8</v>
-      </c>
-      <c r="BT20" t="n">
-        <v>114743178.6</v>
-      </c>
-      <c r="BU20" t="n">
-        <v>148128099</v>
-      </c>
-      <c r="BV20" t="n">
-        <v>67164683.59999999</v>
-      </c>
-      <c r="BW20" t="n">
-        <v>52170691.2</v>
-      </c>
-      <c r="BX20" t="n">
-        <v>88928311</v>
-      </c>
-      <c r="BY20" t="inlineStr"/>
-      <c r="BZ20" t="inlineStr"/>
-      <c r="CA20" t="inlineStr"/>
-      <c r="CB20" t="inlineStr"/>
-      <c r="CC20" t="inlineStr">
-        <is>
-          <t>20260412-190048</t>
-        </is>
-      </c>
-      <c r="CD20" t="inlineStr">
-        <is>
-          <t>2026-04-12T10:00:48+00:00</t>
-        </is>
-      </c>
-      <c r="CE20" t="inlineStr">
-        <is>
-          <t>2026-04-12T19:00:48+09:00</t>
+          <t>2026-04-13T19:00:53+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-14
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE17"/>
+  <dimension ref="A1:CE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -909,7 +909,7 @@
         <v>0</v>
       </c>
       <c r="AE2" t="n">
-        <v>31000</v>
+        <v>30000</v>
       </c>
       <c r="AF2" t="n">
         <v>15000</v>
@@ -932,7 +932,9 @@
       <c r="AL2" t="n">
         <v>31000</v>
       </c>
-      <c r="AM2" t="inlineStr"/>
+      <c r="AM2" t="n">
+        <v>30000</v>
+      </c>
       <c r="AN2" t="n">
         <v>0</v>
       </c>
@@ -954,7 +956,9 @@
       <c r="AT2" t="n">
         <v>0</v>
       </c>
-      <c r="AU2" t="inlineStr"/>
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
@@ -970,55 +974,55 @@
         <v>16200</v>
       </c>
       <c r="BH2" t="n">
-        <v>10400</v>
+        <v>9600</v>
       </c>
       <c r="BI2" t="n">
-        <v>15400</v>
+        <v>16200</v>
       </c>
       <c r="BJ2" t="n">
-        <v>11000</v>
+        <v>22400</v>
       </c>
       <c r="BK2" t="n">
-        <v>25800</v>
+        <v>14200</v>
       </c>
       <c r="BL2" t="n">
-        <v>15800</v>
+        <v>14000</v>
       </c>
       <c r="BM2" t="n">
-        <v>14200</v>
+        <v>16000</v>
       </c>
       <c r="BN2" t="n">
-        <v>25400</v>
+        <v>26400</v>
       </c>
       <c r="BO2" t="n">
         <v>16200</v>
       </c>
       <c r="BP2" t="n">
-        <v>1214600</v>
+        <v>1232000</v>
       </c>
       <c r="BQ2" t="n">
-        <v>831600</v>
+        <v>772000</v>
       </c>
       <c r="BR2" t="n">
-        <v>1212800</v>
+        <v>1272800</v>
       </c>
       <c r="BS2" t="n">
-        <v>852400</v>
+        <v>1628000</v>
       </c>
       <c r="BT2" t="n">
-        <v>1810200</v>
+        <v>993800</v>
       </c>
       <c r="BU2" t="n">
-        <v>1101600</v>
+        <v>979400</v>
       </c>
       <c r="BV2" t="n">
-        <v>955400</v>
+        <v>1072200</v>
       </c>
       <c r="BW2" t="n">
-        <v>1778000</v>
+        <v>1869600</v>
       </c>
       <c r="BX2" t="n">
-        <v>1214600</v>
+        <v>1232000</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1026,17 +1030,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1082,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1104,7 +1108,7 @@
         <v>0</v>
       </c>
       <c r="AE3" t="n">
-        <v>76800</v>
+        <v>78200</v>
       </c>
       <c r="AF3" t="n">
         <v>57400</v>
@@ -1127,7 +1131,9 @@
       <c r="AL3" t="n">
         <v>76800</v>
       </c>
-      <c r="AM3" t="inlineStr"/>
+      <c r="AM3" t="n">
+        <v>78200</v>
+      </c>
       <c r="AN3" t="n">
         <v>0</v>
       </c>
@@ -1149,7 +1155,9 @@
       <c r="AT3" t="n">
         <v>0</v>
       </c>
-      <c r="AU3" t="inlineStr"/>
+      <c r="AU3" t="n">
+        <v>0</v>
+      </c>
       <c r="AV3" t="inlineStr"/>
       <c r="AW3" t="inlineStr"/>
       <c r="AX3" t="inlineStr"/>
@@ -1162,58 +1170,58 @@
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="n">
-        <v>36680</v>
+        <v>38680</v>
       </c>
       <c r="BH3" t="n">
-        <v>75940</v>
+        <v>64700</v>
       </c>
       <c r="BI3" t="n">
-        <v>63460</v>
+        <v>59380</v>
       </c>
       <c r="BJ3" t="n">
-        <v>68420</v>
+        <v>77740</v>
       </c>
       <c r="BK3" t="n">
-        <v>58460</v>
+        <v>48480</v>
       </c>
       <c r="BL3" t="n">
-        <v>101700</v>
+        <v>103840</v>
       </c>
       <c r="BM3" t="n">
-        <v>40220</v>
+        <v>33720</v>
       </c>
       <c r="BN3" t="n">
-        <v>16280</v>
+        <v>13980</v>
       </c>
       <c r="BO3" t="n">
-        <v>36680</v>
+        <v>38680</v>
       </c>
       <c r="BP3" t="n">
-        <v>8475240</v>
+        <v>8961740</v>
       </c>
       <c r="BQ3" t="n">
-        <v>19566000</v>
+        <v>16438180</v>
       </c>
       <c r="BR3" t="n">
-        <v>15580660</v>
+        <v>14522900</v>
       </c>
       <c r="BS3" t="n">
-        <v>15720080</v>
+        <v>17546800</v>
       </c>
       <c r="BT3" t="n">
-        <v>13031980</v>
+        <v>10831060</v>
       </c>
       <c r="BU3" t="n">
-        <v>23672580</v>
+        <v>24264960</v>
       </c>
       <c r="BV3" t="n">
-        <v>9151220</v>
+        <v>7616900</v>
       </c>
       <c r="BW3" t="n">
-        <v>3639380</v>
+        <v>3137240</v>
       </c>
       <c r="BX3" t="n">
-        <v>8475240</v>
+        <v>8961740</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1221,17 +1229,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1281,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>750</v>
+        <v>703</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1299,7 +1307,7 @@
         <v>0</v>
       </c>
       <c r="AE4" t="n">
-        <v>234400</v>
+        <v>246800</v>
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
@@ -1320,7 +1328,9 @@
       <c r="AL4" t="n">
         <v>234400</v>
       </c>
-      <c r="AM4" t="inlineStr"/>
+      <c r="AM4" t="n">
+        <v>246800</v>
+      </c>
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="n">
         <v>0</v>
@@ -1340,7 +1350,9 @@
       <c r="AT4" t="n">
         <v>0</v>
       </c>
-      <c r="AU4" t="inlineStr"/>
+      <c r="AU4" t="n">
+        <v>0</v>
+      </c>
       <c r="AV4" t="inlineStr">
         <is>
           <t>野村證券株式会社</t>
@@ -1375,54 +1387,54 @@
         <v>0</v>
       </c>
       <c r="BG4" t="n">
-        <v>86180</v>
+        <v>101180</v>
       </c>
       <c r="BH4" t="inlineStr"/>
       <c r="BI4" t="n">
-        <v>1096975</v>
+        <v>971220</v>
       </c>
       <c r="BJ4" t="n">
-        <v>229200</v>
+        <v>162400</v>
       </c>
       <c r="BK4" t="n">
-        <v>104900</v>
+        <v>94040</v>
       </c>
       <c r="BL4" t="n">
-        <v>127240</v>
+        <v>125360</v>
       </c>
       <c r="BM4" t="n">
-        <v>82900</v>
+        <v>86440</v>
       </c>
       <c r="BN4" t="n">
-        <v>61860</v>
+        <v>54260</v>
       </c>
       <c r="BO4" t="n">
-        <v>86180</v>
+        <v>101180</v>
       </c>
       <c r="BP4" t="n">
-        <v>67974940</v>
+        <v>77627380</v>
       </c>
       <c r="BQ4" t="inlineStr"/>
       <c r="BR4" t="n">
-        <v>1152932450</v>
+        <v>1018630620</v>
       </c>
       <c r="BS4" t="n">
-        <v>238575980</v>
+        <v>168932740</v>
       </c>
       <c r="BT4" t="n">
-        <v>108578560</v>
+        <v>98665760</v>
       </c>
       <c r="BU4" t="n">
-        <v>123609800</v>
+        <v>119082120</v>
       </c>
       <c r="BV4" t="n">
-        <v>70208720</v>
+        <v>72462920</v>
       </c>
       <c r="BW4" t="n">
-        <v>50250980</v>
+        <v>44134900</v>
       </c>
       <c r="BX4" t="n">
-        <v>67974940</v>
+        <v>77627380</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1430,17 +1442,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1494,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>692</v>
+        <v>677</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1508,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="AE5" t="n">
-        <v>56200</v>
+        <v>59600</v>
       </c>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
@@ -1521,7 +1533,9 @@
       <c r="AL5" t="n">
         <v>56200</v>
       </c>
-      <c r="AM5" t="inlineStr"/>
+      <c r="AM5" t="n">
+        <v>59600</v>
+      </c>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr"/>
@@ -1533,7 +1547,9 @@
       <c r="AT5" t="n">
         <v>0</v>
       </c>
-      <c r="AU5" t="inlineStr"/>
+      <c r="AU5" t="n">
+        <v>0</v>
+      </c>
       <c r="AV5" t="inlineStr"/>
       <c r="AW5" t="inlineStr"/>
       <c r="AX5" t="inlineStr"/>
@@ -1546,7 +1562,7 @@
       <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="n">
-        <v>18880</v>
+        <v>18080</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="inlineStr"/>
@@ -1554,16 +1570,16 @@
       <c r="BK5" t="inlineStr"/>
       <c r="BL5" t="inlineStr"/>
       <c r="BM5" t="n">
-        <v>318525</v>
+        <v>262360</v>
       </c>
       <c r="BN5" t="n">
-        <v>30900</v>
+        <v>28760</v>
       </c>
       <c r="BO5" t="n">
-        <v>18880</v>
+        <v>18080</v>
       </c>
       <c r="BP5" t="n">
-        <v>12917580</v>
+        <v>12388760</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="inlineStr"/>
@@ -1571,13 +1587,13 @@
       <c r="BT5" t="inlineStr"/>
       <c r="BU5" t="inlineStr"/>
       <c r="BV5" t="n">
-        <v>247000550</v>
+        <v>202733020</v>
       </c>
       <c r="BW5" t="n">
-        <v>21013720</v>
+        <v>19548000</v>
       </c>
       <c r="BX5" t="n">
-        <v>12917580</v>
+        <v>12388760</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1585,17 +1601,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1653,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>668</v>
+        <v>660</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1663,7 +1679,7 @@
         <v>0</v>
       </c>
       <c r="AE6" t="n">
-        <v>106000</v>
+        <v>181100</v>
       </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
@@ -1676,7 +1692,9 @@
       <c r="AL6" t="n">
         <v>106000</v>
       </c>
-      <c r="AM6" t="inlineStr"/>
+      <c r="AM6" t="n">
+        <v>181100</v>
+      </c>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="inlineStr"/>
@@ -1688,7 +1706,9 @@
       <c r="AT6" t="n">
         <v>0</v>
       </c>
-      <c r="AU6" t="inlineStr"/>
+      <c r="AU6" t="n">
+        <v>0</v>
+      </c>
       <c r="AV6" t="inlineStr"/>
       <c r="AW6" t="inlineStr"/>
       <c r="AX6" t="inlineStr"/>
@@ -1701,7 +1721,7 @@
       <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="n">
-        <v>40500</v>
+        <v>35420</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
@@ -1709,16 +1729,16 @@
       <c r="BK6" t="inlineStr"/>
       <c r="BL6" t="inlineStr"/>
       <c r="BM6" t="n">
-        <v>540325</v>
+        <v>484140</v>
       </c>
       <c r="BN6" t="n">
-        <v>140100</v>
+        <v>96860</v>
       </c>
       <c r="BO6" t="n">
-        <v>40500</v>
+        <v>35420</v>
       </c>
       <c r="BP6" t="n">
-        <v>27184060</v>
+        <v>23739800</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
@@ -1726,13 +1746,13 @@
       <c r="BT6" t="inlineStr"/>
       <c r="BU6" t="inlineStr"/>
       <c r="BV6" t="n">
-        <v>389225050</v>
+        <v>348791500</v>
       </c>
       <c r="BW6" t="n">
-        <v>98474520</v>
+        <v>66866560</v>
       </c>
       <c r="BX6" t="n">
-        <v>27184060</v>
+        <v>23739800</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1740,44 +1760,44 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>523A</t>
+          <t>543A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>セイワホールディングス</t>
+          <t>ＡＲＣＨＩＯＮ</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>グロース</t>
+          <t>プライム</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>建設・資材</t>
+          <t>自動車・輸送機</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>金属製品</t>
+          <t>輸送用機器</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1792,7 +1812,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>1497</v>
+        <v>408</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1815,46 +1835,38 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="n">
-        <v>0</v>
+        <v>92700</v>
       </c>
       <c r="AE7" t="n">
-        <v>634100</v>
+        <v>8141200</v>
       </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="n">
-        <v>408200</v>
-      </c>
+      <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="n">
-        <v>634100</v>
-      </c>
-      <c r="AM7" t="inlineStr"/>
+        <v>3478500</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>8141200</v>
+      </c>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="n">
-        <v>0</v>
-      </c>
+      <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr">
-        <is>
-          <t>Jump Trading Pacific Pte Ltd</t>
-        </is>
-      </c>
-      <c r="AW7" t="n">
-        <v>0.0051</v>
-      </c>
-      <c r="AX7" t="n">
-        <v>97000</v>
-      </c>
+        <v>673100</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>92700</v>
+      </c>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
       <c r="AY7" t="inlineStr"/>
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="inlineStr"/>
@@ -1862,42 +1874,36 @@
       <c r="BC7" t="inlineStr"/>
       <c r="BD7" t="inlineStr"/>
       <c r="BE7" t="inlineStr"/>
-      <c r="BF7" t="n">
-        <v>97000</v>
-      </c>
+      <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>579780</v>
+        <v>11416840</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
       <c r="BJ7" t="inlineStr"/>
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="n">
-        <v>7535550</v>
-      </c>
+      <c r="BM7" t="inlineStr"/>
       <c r="BN7" t="n">
-        <v>2620900</v>
+        <v>21773700</v>
       </c>
       <c r="BO7" t="n">
-        <v>579780</v>
+        <v>11416840</v>
       </c>
       <c r="BP7" t="n">
-        <v>866355580</v>
+        <v>4775020380</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
-      <c r="BV7" t="n">
-        <v>11342836750</v>
-      </c>
+      <c r="BV7" t="inlineStr"/>
       <c r="BW7" t="n">
-        <v>3937584140</v>
+        <v>10269101440</v>
       </c>
       <c r="BX7" t="n">
-        <v>866355580</v>
+        <v>4775020380</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -1905,29 +1911,29 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>543A</t>
+          <t>544A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ＡＲＣＨＩＯＮ</t>
+          <t>ＧＭＳグループ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1937,12 +1943,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>自動車・輸送機</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>輸送用機器</t>
+          <t>機械</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1957,7 +1963,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>428</v>
+        <v>409</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -1980,10 +1986,10 @@
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="n">
-        <v>673100</v>
+        <v>21600</v>
       </c>
       <c r="AE8" t="n">
-        <v>3478500</v>
+        <v>187000</v>
       </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
@@ -1992,9 +1998,11 @@
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="n">
-        <v>3478500</v>
-      </c>
-      <c r="AM8" t="inlineStr"/>
+        <v>126500</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>187000</v>
+      </c>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
@@ -2002,12 +2010,22 @@
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="n">
-        <v>673100</v>
-      </c>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
+        <v>39200</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>21600</v>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>GOLDMAN SACHS INTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.0053</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>379285</v>
+      </c>
       <c r="AY8" t="inlineStr"/>
       <c r="AZ8" t="inlineStr"/>
       <c r="BA8" t="inlineStr"/>
@@ -2015,9 +2033,11 @@
       <c r="BC8" t="inlineStr"/>
       <c r="BD8" t="inlineStr"/>
       <c r="BE8" t="inlineStr"/>
-      <c r="BF8" t="inlineStr"/>
+      <c r="BF8" t="n">
+        <v>379285</v>
+      </c>
       <c r="BG8" t="n">
-        <v>14445560</v>
+        <v>156560</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
@@ -2026,13 +2046,13 @@
       <c r="BL8" t="inlineStr"/>
       <c r="BM8" t="inlineStr"/>
       <c r="BN8" t="n">
-        <v>22304225</v>
+        <v>240660</v>
       </c>
       <c r="BO8" t="n">
-        <v>14445560</v>
+        <v>156560</v>
       </c>
       <c r="BP8" t="n">
-        <v>6156474700</v>
+        <v>64864340</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
@@ -2041,10 +2061,10 @@
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="inlineStr"/>
       <c r="BW8" t="n">
-        <v>10645521900</v>
+        <v>100115340</v>
       </c>
       <c r="BX8" t="n">
-        <v>6156474700</v>
+        <v>64864340</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2052,29 +2072,29 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>544A</t>
+          <t>545A</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ＧＭＳグループ</t>
+          <t>トランヴィア</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2084,12 +2104,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>機械</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>機械</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2104,7 +2124,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>410</v>
+        <v>928</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2127,10 +2147,10 @@
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
-        <v>39200</v>
+        <v>2200</v>
       </c>
       <c r="AE9" t="n">
-        <v>126500</v>
+        <v>62400</v>
       </c>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
@@ -2139,9 +2159,11 @@
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="n">
-        <v>126500</v>
-      </c>
-      <c r="AM9" t="inlineStr"/>
+        <v>62800</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>62400</v>
+      </c>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
@@ -2149,20 +2171,14 @@
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="n">
-        <v>39200</v>
-      </c>
-      <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr">
-        <is>
-          <t>GOLDMAN SACHS INTERNATIONAL</t>
-        </is>
-      </c>
-      <c r="AW9" t="n">
-        <v>0.0053</v>
-      </c>
-      <c r="AX9" t="n">
-        <v>379285</v>
-      </c>
+        <v>2200</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>2200</v>
+      </c>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
       <c r="AY9" t="inlineStr"/>
       <c r="AZ9" t="inlineStr"/>
       <c r="BA9" t="inlineStr"/>
@@ -2170,11 +2186,9 @@
       <c r="BC9" t="inlineStr"/>
       <c r="BD9" t="inlineStr"/>
       <c r="BE9" t="inlineStr"/>
-      <c r="BF9" t="n">
-        <v>379285</v>
-      </c>
+      <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>173700</v>
+        <v>77420</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
@@ -2183,13 +2197,13 @@
       <c r="BL9" t="inlineStr"/>
       <c r="BM9" t="inlineStr"/>
       <c r="BN9" t="n">
-        <v>248475</v>
+        <v>167980</v>
       </c>
       <c r="BO9" t="n">
-        <v>173700</v>
+        <v>77420</v>
       </c>
       <c r="BP9" t="n">
-        <v>72047820</v>
+        <v>72912260</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
@@ -2198,10 +2212,10 @@
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="inlineStr"/>
       <c r="BW9" t="n">
-        <v>103489250</v>
+        <v>156119560</v>
       </c>
       <c r="BX9" t="n">
-        <v>72047820</v>
+        <v>72912260</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2209,29 +2223,29 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>545A</t>
+          <t>546A</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>トランヴィア</t>
+          <t>ＭＩＲＡＩＮＩホールディングス</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2241,12 +2255,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>商社・卸売</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>卸売業</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2261,7 +2275,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>940</v>
+        <v>1870</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2284,10 +2298,10 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
-        <v>2200</v>
+        <v>12900</v>
       </c>
       <c r="AE10" t="n">
-        <v>62800</v>
+        <v>512700</v>
       </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
@@ -2296,9 +2310,11 @@
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="n">
-        <v>62800</v>
-      </c>
-      <c r="AM10" t="inlineStr"/>
+        <v>546000</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>512700</v>
+      </c>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
@@ -2306,22 +2322,36 @@
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="n">
-        <v>2200</v>
-      </c>
-      <c r="AU10" t="inlineStr"/>
-      <c r="AV10" t="inlineStr"/>
-      <c r="AW10" t="inlineStr"/>
-      <c r="AX10" t="inlineStr"/>
+        <v>6700</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>12900</v>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>GOLDMAN SACHS INTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.0041</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>146386</v>
+      </c>
       <c r="AY10" t="inlineStr"/>
       <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="inlineStr"/>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
       <c r="BD10" t="inlineStr"/>
-      <c r="BE10" t="inlineStr"/>
-      <c r="BF10" t="inlineStr"/>
+      <c r="BE10" t="n">
+        <v>194633</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>146386</v>
+      </c>
       <c r="BG10" t="n">
-        <v>98700</v>
+        <v>156680</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2330,13 +2360,13 @@
       <c r="BL10" t="inlineStr"/>
       <c r="BM10" t="inlineStr"/>
       <c r="BN10" t="n">
-        <v>171850</v>
+        <v>181100</v>
       </c>
       <c r="BO10" t="n">
-        <v>98700</v>
+        <v>156680</v>
       </c>
       <c r="BP10" t="n">
-        <v>92168220</v>
+        <v>295083620</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2345,10 +2375,10 @@
       <c r="BU10" t="inlineStr"/>
       <c r="BV10" t="inlineStr"/>
       <c r="BW10" t="n">
-        <v>160315700</v>
+        <v>330671340</v>
       </c>
       <c r="BX10" t="n">
-        <v>92168220</v>
+        <v>295083620</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2356,29 +2386,29 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>546A</t>
+          <t>547A</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ＭＩＲＡＩＮＩホールディングス</t>
+          <t>ムニノバホールディングス</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2388,12 +2418,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>商社・卸売</t>
+          <t>金融（除く銀行）</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>卸売業</t>
+          <t>その他金融業</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2408,7 +2438,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>1883</v>
+        <v>420</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2431,10 +2461,10 @@
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="n">
-        <v>6700</v>
+        <v>84500</v>
       </c>
       <c r="AE11" t="n">
-        <v>546000</v>
+        <v>12401300</v>
       </c>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
@@ -2443,9 +2473,11 @@
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="n">
-        <v>546000</v>
-      </c>
-      <c r="AM11" t="inlineStr"/>
+        <v>11624300</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>12401300</v>
+      </c>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
@@ -2453,34 +2485,24 @@
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="n">
-        <v>6700</v>
-      </c>
-      <c r="AU11" t="inlineStr"/>
-      <c r="AV11" t="inlineStr">
-        <is>
-          <t>GOLDMAN SACHS INTERNATIONAL</t>
-        </is>
-      </c>
-      <c r="AW11" t="n">
-        <v>0.0041</v>
-      </c>
-      <c r="AX11" t="n">
-        <v>146386</v>
-      </c>
+        <v>86900</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>84500</v>
+      </c>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
       <c r="AY11" t="inlineStr"/>
       <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="inlineStr"/>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
       <c r="BD11" t="inlineStr"/>
-      <c r="BE11" t="n">
-        <v>194633</v>
-      </c>
-      <c r="BF11" t="n">
-        <v>146386</v>
-      </c>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>152960</v>
+        <v>2388520</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2489,13 +2511,13 @@
       <c r="BL11" t="inlineStr"/>
       <c r="BM11" t="inlineStr"/>
       <c r="BN11" t="n">
-        <v>201300</v>
+        <v>2009960</v>
       </c>
       <c r="BO11" t="n">
-        <v>152960</v>
+        <v>2388520</v>
       </c>
       <c r="BP11" t="n">
-        <v>287691620</v>
+        <v>1012081120</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2504,10 +2526,10 @@
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="inlineStr"/>
       <c r="BW11" t="n">
-        <v>366972875</v>
+        <v>871040860</v>
       </c>
       <c r="BX11" t="n">
-        <v>287691620</v>
+        <v>1012081120</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2515,44 +2537,44 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>547A</t>
+          <t>548A</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ムニノバホールディングス</t>
+          <t>システムエグゼ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>プライム</t>
+          <t>スタンダード</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>金融（除く銀行）</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>その他金融業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2567,7 +2589,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>407</v>
+        <v>934</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2590,10 +2612,10 @@
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="n">
-        <v>86900</v>
+        <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>11624300</v>
+        <v>353800</v>
       </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
@@ -2601,23 +2623,31 @@
       <c r="AI12" t="inlineStr"/>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="n">
-        <v>11624300</v>
-      </c>
-      <c r="AM12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="n">
+        <v>353800</v>
+      </c>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
       <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="n">
-        <v>86900</v>
-      </c>
-      <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>Nomura International plc、モルガン・スタンレーMUFG証券株式会社</t>
+        </is>
+      </c>
+      <c r="AW12" t="n">
+        <v>0.0117</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>110500</v>
+      </c>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
       <c r="BA12" t="inlineStr"/>
@@ -2627,7 +2657,7 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>2212760</v>
+        <v>1582900</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2636,13 +2666,13 @@
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="n">
-        <v>2140650</v>
+        <v>2754150</v>
       </c>
       <c r="BO12" t="n">
-        <v>2212760</v>
+        <v>1582900</v>
       </c>
       <c r="BP12" t="n">
-        <v>938631960</v>
+        <v>1684388100</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2651,10 +2681,10 @@
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="n">
-        <v>932730175</v>
+        <v>2897407950</v>
       </c>
       <c r="BX12" t="n">
-        <v>938631960</v>
+        <v>1684388100</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2662,29 +2692,29 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>548A</t>
+          <t>549A</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>システムエグゼ</t>
+          <t>ヒトトヒトホールディングス</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2699,7 +2729,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>サービス業</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2714,7 +2744,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>966</v>
+        <v>530</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2736,8 +2766,12 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
+      <c r="AD13" t="n">
+        <v>1500</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>867300</v>
+      </c>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr"/>
@@ -2745,7 +2779,9 @@
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
       <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
+      <c r="AM13" t="n">
+        <v>867300</v>
+      </c>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
@@ -2753,17 +2789,19 @@
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="inlineStr"/>
+      <c r="AU13" t="n">
+        <v>1500</v>
+      </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>Nomura International plc、モルガン・スタンレーMUFG証券株式会社</t>
+          <t>野村證券株式会社</t>
         </is>
       </c>
       <c r="AW13" t="n">
-        <v>0.0077</v>
+        <v>0.0375</v>
       </c>
       <c r="AX13" t="n">
-        <v>72800</v>
+        <v>525000</v>
       </c>
       <c r="AY13" t="inlineStr"/>
       <c r="AZ13" t="inlineStr"/>
@@ -2772,9 +2810,11 @@
       <c r="BC13" t="inlineStr"/>
       <c r="BD13" t="inlineStr"/>
       <c r="BE13" t="inlineStr"/>
-      <c r="BF13" t="inlineStr"/>
+      <c r="BF13" t="n">
+        <v>525000</v>
+      </c>
       <c r="BG13" t="n">
-        <v>2177820</v>
+        <v>5546820</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2783,13 +2823,13 @@
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="n">
-        <v>2057900</v>
+        <v>5849500</v>
       </c>
       <c r="BO13" t="n">
-        <v>2177820</v>
+        <v>5546820</v>
       </c>
       <c r="BP13" t="n">
-        <v>2332905800</v>
+        <v>3314988320</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2798,10 +2838,10 @@
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="n">
-        <v>2105307200</v>
+        <v>2571111900</v>
       </c>
       <c r="BX13" t="n">
-        <v>2332905800</v>
+        <v>3314988320</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2809,29 +2849,29 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>549A</t>
+          <t>550A</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ヒトトヒトホールディングス</t>
+          <t>ソフトテックス</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2846,7 +2886,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>サービス業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2861,7 +2901,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>596</v>
+        <v>4515</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -2883,8 +2923,12 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
+      <c r="AD14" t="n">
+        <v>6900</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>78200</v>
+      </c>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
       <c r="AH14" t="inlineStr"/>
@@ -2892,7 +2936,9 @@
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
       <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr"/>
+      <c r="AM14" t="n">
+        <v>78200</v>
+      </c>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
@@ -2900,18 +2946,12 @@
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="inlineStr"/>
-      <c r="AU14" t="inlineStr"/>
-      <c r="AV14" t="inlineStr">
-        <is>
-          <t>野村證券株式会社</t>
-        </is>
-      </c>
-      <c r="AW14" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="AX14" t="n">
-        <v>525000</v>
-      </c>
+      <c r="AU14" t="n">
+        <v>6900</v>
+      </c>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
       <c r="AY14" t="inlineStr"/>
       <c r="AZ14" t="inlineStr"/>
       <c r="BA14" t="inlineStr"/>
@@ -2919,11 +2959,9 @@
       <c r="BC14" t="inlineStr"/>
       <c r="BD14" t="inlineStr"/>
       <c r="BE14" t="inlineStr"/>
-      <c r="BF14" t="n">
-        <v>525000</v>
-      </c>
+      <c r="BF14" t="inlineStr"/>
       <c r="BG14" t="n">
-        <v>6291160</v>
+        <v>475350</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -2933,10 +2971,10 @@
       <c r="BM14" t="inlineStr"/>
       <c r="BN14" t="inlineStr"/>
       <c r="BO14" t="n">
-        <v>6291160</v>
+        <v>475350</v>
       </c>
       <c r="BP14" t="n">
-        <v>3593526160</v>
+        <v>1449007250</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -2946,7 +2984,7 @@
       <c r="BV14" t="inlineStr"/>
       <c r="BW14" t="inlineStr"/>
       <c r="BX14" t="n">
-        <v>3593526160</v>
+        <v>1449007250</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -2954,29 +2992,29 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>550A</t>
+          <t>8301</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ソフトテックス</t>
+          <t>日本銀行</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2986,12 +3024,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>情報通信・サービスその他</t>
+          <t>銀行</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>情報･通信業</t>
+          <t>銀行業</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3006,7 +3044,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>3815</v>
+        <v>25000</v>
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -3058,30 +3096,58 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>631566.6666666666</v>
-      </c>
-      <c r="BH15" t="inlineStr"/>
-      <c r="BI15" t="inlineStr"/>
-      <c r="BJ15" t="inlineStr"/>
-      <c r="BK15" t="inlineStr"/>
-      <c r="BL15" t="inlineStr"/>
-      <c r="BM15" t="inlineStr"/>
-      <c r="BN15" t="inlineStr"/>
+        <v>150</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>300</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>200</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>500</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>260</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>233.3333333333333</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>250</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>250</v>
+      </c>
       <c r="BO15" t="n">
-        <v>631566.6666666666</v>
+        <v>150</v>
       </c>
       <c r="BP15" t="n">
-        <v>1921926166.666667</v>
-      </c>
-      <c r="BQ15" t="inlineStr"/>
-      <c r="BR15" t="inlineStr"/>
-      <c r="BS15" t="inlineStr"/>
-      <c r="BT15" t="inlineStr"/>
-      <c r="BU15" t="inlineStr"/>
-      <c r="BV15" t="inlineStr"/>
-      <c r="BW15" t="inlineStr"/>
+        <v>3735250</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>7920750</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>5100000</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>12464000</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>6487600</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>5785000</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>6204000</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>6186000</v>
+      </c>
       <c r="BX15" t="n">
-        <v>1921926166.666667</v>
+        <v>3735250</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3089,29 +3155,29 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8301</t>
+          <t>9399</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>日本銀行</t>
+          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3121,12 +3187,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>銀行</t>
+          <t>情報通信・サービスその他</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>銀行業</t>
+          <t>情報･通信業</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3141,7 +3207,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>25000</v>
+        <v>30</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3163,24 +3229,60 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
-      <c r="AL16" t="inlineStr"/>
-      <c r="AM16" t="inlineStr"/>
-      <c r="AN16" t="inlineStr"/>
-      <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr"/>
-      <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr"/>
-      <c r="AS16" t="inlineStr"/>
-      <c r="AT16" t="inlineStr"/>
-      <c r="AU16" t="inlineStr"/>
+      <c r="AD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>112008</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>204885</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>97185</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>93675</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>126528</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>99264</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>96080</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>122230</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>112008</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>0</v>
+      </c>
       <c r="AV16" t="inlineStr"/>
       <c r="AW16" t="inlineStr"/>
       <c r="AX16" t="inlineStr"/>
@@ -3193,58 +3295,58 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>166.6666666666667</v>
+        <v>3641893.8</v>
       </c>
       <c r="BH16" t="n">
-        <v>875</v>
+        <v>13641653.6</v>
       </c>
       <c r="BI16" t="n">
-        <v>100</v>
+        <v>4141412.2</v>
       </c>
       <c r="BJ16" t="n">
-        <v>450</v>
+        <v>3244477</v>
       </c>
       <c r="BK16" t="n">
-        <v>300</v>
+        <v>3121484.8</v>
       </c>
       <c r="BL16" t="n">
-        <v>166.6666666666667</v>
+        <v>4791179.2</v>
       </c>
       <c r="BM16" t="n">
-        <v>250</v>
+        <v>1602701</v>
       </c>
       <c r="BN16" t="n">
-        <v>266.6666666666667</v>
+        <v>2038676.2</v>
       </c>
       <c r="BO16" t="n">
-        <v>166.6666666666667</v>
+        <v>3641893.8</v>
       </c>
       <c r="BP16" t="n">
-        <v>4147000</v>
+        <v>106573609</v>
       </c>
       <c r="BQ16" t="n">
-        <v>23735750</v>
+        <v>361089200</v>
       </c>
       <c r="BR16" t="n">
-        <v>2650000</v>
+        <v>112574536.8</v>
       </c>
       <c r="BS16" t="n">
-        <v>11285000</v>
+        <v>89198367.8</v>
       </c>
       <c r="BT16" t="n">
-        <v>7486400</v>
+        <v>91308870.59999999</v>
       </c>
       <c r="BU16" t="n">
-        <v>4104666.666666667</v>
+        <v>152865029.4</v>
       </c>
       <c r="BV16" t="n">
-        <v>6260000</v>
+        <v>47100971.4</v>
       </c>
       <c r="BW16" t="n">
-        <v>6588333.333333333</v>
+        <v>54470723.6</v>
       </c>
       <c r="BX16" t="n">
-        <v>4147000</v>
+        <v>106573609</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3252,212 +3354,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260414-000500</t>
+          <t>20260414-190100</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-13T15:05:00+00:00</t>
+          <t>2026-04-14T10:01:00+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-14T00:05:00+09:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>9399</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ビート・ホールディングス・リミテッド（貝徳控股有限公司）</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>スタンダード</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>情報通信・サービスその他</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>情報･通信業</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>fins_summary_api_fail</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>RuntimeError: empty /fins/summary</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>28</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
-      <c r="AD17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE17" t="n">
-        <v>122230</v>
-      </c>
-      <c r="AF17" t="n">
-        <v>204885</v>
-      </c>
-      <c r="AG17" t="n">
-        <v>97185</v>
-      </c>
-      <c r="AH17" t="n">
-        <v>93675</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>126528</v>
-      </c>
-      <c r="AJ17" t="n">
-        <v>99264</v>
-      </c>
-      <c r="AK17" t="n">
-        <v>96080</v>
-      </c>
-      <c r="AL17" t="n">
-        <v>122230</v>
-      </c>
-      <c r="AM17" t="inlineStr"/>
-      <c r="AN17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU17" t="inlineStr"/>
-      <c r="AV17" t="inlineStr"/>
-      <c r="AW17" t="inlineStr"/>
-      <c r="AX17" t="inlineStr"/>
-      <c r="AY17" t="inlineStr"/>
-      <c r="AZ17" t="inlineStr"/>
-      <c r="BA17" t="inlineStr"/>
-      <c r="BB17" t="inlineStr"/>
-      <c r="BC17" t="inlineStr"/>
-      <c r="BD17" t="inlineStr"/>
-      <c r="BE17" t="inlineStr"/>
-      <c r="BF17" t="inlineStr"/>
-      <c r="BG17" t="n">
-        <v>3463774</v>
-      </c>
-      <c r="BH17" t="n">
-        <v>13931419.2</v>
-      </c>
-      <c r="BI17" t="n">
-        <v>5104435.2</v>
-      </c>
-      <c r="BJ17" t="n">
-        <v>3130213.4</v>
-      </c>
-      <c r="BK17" t="n">
-        <v>3424175.2</v>
-      </c>
-      <c r="BL17" t="n">
-        <v>4747035.2</v>
-      </c>
-      <c r="BM17" t="n">
-        <v>1966370.8</v>
-      </c>
-      <c r="BN17" t="n">
-        <v>1960023.6</v>
-      </c>
-      <c r="BO17" t="n">
-        <v>3463774</v>
-      </c>
-      <c r="BP17" t="n">
-        <v>100737881.8</v>
-      </c>
-      <c r="BQ17" t="n">
-        <v>356289258</v>
-      </c>
-      <c r="BR17" t="n">
-        <v>147240261</v>
-      </c>
-      <c r="BS17" t="n">
-        <v>83366454.8</v>
-      </c>
-      <c r="BT17" t="n">
-        <v>100089101.6</v>
-      </c>
-      <c r="BU17" t="n">
-        <v>150288273.6</v>
-      </c>
-      <c r="BV17" t="n">
-        <v>58329980.2</v>
-      </c>
-      <c r="BW17" t="n">
-        <v>52706922.8</v>
-      </c>
-      <c r="BX17" t="n">
-        <v>100737881.8</v>
-      </c>
-      <c r="BY17" t="inlineStr"/>
-      <c r="BZ17" t="inlineStr"/>
-      <c r="CA17" t="inlineStr"/>
-      <c r="CB17" t="inlineStr"/>
-      <c r="CC17" t="inlineStr">
-        <is>
-          <t>20260414-000500</t>
-        </is>
-      </c>
-      <c r="CD17" t="inlineStr">
-        <is>
-          <t>2026-04-13T15:05:00+00:00</t>
-        </is>
-      </c>
-      <c r="CE17" t="inlineStr">
-        <is>
-          <t>2026-04-14T00:05:00+09:00</t>
+          <t>2026-04-14T19:01:00+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-15
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -971,58 +971,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>16200</v>
+        <v>12400</v>
       </c>
       <c r="BH2" t="n">
-        <v>9600</v>
+        <v>9200</v>
       </c>
       <c r="BI2" t="n">
-        <v>16200</v>
+        <v>17800</v>
       </c>
       <c r="BJ2" t="n">
-        <v>22400</v>
+        <v>21800</v>
       </c>
       <c r="BK2" t="n">
-        <v>14200</v>
+        <v>13200</v>
       </c>
       <c r="BL2" t="n">
-        <v>14000</v>
+        <v>14800</v>
       </c>
       <c r="BM2" t="n">
-        <v>16000</v>
+        <v>14600</v>
       </c>
       <c r="BN2" t="n">
-        <v>26400</v>
+        <v>34400</v>
       </c>
       <c r="BO2" t="n">
-        <v>16200</v>
+        <v>12400</v>
       </c>
       <c r="BP2" t="n">
-        <v>1232000</v>
+        <v>972000</v>
       </c>
       <c r="BQ2" t="n">
-        <v>772000</v>
+        <v>742000</v>
       </c>
       <c r="BR2" t="n">
-        <v>1272800</v>
+        <v>1394000</v>
       </c>
       <c r="BS2" t="n">
-        <v>1628000</v>
+        <v>1567400</v>
       </c>
       <c r="BT2" t="n">
-        <v>993800</v>
+        <v>921000</v>
       </c>
       <c r="BU2" t="n">
-        <v>979400</v>
+        <v>1033200</v>
       </c>
       <c r="BV2" t="n">
-        <v>1072200</v>
+        <v>975800</v>
       </c>
       <c r="BW2" t="n">
-        <v>1869600</v>
+        <v>2473200</v>
       </c>
       <c r="BX2" t="n">
-        <v>1232000</v>
+        <v>972000</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1030,17 +1030,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1170,58 +1170,58 @@
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="n">
-        <v>38680</v>
+        <v>35380</v>
       </c>
       <c r="BH3" t="n">
-        <v>64700</v>
+        <v>66220</v>
       </c>
       <c r="BI3" t="n">
-        <v>59380</v>
+        <v>65160</v>
       </c>
       <c r="BJ3" t="n">
-        <v>77740</v>
+        <v>71700</v>
       </c>
       <c r="BK3" t="n">
-        <v>48480</v>
+        <v>76300</v>
       </c>
       <c r="BL3" t="n">
-        <v>103840</v>
+        <v>71860</v>
       </c>
       <c r="BM3" t="n">
-        <v>33720</v>
+        <v>28740</v>
       </c>
       <c r="BN3" t="n">
-        <v>13980</v>
+        <v>19560</v>
       </c>
       <c r="BO3" t="n">
-        <v>38680</v>
+        <v>35380</v>
       </c>
       <c r="BP3" t="n">
-        <v>8961740</v>
+        <v>8239780</v>
       </c>
       <c r="BQ3" t="n">
-        <v>16438180</v>
+        <v>16615420</v>
       </c>
       <c r="BR3" t="n">
-        <v>14522900</v>
+        <v>15752240</v>
       </c>
       <c r="BS3" t="n">
-        <v>17546800</v>
+        <v>16048700</v>
       </c>
       <c r="BT3" t="n">
-        <v>10831060</v>
+        <v>17525360</v>
       </c>
       <c r="BU3" t="n">
-        <v>24264960</v>
+        <v>16693620</v>
       </c>
       <c r="BV3" t="n">
-        <v>7616900</v>
+        <v>6423760</v>
       </c>
       <c r="BW3" t="n">
-        <v>3137240</v>
+        <v>4404040</v>
       </c>
       <c r="BX3" t="n">
-        <v>8961740</v>
+        <v>8239780</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1229,17 +1229,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1387,54 +1387,58 @@
         <v>0</v>
       </c>
       <c r="BG4" t="n">
-        <v>101180</v>
-      </c>
-      <c r="BH4" t="inlineStr"/>
+        <v>117560</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>2819200</v>
+      </c>
       <c r="BI4" t="n">
-        <v>971220</v>
+        <v>469840</v>
       </c>
       <c r="BJ4" t="n">
-        <v>162400</v>
+        <v>119060</v>
       </c>
       <c r="BK4" t="n">
-        <v>94040</v>
+        <v>101440</v>
       </c>
       <c r="BL4" t="n">
-        <v>125360</v>
+        <v>110180</v>
       </c>
       <c r="BM4" t="n">
-        <v>86440</v>
+        <v>96620</v>
       </c>
       <c r="BN4" t="n">
-        <v>54260</v>
+        <v>49560</v>
       </c>
       <c r="BO4" t="n">
-        <v>101180</v>
+        <v>117560</v>
       </c>
       <c r="BP4" t="n">
-        <v>77627380</v>
-      </c>
-      <c r="BQ4" t="inlineStr"/>
+        <v>86352360</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>3093295700</v>
+      </c>
       <c r="BR4" t="n">
-        <v>1018630620</v>
+        <v>467821240</v>
       </c>
       <c r="BS4" t="n">
-        <v>168932740</v>
+        <v>120823060</v>
       </c>
       <c r="BT4" t="n">
-        <v>98665760</v>
+        <v>106038140</v>
       </c>
       <c r="BU4" t="n">
-        <v>119082120</v>
+        <v>101965460</v>
       </c>
       <c r="BV4" t="n">
-        <v>72462920</v>
+        <v>79752720</v>
       </c>
       <c r="BW4" t="n">
-        <v>44134900</v>
+        <v>41043140</v>
       </c>
       <c r="BX4" t="n">
-        <v>77627380</v>
+        <v>86352360</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1442,17 +1446,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1498,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1562,38 +1566,42 @@
       <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="n">
-        <v>18080</v>
+        <v>16800</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="inlineStr"/>
       <c r="BK5" t="inlineStr"/>
-      <c r="BL5" t="inlineStr"/>
+      <c r="BL5" t="n">
+        <v>800000</v>
+      </c>
       <c r="BM5" t="n">
-        <v>262360</v>
+        <v>116000</v>
       </c>
       <c r="BN5" t="n">
-        <v>28760</v>
+        <v>19780</v>
       </c>
       <c r="BO5" t="n">
-        <v>18080</v>
+        <v>16800</v>
       </c>
       <c r="BP5" t="n">
-        <v>12388760</v>
+        <v>11470660</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="inlineStr"/>
       <c r="BS5" t="inlineStr"/>
       <c r="BT5" t="inlineStr"/>
-      <c r="BU5" t="inlineStr"/>
+      <c r="BU5" t="n">
+        <v>643551400</v>
+      </c>
       <c r="BV5" t="n">
-        <v>202733020</v>
+        <v>83306260</v>
       </c>
       <c r="BW5" t="n">
-        <v>19548000</v>
+        <v>13478760</v>
       </c>
       <c r="BX5" t="n">
-        <v>12388760</v>
+        <v>11470660</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1601,17 +1609,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1661,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>660</v>
+        <v>650</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1721,38 +1729,42 @@
       <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="n">
-        <v>35420</v>
+        <v>33780</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="inlineStr"/>
       <c r="BK6" t="inlineStr"/>
-      <c r="BL6" t="inlineStr"/>
+      <c r="BL6" t="n">
+        <v>989300</v>
+      </c>
       <c r="BM6" t="n">
-        <v>484140</v>
+        <v>313140</v>
       </c>
       <c r="BN6" t="n">
-        <v>96860</v>
+        <v>80500</v>
       </c>
       <c r="BO6" t="n">
-        <v>35420</v>
+        <v>33780</v>
       </c>
       <c r="BP6" t="n">
-        <v>23739800</v>
+        <v>22425580</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="inlineStr"/>
       <c r="BT6" t="inlineStr"/>
-      <c r="BU6" t="inlineStr"/>
+      <c r="BU6" t="n">
+        <v>737786900</v>
+      </c>
       <c r="BV6" t="n">
-        <v>348791500</v>
+        <v>220473800</v>
       </c>
       <c r="BW6" t="n">
-        <v>66866560</v>
+        <v>54726680</v>
       </c>
       <c r="BX6" t="n">
-        <v>23739800</v>
+        <v>22425580</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1760,17 +1772,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1824,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1876,34 +1888,38 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>11416840</v>
+        <v>8132220</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
       <c r="BJ7" t="inlineStr"/>
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
-      <c r="BM7" t="inlineStr"/>
+      <c r="BM7" t="n">
+        <v>10246600</v>
+      </c>
       <c r="BN7" t="n">
-        <v>21773700</v>
+        <v>23838300</v>
       </c>
       <c r="BO7" t="n">
-        <v>11416840</v>
+        <v>8132220</v>
       </c>
       <c r="BP7" t="n">
-        <v>4775020380</v>
+        <v>3336125740</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
-      <c r="BV7" t="inlineStr"/>
+      <c r="BV7" t="n">
+        <v>4296843900</v>
+      </c>
       <c r="BW7" t="n">
-        <v>10269101440</v>
+        <v>11182826880</v>
       </c>
       <c r="BX7" t="n">
-        <v>4775020380</v>
+        <v>3336125740</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -1911,17 +1927,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1979,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2037,34 +2053,38 @@
         <v>379285</v>
       </c>
       <c r="BG8" t="n">
-        <v>156560</v>
+        <v>152080</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
       <c r="BJ8" t="inlineStr"/>
       <c r="BK8" t="inlineStr"/>
       <c r="BL8" t="inlineStr"/>
-      <c r="BM8" t="inlineStr"/>
+      <c r="BM8" t="n">
+        <v>244800</v>
+      </c>
       <c r="BN8" t="n">
-        <v>240660</v>
+        <v>222760</v>
       </c>
       <c r="BO8" t="n">
-        <v>156560</v>
+        <v>152080</v>
       </c>
       <c r="BP8" t="n">
-        <v>64864340</v>
+        <v>62668840</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
       <c r="BS8" t="inlineStr"/>
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
-      <c r="BV8" t="inlineStr"/>
+      <c r="BV8" t="n">
+        <v>102953000</v>
+      </c>
       <c r="BW8" t="n">
-        <v>100115340</v>
+        <v>92551780</v>
       </c>
       <c r="BX8" t="n">
-        <v>64864340</v>
+        <v>62668840</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2072,17 +2092,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2144,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>928</v>
+        <v>938</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2188,34 +2208,38 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>77420</v>
+        <v>55260</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
       <c r="BJ9" t="inlineStr"/>
       <c r="BK9" t="inlineStr"/>
       <c r="BL9" t="inlineStr"/>
-      <c r="BM9" t="inlineStr"/>
+      <c r="BM9" t="n">
+        <v>91400</v>
+      </c>
       <c r="BN9" t="n">
-        <v>167980</v>
+        <v>177860</v>
       </c>
       <c r="BO9" t="n">
-        <v>77420</v>
+        <v>55260</v>
       </c>
       <c r="BP9" t="n">
-        <v>72912260</v>
+        <v>52215820</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
       <c r="BS9" t="inlineStr"/>
       <c r="BT9" t="inlineStr"/>
       <c r="BU9" t="inlineStr"/>
-      <c r="BV9" t="inlineStr"/>
+      <c r="BV9" t="n">
+        <v>81195700</v>
+      </c>
       <c r="BW9" t="n">
-        <v>156119560</v>
+        <v>166188720</v>
       </c>
       <c r="BX9" t="n">
-        <v>72912260</v>
+        <v>52215820</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2223,17 +2247,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2299,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1870</v>
+        <v>1925</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2351,34 +2375,38 @@
         <v>146386</v>
       </c>
       <c r="BG10" t="n">
-        <v>156680</v>
+        <v>145300</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
       <c r="BJ10" t="inlineStr"/>
       <c r="BK10" t="inlineStr"/>
       <c r="BL10" t="inlineStr"/>
-      <c r="BM10" t="inlineStr"/>
+      <c r="BM10" t="n">
+        <v>157200</v>
+      </c>
       <c r="BN10" t="n">
-        <v>181100</v>
+        <v>199220</v>
       </c>
       <c r="BO10" t="n">
-        <v>156680</v>
+        <v>145300</v>
       </c>
       <c r="BP10" t="n">
-        <v>295083620</v>
+        <v>273095260</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
       <c r="BS10" t="inlineStr"/>
       <c r="BT10" t="inlineStr"/>
       <c r="BU10" t="inlineStr"/>
-      <c r="BV10" t="inlineStr"/>
+      <c r="BV10" t="n">
+        <v>278865400</v>
+      </c>
       <c r="BW10" t="n">
-        <v>330671340</v>
+        <v>369146580</v>
       </c>
       <c r="BX10" t="n">
-        <v>295083620</v>
+        <v>273095260</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2386,17 +2414,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2466,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2502,34 +2530,38 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>2388520</v>
+        <v>2321580</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
       <c r="BJ11" t="inlineStr"/>
       <c r="BK11" t="inlineStr"/>
       <c r="BL11" t="inlineStr"/>
-      <c r="BM11" t="inlineStr"/>
+      <c r="BM11" t="n">
+        <v>2383200</v>
+      </c>
       <c r="BN11" t="n">
-        <v>2009960</v>
+        <v>1942060</v>
       </c>
       <c r="BO11" t="n">
-        <v>2388520</v>
+        <v>2321580</v>
       </c>
       <c r="BP11" t="n">
-        <v>1012081120</v>
+        <v>977711240</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
       <c r="BS11" t="inlineStr"/>
       <c r="BT11" t="inlineStr"/>
       <c r="BU11" t="inlineStr"/>
-      <c r="BV11" t="inlineStr"/>
+      <c r="BV11" t="n">
+        <v>1069834200</v>
+      </c>
       <c r="BW11" t="n">
-        <v>871040860</v>
+        <v>837295120</v>
       </c>
       <c r="BX11" t="n">
-        <v>1012081120</v>
+        <v>977711240</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2537,17 +2569,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -2589,7 +2621,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>934</v>
+        <v>943</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2657,7 +2689,7 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>1582900</v>
+        <v>738820</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2666,13 +2698,13 @@
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="n">
-        <v>2754150</v>
+        <v>3354300</v>
       </c>
       <c r="BO12" t="n">
-        <v>1582900</v>
+        <v>738820</v>
       </c>
       <c r="BP12" t="n">
-        <v>1684388100</v>
+        <v>743363920</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2681,10 +2713,10 @@
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="n">
-        <v>2897407950</v>
+        <v>3606050766.666667</v>
       </c>
       <c r="BX12" t="n">
-        <v>1684388100</v>
+        <v>743363920</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2692,17 +2724,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2776,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>530</v>
+        <v>496</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2814,7 +2846,7 @@
         <v>525000</v>
       </c>
       <c r="BG13" t="n">
-        <v>5546820</v>
+        <v>5249680</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2823,13 +2855,13 @@
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="n">
-        <v>5849500</v>
+        <v>4432950</v>
       </c>
       <c r="BO13" t="n">
-        <v>5546820</v>
+        <v>5249680</v>
       </c>
       <c r="BP13" t="n">
-        <v>3314988320</v>
+        <v>3163632980</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2838,10 +2870,10 @@
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="n">
-        <v>2571111900</v>
+        <v>2059503450</v>
       </c>
       <c r="BX13" t="n">
-        <v>3314988320</v>
+        <v>3163632980</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2849,17 +2881,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2933,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>4515</v>
+        <v>4115</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -2961,7 +2993,7 @@
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="inlineStr"/>
       <c r="BG14" t="n">
-        <v>475350</v>
+        <v>545060</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -2971,10 +3003,10 @@
       <c r="BM14" t="inlineStr"/>
       <c r="BN14" t="inlineStr"/>
       <c r="BO14" t="n">
-        <v>475350</v>
+        <v>545060</v>
       </c>
       <c r="BP14" t="n">
-        <v>1449007250</v>
+        <v>1922554100</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -2984,7 +3016,7 @@
       <c r="BV14" t="inlineStr"/>
       <c r="BW14" t="inlineStr"/>
       <c r="BX14" t="n">
-        <v>1449007250</v>
+        <v>1922554100</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -2992,17 +3024,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -3043,9 +3075,7 @@
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="n">
-        <v>25000</v>
-      </c>
+      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
@@ -3096,58 +3126,58 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>150</v>
+        <v>166.6666666666667</v>
       </c>
       <c r="BH15" t="n">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="BI15" t="n">
         <v>200</v>
       </c>
       <c r="BJ15" t="n">
-        <v>500</v>
+        <v>366.6666666666667</v>
       </c>
       <c r="BK15" t="n">
-        <v>260</v>
+        <v>300</v>
       </c>
       <c r="BL15" t="n">
         <v>233.3333333333333</v>
       </c>
       <c r="BM15" t="n">
-        <v>250</v>
+        <v>266.6666666666667</v>
       </c>
       <c r="BN15" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="BO15" t="n">
-        <v>150</v>
+        <v>166.6666666666667</v>
       </c>
       <c r="BP15" t="n">
-        <v>3735250</v>
+        <v>4153666.666666667</v>
       </c>
       <c r="BQ15" t="n">
-        <v>7920750</v>
+        <v>2637666.666666667</v>
       </c>
       <c r="BR15" t="n">
         <v>5100000</v>
       </c>
       <c r="BS15" t="n">
-        <v>12464000</v>
+        <v>9128666.666666666</v>
       </c>
       <c r="BT15" t="n">
-        <v>6487600</v>
+        <v>7495000</v>
       </c>
       <c r="BU15" t="n">
         <v>5785000</v>
       </c>
       <c r="BV15" t="n">
-        <v>6204000</v>
+        <v>6586333.333333333</v>
       </c>
       <c r="BW15" t="n">
-        <v>6186000</v>
+        <v>3750500</v>
       </c>
       <c r="BX15" t="n">
-        <v>3735250</v>
+        <v>4153666.666666667</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3155,17 +3185,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3237,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3295,58 +3325,58 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>3641893.8</v>
+        <v>4097141.2</v>
       </c>
       <c r="BH16" t="n">
-        <v>13641653.6</v>
+        <v>12179098.2</v>
       </c>
       <c r="BI16" t="n">
-        <v>4141412.2</v>
+        <v>3700743.4</v>
       </c>
       <c r="BJ16" t="n">
-        <v>3244477</v>
+        <v>2944529.2</v>
       </c>
       <c r="BK16" t="n">
-        <v>3121484.8</v>
+        <v>3526709.6</v>
       </c>
       <c r="BL16" t="n">
-        <v>4791179.2</v>
+        <v>4273540.8</v>
       </c>
       <c r="BM16" t="n">
-        <v>1602701</v>
+        <v>1520583.8</v>
       </c>
       <c r="BN16" t="n">
-        <v>2038676.2</v>
+        <v>2187308.8</v>
       </c>
       <c r="BO16" t="n">
-        <v>3641893.8</v>
+        <v>4097141.2</v>
       </c>
       <c r="BP16" t="n">
-        <v>106573609</v>
+        <v>122073693.6</v>
       </c>
       <c r="BQ16" t="n">
-        <v>361089200</v>
+        <v>342936198.6</v>
       </c>
       <c r="BR16" t="n">
-        <v>112574536.8</v>
+        <v>97185042.40000001</v>
       </c>
       <c r="BS16" t="n">
-        <v>89198367.8</v>
+        <v>82702191</v>
       </c>
       <c r="BT16" t="n">
-        <v>91308870.59999999</v>
+        <v>103461676.8</v>
       </c>
       <c r="BU16" t="n">
-        <v>152865029.4</v>
+        <v>138019536.4</v>
       </c>
       <c r="BV16" t="n">
-        <v>47100971.4</v>
+        <v>43926478</v>
       </c>
       <c r="BW16" t="n">
-        <v>54470723.6</v>
+        <v>58501407.4</v>
       </c>
       <c r="BX16" t="n">
-        <v>106573609</v>
+        <v>122073693.6</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3354,17 +3384,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260415-000339</t>
+          <t>20260415-163904</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-14T15:03:39+00:00</t>
+          <t>2026-04-15T07:39:04+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-15T00:03:39+09:00</t>
+          <t>2026-04-15T16:39:04+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-16
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -971,58 +971,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>12400</v>
+        <v>13000</v>
       </c>
       <c r="BH2" t="n">
-        <v>9200</v>
+        <v>12200</v>
       </c>
       <c r="BI2" t="n">
-        <v>17800</v>
+        <v>14800</v>
       </c>
       <c r="BJ2" t="n">
-        <v>21800</v>
+        <v>22000</v>
       </c>
       <c r="BK2" t="n">
-        <v>13200</v>
+        <v>14600</v>
       </c>
       <c r="BL2" t="n">
-        <v>14800</v>
+        <v>12600</v>
       </c>
       <c r="BM2" t="n">
-        <v>14600</v>
+        <v>19600</v>
       </c>
       <c r="BN2" t="n">
-        <v>34400</v>
+        <v>29400</v>
       </c>
       <c r="BO2" t="n">
-        <v>12400</v>
+        <v>13000</v>
       </c>
       <c r="BP2" t="n">
-        <v>972000</v>
+        <v>1022200</v>
       </c>
       <c r="BQ2" t="n">
-        <v>742000</v>
+        <v>979000</v>
       </c>
       <c r="BR2" t="n">
-        <v>1394000</v>
+        <v>1153000</v>
       </c>
       <c r="BS2" t="n">
-        <v>1567400</v>
+        <v>1572800</v>
       </c>
       <c r="BT2" t="n">
-        <v>921000</v>
+        <v>1021400</v>
       </c>
       <c r="BU2" t="n">
-        <v>1033200</v>
+        <v>873200</v>
       </c>
       <c r="BV2" t="n">
-        <v>975800</v>
+        <v>1322400</v>
       </c>
       <c r="BW2" t="n">
-        <v>2473200</v>
+        <v>2134200</v>
       </c>
       <c r="BX2" t="n">
-        <v>972000</v>
+        <v>1022200</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1030,17 +1030,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1170,58 +1170,58 @@
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="n">
-        <v>35380</v>
+        <v>37000</v>
       </c>
       <c r="BH3" t="n">
-        <v>66220</v>
+        <v>68220</v>
       </c>
       <c r="BI3" t="n">
-        <v>65160</v>
+        <v>72660</v>
       </c>
       <c r="BJ3" t="n">
-        <v>71700</v>
+        <v>54760</v>
       </c>
       <c r="BK3" t="n">
-        <v>76300</v>
+        <v>79640</v>
       </c>
       <c r="BL3" t="n">
-        <v>71860</v>
+        <v>65180</v>
       </c>
       <c r="BM3" t="n">
-        <v>28740</v>
+        <v>28680</v>
       </c>
       <c r="BN3" t="n">
-        <v>19560</v>
+        <v>17240</v>
       </c>
       <c r="BO3" t="n">
-        <v>35380</v>
+        <v>37000</v>
       </c>
       <c r="BP3" t="n">
-        <v>8239780</v>
+        <v>8618280</v>
       </c>
       <c r="BQ3" t="n">
-        <v>16615420</v>
+        <v>16851020</v>
       </c>
       <c r="BR3" t="n">
-        <v>15752240</v>
+        <v>17113740</v>
       </c>
       <c r="BS3" t="n">
-        <v>16048700</v>
+        <v>12314000</v>
       </c>
       <c r="BT3" t="n">
-        <v>17525360</v>
+        <v>18335000</v>
       </c>
       <c r="BU3" t="n">
-        <v>16693620</v>
+        <v>15121560</v>
       </c>
       <c r="BV3" t="n">
-        <v>6423760</v>
+        <v>6394280</v>
       </c>
       <c r="BW3" t="n">
-        <v>4404040</v>
+        <v>3875160</v>
       </c>
       <c r="BX3" t="n">
-        <v>8239780</v>
+        <v>8618280</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1229,17 +1229,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>707</v>
+        <v>682</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1387,58 +1387,58 @@
         <v>0</v>
       </c>
       <c r="BG4" t="n">
-        <v>117560</v>
+        <v>121000</v>
       </c>
       <c r="BH4" t="n">
-        <v>2819200</v>
+        <v>1685750</v>
       </c>
       <c r="BI4" t="n">
-        <v>469840</v>
+        <v>386680</v>
       </c>
       <c r="BJ4" t="n">
-        <v>119060</v>
+        <v>112920</v>
       </c>
       <c r="BK4" t="n">
-        <v>101440</v>
+        <v>103520</v>
       </c>
       <c r="BL4" t="n">
-        <v>110180</v>
+        <v>101680</v>
       </c>
       <c r="BM4" t="n">
-        <v>96620</v>
+        <v>93360</v>
       </c>
       <c r="BN4" t="n">
-        <v>49560</v>
+        <v>59880</v>
       </c>
       <c r="BO4" t="n">
-        <v>117560</v>
+        <v>121000</v>
       </c>
       <c r="BP4" t="n">
-        <v>86352360</v>
+        <v>86568060</v>
       </c>
       <c r="BQ4" t="n">
-        <v>3093295700</v>
+        <v>1822441950</v>
       </c>
       <c r="BR4" t="n">
-        <v>467821240</v>
+        <v>385590560</v>
       </c>
       <c r="BS4" t="n">
-        <v>120823060</v>
+        <v>114817520</v>
       </c>
       <c r="BT4" t="n">
-        <v>106038140</v>
+        <v>107356060</v>
       </c>
       <c r="BU4" t="n">
-        <v>101965460</v>
+        <v>91259340</v>
       </c>
       <c r="BV4" t="n">
-        <v>79752720</v>
+        <v>76451260</v>
       </c>
       <c r="BW4" t="n">
-        <v>41043140</v>
+        <v>48844340</v>
       </c>
       <c r="BX4" t="n">
-        <v>86352360</v>
+        <v>86568060</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1446,17 +1446,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1566,42 +1566,42 @@
       <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="n">
-        <v>16800</v>
+        <v>18880</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="inlineStr"/>
       <c r="BK5" t="inlineStr"/>
       <c r="BL5" t="n">
-        <v>800000</v>
+        <v>494650</v>
       </c>
       <c r="BM5" t="n">
-        <v>116000</v>
+        <v>81840</v>
       </c>
       <c r="BN5" t="n">
-        <v>19780</v>
+        <v>19340</v>
       </c>
       <c r="BO5" t="n">
-        <v>16800</v>
+        <v>18880</v>
       </c>
       <c r="BP5" t="n">
-        <v>11470660</v>
+        <v>12876700</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="inlineStr"/>
       <c r="BS5" t="inlineStr"/>
       <c r="BT5" t="inlineStr"/>
       <c r="BU5" t="n">
-        <v>643551400</v>
+        <v>394376800</v>
       </c>
       <c r="BV5" t="n">
-        <v>83306260</v>
+        <v>56793080</v>
       </c>
       <c r="BW5" t="n">
-        <v>13478760</v>
+        <v>13185240</v>
       </c>
       <c r="BX5" t="n">
-        <v>11470660</v>
+        <v>12876700</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1609,17 +1609,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>650</v>
+        <v>639</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1729,42 +1729,42 @@
       <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="n">
-        <v>33780</v>
+        <v>41880</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="inlineStr"/>
       <c r="BK6" t="inlineStr"/>
       <c r="BL6" t="n">
-        <v>989300</v>
+        <v>662250</v>
       </c>
       <c r="BM6" t="n">
-        <v>313140</v>
+        <v>268820</v>
       </c>
       <c r="BN6" t="n">
-        <v>80500</v>
+        <v>63160</v>
       </c>
       <c r="BO6" t="n">
-        <v>33780</v>
+        <v>41880</v>
       </c>
       <c r="BP6" t="n">
-        <v>22425580</v>
+        <v>27433920</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="inlineStr"/>
       <c r="BT6" t="inlineStr"/>
       <c r="BU6" t="n">
-        <v>737786900</v>
+        <v>486764000</v>
       </c>
       <c r="BV6" t="n">
-        <v>220473800</v>
+        <v>189029760</v>
       </c>
       <c r="BW6" t="n">
-        <v>54726680</v>
+        <v>42663760</v>
       </c>
       <c r="BX6" t="n">
-        <v>22425580</v>
+        <v>27433920</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1772,17 +1772,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1896,7 +1896,7 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="n">
-        <v>8132220</v>
+        <v>7053860</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1904,16 +1904,16 @@
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="n">
-        <v>10246600</v>
+        <v>10922450</v>
       </c>
       <c r="BN7" t="n">
-        <v>23838300</v>
+        <v>24024360</v>
       </c>
       <c r="BO7" t="n">
-        <v>8132220</v>
+        <v>7053860</v>
       </c>
       <c r="BP7" t="n">
-        <v>3336125740</v>
+        <v>2864719100</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
@@ -1921,13 +1921,13 @@
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="n">
-        <v>4296843900</v>
+        <v>4758047550</v>
       </c>
       <c r="BW7" t="n">
-        <v>11182826880</v>
+        <v>11174434740</v>
       </c>
       <c r="BX7" t="n">
-        <v>3336125740</v>
+        <v>2864719100</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -1935,17 +1935,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>408</v>
+        <v>414</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2061,7 +2061,7 @@
         <v>379285</v>
       </c>
       <c r="BG8" t="n">
-        <v>152080</v>
+        <v>159720</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
@@ -2069,16 +2069,16 @@
       <c r="BK8" t="inlineStr"/>
       <c r="BL8" t="inlineStr"/>
       <c r="BM8" t="n">
-        <v>244800</v>
+        <v>247150</v>
       </c>
       <c r="BN8" t="n">
-        <v>222760</v>
+        <v>201040</v>
       </c>
       <c r="BO8" t="n">
-        <v>152080</v>
+        <v>159720</v>
       </c>
       <c r="BP8" t="n">
-        <v>62668840</v>
+        <v>65665880</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
@@ -2086,13 +2086,13 @@
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="n">
-        <v>102953000</v>
+        <v>102748250</v>
       </c>
       <c r="BW8" t="n">
-        <v>92551780</v>
+        <v>83837520</v>
       </c>
       <c r="BX8" t="n">
-        <v>62668840</v>
+        <v>65665880</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2100,17 +2100,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2152,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>938</v>
+        <v>929</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2216,7 +2216,7 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>55260</v>
+        <v>45760</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
@@ -2224,16 +2224,16 @@
       <c r="BK9" t="inlineStr"/>
       <c r="BL9" t="inlineStr"/>
       <c r="BM9" t="n">
-        <v>91400</v>
+        <v>155450</v>
       </c>
       <c r="BN9" t="n">
-        <v>177860</v>
+        <v>150280</v>
       </c>
       <c r="BO9" t="n">
-        <v>55260</v>
+        <v>45760</v>
       </c>
       <c r="BP9" t="n">
-        <v>52215820</v>
+        <v>43020500</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
@@ -2241,13 +2241,13 @@
       <c r="BT9" t="inlineStr"/>
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="n">
-        <v>81195700</v>
+        <v>144927050</v>
       </c>
       <c r="BW9" t="n">
-        <v>166188720</v>
+        <v>140007220</v>
       </c>
       <c r="BX9" t="n">
-        <v>52215820</v>
+        <v>43020500</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2255,17 +2255,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2307,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1925</v>
+        <v>1962</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2383,7 +2383,7 @@
         <v>146386</v>
       </c>
       <c r="BG10" t="n">
-        <v>145300</v>
+        <v>164860</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2391,16 +2391,16 @@
       <c r="BK10" t="inlineStr"/>
       <c r="BL10" t="inlineStr"/>
       <c r="BM10" t="n">
-        <v>157200</v>
+        <v>195250</v>
       </c>
       <c r="BN10" t="n">
-        <v>199220</v>
+        <v>184180</v>
       </c>
       <c r="BO10" t="n">
-        <v>145300</v>
+        <v>164860</v>
       </c>
       <c r="BP10" t="n">
-        <v>273095260</v>
+        <v>314149400</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2408,13 +2408,13 @@
       <c r="BT10" t="inlineStr"/>
       <c r="BU10" t="inlineStr"/>
       <c r="BV10" t="n">
-        <v>278865400</v>
+        <v>351530650</v>
       </c>
       <c r="BW10" t="n">
-        <v>369146580</v>
+        <v>343918960</v>
       </c>
       <c r="BX10" t="n">
-        <v>273095260</v>
+        <v>314149400</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2422,17 +2422,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2538,7 +2538,7 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>2321580</v>
+        <v>2531780</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2546,16 +2546,16 @@
       <c r="BK11" t="inlineStr"/>
       <c r="BL11" t="inlineStr"/>
       <c r="BM11" t="n">
-        <v>2383200</v>
+        <v>2210850</v>
       </c>
       <c r="BN11" t="n">
-        <v>1942060</v>
+        <v>1845660</v>
       </c>
       <c r="BO11" t="n">
-        <v>2321580</v>
+        <v>2531780</v>
       </c>
       <c r="BP11" t="n">
-        <v>977711240</v>
+        <v>1073563280</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2563,13 +2563,13 @@
       <c r="BT11" t="inlineStr"/>
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="n">
-        <v>1069834200</v>
+        <v>984957200</v>
       </c>
       <c r="BW11" t="n">
-        <v>837295120</v>
+        <v>791971060</v>
       </c>
       <c r="BX11" t="n">
-        <v>977711240</v>
+        <v>1073563280</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2577,17 +2577,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>943</v>
+        <v>1009</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2679,14 +2679,14 @@
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>モルガン・スタンレーMUFG証券株式会社、Jump Trading Pacific Pte Ltd、Nomura International plc</t>
+          <t>モルガン・スタンレーMUFG証券株式会社、Nomura International plc、Jump Trading Pacific Pte Ltd</t>
         </is>
       </c>
       <c r="AW12" t="n">
-        <v>0.0264</v>
+        <v>0.0398</v>
       </c>
       <c r="AX12" t="n">
-        <v>224100</v>
+        <v>293100</v>
       </c>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
@@ -2697,7 +2697,7 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="n">
-        <v>738820</v>
+        <v>543420</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2706,13 +2706,13 @@
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="n">
-        <v>3354300</v>
+        <v>2872425</v>
       </c>
       <c r="BO12" t="n">
-        <v>738820</v>
+        <v>543420</v>
       </c>
       <c r="BP12" t="n">
-        <v>743363920</v>
+        <v>530125660</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2721,10 +2721,10 @@
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="n">
-        <v>3606050766.666667</v>
+        <v>3084106450</v>
       </c>
       <c r="BX12" t="n">
-        <v>743363920</v>
+        <v>530125660</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2732,17 +2732,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>496</v>
+        <v>467</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2834,14 +2834,14 @@
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>野村證券株式会社</t>
+          <t>野村證券株式会社、Nomura International plc</t>
         </is>
       </c>
       <c r="AW13" t="n">
         <v>0.0375</v>
       </c>
       <c r="AX13" t="n">
-        <v>525000</v>
+        <v>766300</v>
       </c>
       <c r="AY13" t="inlineStr"/>
       <c r="AZ13" t="inlineStr"/>
@@ -2854,7 +2854,7 @@
         <v>525000</v>
       </c>
       <c r="BG13" t="n">
-        <v>5249680</v>
+        <v>5339820</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2863,13 +2863,13 @@
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="n">
-        <v>4432950</v>
+        <v>3251933.333333333</v>
       </c>
       <c r="BO13" t="n">
-        <v>5249680</v>
+        <v>5339820</v>
       </c>
       <c r="BP13" t="n">
-        <v>3163632980</v>
+        <v>3184952700</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2878,10 +2878,10 @@
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="n">
-        <v>2059503450</v>
+        <v>1553883300</v>
       </c>
       <c r="BX13" t="n">
-        <v>3163632980</v>
+        <v>3184952700</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2889,17 +2889,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>4115</v>
+        <v>3835</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -3001,7 +3001,7 @@
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="inlineStr"/>
       <c r="BG14" t="n">
-        <v>545060</v>
+        <v>390100</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -3009,12 +3009,14 @@
       <c r="BK14" t="inlineStr"/>
       <c r="BL14" t="inlineStr"/>
       <c r="BM14" t="inlineStr"/>
-      <c r="BN14" t="inlineStr"/>
+      <c r="BN14" t="n">
+        <v>1185300</v>
+      </c>
       <c r="BO14" t="n">
-        <v>545060</v>
+        <v>390100</v>
       </c>
       <c r="BP14" t="n">
-        <v>1922554100</v>
+        <v>1547782700</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -3022,9 +3024,11 @@
       <c r="BT14" t="inlineStr"/>
       <c r="BU14" t="inlineStr"/>
       <c r="BV14" t="inlineStr"/>
-      <c r="BW14" t="inlineStr"/>
+      <c r="BW14" t="n">
+        <v>3532839500</v>
+      </c>
       <c r="BX14" t="n">
-        <v>1922554100</v>
+        <v>1547782700</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -3032,17 +3036,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -3140,19 +3144,19 @@
         <v>100</v>
       </c>
       <c r="BI15" t="n">
-        <v>200</v>
+        <v>450</v>
       </c>
       <c r="BJ15" t="n">
-        <v>366.6666666666667</v>
+        <v>166.6666666666667</v>
       </c>
       <c r="BK15" t="n">
-        <v>300</v>
+        <v>325</v>
       </c>
       <c r="BL15" t="n">
         <v>233.3333333333333</v>
       </c>
       <c r="BM15" t="n">
-        <v>266.6666666666667</v>
+        <v>300</v>
       </c>
       <c r="BN15" t="n">
         <v>150</v>
@@ -3164,22 +3168,22 @@
         <v>4153666.666666667</v>
       </c>
       <c r="BQ15" t="n">
-        <v>2637666.666666667</v>
+        <v>2645000</v>
       </c>
       <c r="BR15" t="n">
-        <v>5100000</v>
+        <v>11285000</v>
       </c>
       <c r="BS15" t="n">
-        <v>9128666.666666666</v>
+        <v>4161000</v>
       </c>
       <c r="BT15" t="n">
-        <v>7495000</v>
+        <v>8085750</v>
       </c>
       <c r="BU15" t="n">
-        <v>5785000</v>
+        <v>5813333.333333333</v>
       </c>
       <c r="BV15" t="n">
-        <v>6586333.333333333</v>
+        <v>7372000</v>
       </c>
       <c r="BW15" t="n">
         <v>3750500</v>
@@ -3193,17 +3197,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -3333,58 +3337,58 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>4097141.2</v>
+        <v>4111983.8</v>
       </c>
       <c r="BH16" t="n">
-        <v>12179098.2</v>
+        <v>9570452.800000001</v>
       </c>
       <c r="BI16" t="n">
-        <v>3700743.4</v>
+        <v>3267717.4</v>
       </c>
       <c r="BJ16" t="n">
-        <v>2944529.2</v>
+        <v>3674551.2</v>
       </c>
       <c r="BK16" t="n">
-        <v>3526709.6</v>
+        <v>4241035.4</v>
       </c>
       <c r="BL16" t="n">
-        <v>4273540.8</v>
+        <v>3010975.8</v>
       </c>
       <c r="BM16" t="n">
-        <v>1520583.8</v>
+        <v>1764609.6</v>
       </c>
       <c r="BN16" t="n">
-        <v>2187308.8</v>
+        <v>1690468.6</v>
       </c>
       <c r="BO16" t="n">
-        <v>4097141.2</v>
+        <v>4111983.8</v>
       </c>
       <c r="BP16" t="n">
-        <v>122073693.6</v>
+        <v>124253885.4</v>
       </c>
       <c r="BQ16" t="n">
-        <v>342936198.6</v>
+        <v>292344615.4</v>
       </c>
       <c r="BR16" t="n">
-        <v>97185042.40000001</v>
+        <v>83737882</v>
       </c>
       <c r="BS16" t="n">
-        <v>82702191</v>
+        <v>107086813.6</v>
       </c>
       <c r="BT16" t="n">
-        <v>103461676.8</v>
+        <v>131265781.6</v>
       </c>
       <c r="BU16" t="n">
-        <v>138019536.4</v>
+        <v>92793402.59999999</v>
       </c>
       <c r="BV16" t="n">
-        <v>43926478</v>
+        <v>48812478.4</v>
       </c>
       <c r="BW16" t="n">
-        <v>58501407.4</v>
+        <v>45282081.2</v>
       </c>
       <c r="BX16" t="n">
-        <v>122073693.6</v>
+        <v>124253885.4</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3392,17 +3396,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260415-235445</t>
+          <t>20260416-190053</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-15T14:54:45+00:00</t>
+          <t>2026-04-16T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-15T23:54:45+09:00</t>
+          <t>2026-04-16T19:00:53+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-17
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -883,7 +883,7 @@
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -912,29 +912,27 @@
         <v>30000</v>
       </c>
       <c r="AF2" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="AG2" t="n">
-        <v>16000</v>
+        <v>33000</v>
       </c>
       <c r="AH2" t="n">
-        <v>33000</v>
+        <v>45000</v>
       </c>
       <c r="AI2" t="n">
-        <v>45000</v>
+        <v>46000</v>
       </c>
       <c r="AJ2" t="n">
-        <v>46000</v>
+        <v>43000</v>
       </c>
       <c r="AK2" t="n">
-        <v>43000</v>
+        <v>31000</v>
       </c>
       <c r="AL2" t="n">
-        <v>31000</v>
-      </c>
-      <c r="AM2" t="n">
         <v>30000</v>
       </c>
+      <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="n">
         <v>0</v>
       </c>
@@ -956,9 +954,7 @@
       <c r="AT2" t="n">
         <v>0</v>
       </c>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU2" t="inlineStr"/>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
@@ -971,58 +967,58 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="n">
-        <v>13000</v>
+        <v>14800</v>
       </c>
       <c r="BH2" t="n">
-        <v>12200</v>
+        <v>13400</v>
       </c>
       <c r="BI2" t="n">
         <v>14800</v>
       </c>
       <c r="BJ2" t="n">
-        <v>22000</v>
+        <v>22800</v>
       </c>
       <c r="BK2" t="n">
-        <v>14600</v>
+        <v>14000</v>
       </c>
       <c r="BL2" t="n">
-        <v>12600</v>
+        <v>13800</v>
       </c>
       <c r="BM2" t="n">
+        <v>27200</v>
+      </c>
+      <c r="BN2" t="n">
         <v>19600</v>
       </c>
-      <c r="BN2" t="n">
-        <v>29400</v>
-      </c>
       <c r="BO2" t="n">
-        <v>13000</v>
+        <v>14800</v>
       </c>
       <c r="BP2" t="n">
-        <v>1022200</v>
+        <v>1166000</v>
       </c>
       <c r="BQ2" t="n">
-        <v>979000</v>
+        <v>1074800</v>
       </c>
       <c r="BR2" t="n">
-        <v>1153000</v>
+        <v>1151800</v>
       </c>
       <c r="BS2" t="n">
-        <v>1572800</v>
+        <v>1615200</v>
       </c>
       <c r="BT2" t="n">
-        <v>1021400</v>
+        <v>981400</v>
       </c>
       <c r="BU2" t="n">
-        <v>873200</v>
+        <v>947600</v>
       </c>
       <c r="BV2" t="n">
-        <v>1322400</v>
+        <v>1862000</v>
       </c>
       <c r="BW2" t="n">
-        <v>2134200</v>
+        <v>1452600</v>
       </c>
       <c r="BX2" t="n">
-        <v>1022200</v>
+        <v>1166000</v>
       </c>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr"/>
@@ -1030,17 +1026,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1078,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
@@ -1111,29 +1107,27 @@
         <v>78200</v>
       </c>
       <c r="AF3" t="n">
-        <v>57400</v>
+        <v>57100</v>
       </c>
       <c r="AG3" t="n">
-        <v>57100</v>
+        <v>57700</v>
       </c>
       <c r="AH3" t="n">
-        <v>57700</v>
+        <v>78800</v>
       </c>
       <c r="AI3" t="n">
-        <v>78800</v>
+        <v>80100</v>
       </c>
       <c r="AJ3" t="n">
-        <v>80100</v>
+        <v>76600</v>
       </c>
       <c r="AK3" t="n">
-        <v>76600</v>
+        <v>76800</v>
       </c>
       <c r="AL3" t="n">
-        <v>76800</v>
-      </c>
-      <c r="AM3" t="n">
         <v>78200</v>
       </c>
+      <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="n">
         <v>0</v>
       </c>
@@ -1155,9 +1149,7 @@
       <c r="AT3" t="n">
         <v>0</v>
       </c>
-      <c r="AU3" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU3" t="inlineStr"/>
       <c r="AV3" t="inlineStr"/>
       <c r="AW3" t="inlineStr"/>
       <c r="AX3" t="inlineStr"/>
@@ -1170,58 +1162,58 @@
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="n">
-        <v>37000</v>
+        <v>35260</v>
       </c>
       <c r="BH3" t="n">
-        <v>68220</v>
+        <v>59380</v>
       </c>
       <c r="BI3" t="n">
-        <v>72660</v>
+        <v>68320</v>
       </c>
       <c r="BJ3" t="n">
-        <v>54760</v>
+        <v>58860</v>
       </c>
       <c r="BK3" t="n">
-        <v>79640</v>
+        <v>79320</v>
       </c>
       <c r="BL3" t="n">
-        <v>65180</v>
+        <v>63700</v>
       </c>
       <c r="BM3" t="n">
-        <v>28680</v>
+        <v>26220</v>
       </c>
       <c r="BN3" t="n">
-        <v>17240</v>
+        <v>18480</v>
       </c>
       <c r="BO3" t="n">
-        <v>37000</v>
+        <v>35260</v>
       </c>
       <c r="BP3" t="n">
-        <v>8618280</v>
+        <v>8229800</v>
       </c>
       <c r="BQ3" t="n">
-        <v>16851020</v>
+        <v>14569660</v>
       </c>
       <c r="BR3" t="n">
-        <v>17113740</v>
+        <v>15978460</v>
       </c>
       <c r="BS3" t="n">
-        <v>12314000</v>
+        <v>13221880</v>
       </c>
       <c r="BT3" t="n">
-        <v>18335000</v>
+        <v>18258940</v>
       </c>
       <c r="BU3" t="n">
-        <v>15121560</v>
+        <v>14797380</v>
       </c>
       <c r="BV3" t="n">
-        <v>6394280</v>
+        <v>5820080</v>
       </c>
       <c r="BW3" t="n">
-        <v>3875160</v>
+        <v>4174480</v>
       </c>
       <c r="BX3" t="n">
-        <v>8618280</v>
+        <v>8229800</v>
       </c>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr"/>
@@ -1229,17 +1221,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1273,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>682</v>
+        <v>722</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
@@ -1309,29 +1301,31 @@
       <c r="AE4" t="n">
         <v>246800</v>
       </c>
-      <c r="AF4" t="inlineStr"/>
+      <c r="AF4" t="n">
+        <v>222300</v>
+      </c>
       <c r="AG4" t="n">
-        <v>222300</v>
+        <v>216400</v>
       </c>
       <c r="AH4" t="n">
-        <v>216400</v>
+        <v>204600</v>
       </c>
       <c r="AI4" t="n">
-        <v>204600</v>
+        <v>212600</v>
       </c>
       <c r="AJ4" t="n">
-        <v>212600</v>
+        <v>227900</v>
       </c>
       <c r="AK4" t="n">
-        <v>227900</v>
+        <v>234400</v>
       </c>
       <c r="AL4" t="n">
-        <v>234400</v>
-      </c>
-      <c r="AM4" t="n">
         <v>246800</v>
       </c>
-      <c r="AN4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="n">
+        <v>0</v>
+      </c>
       <c r="AO4" t="n">
         <v>0</v>
       </c>
@@ -1342,17 +1336,15 @@
         <v>0</v>
       </c>
       <c r="AR4" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="AS4" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="AT4" t="n">
         <v>0</v>
       </c>
-      <c r="AU4" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr">
         <is>
           <t>野村證券株式会社</t>
@@ -1364,18 +1356,20 @@
       <c r="AX4" t="n">
         <v>0</v>
       </c>
-      <c r="AY4" t="inlineStr"/>
+      <c r="AY4" t="n">
+        <v>2482900</v>
+      </c>
       <c r="AZ4" t="n">
-        <v>2482900</v>
+        <v>1080200</v>
       </c>
       <c r="BA4" t="n">
         <v>1080200</v>
       </c>
       <c r="BB4" t="n">
-        <v>1080200</v>
+        <v>1041600</v>
       </c>
       <c r="BC4" t="n">
-        <v>1041600</v>
+        <v>0</v>
       </c>
       <c r="BD4" t="n">
         <v>0</v>
@@ -1387,58 +1381,58 @@
         <v>0</v>
       </c>
       <c r="BG4" t="n">
-        <v>121000</v>
+        <v>112320</v>
       </c>
       <c r="BH4" t="n">
-        <v>1685750</v>
+        <v>1302366.666666667</v>
       </c>
       <c r="BI4" t="n">
-        <v>386680</v>
+        <v>300260</v>
       </c>
       <c r="BJ4" t="n">
-        <v>112920</v>
+        <v>111260</v>
       </c>
       <c r="BK4" t="n">
-        <v>103520</v>
+        <v>117620</v>
       </c>
       <c r="BL4" t="n">
-        <v>101680</v>
+        <v>86180</v>
       </c>
       <c r="BM4" t="n">
-        <v>93360</v>
+        <v>82320</v>
       </c>
       <c r="BN4" t="n">
-        <v>59880</v>
+        <v>76980</v>
       </c>
       <c r="BO4" t="n">
-        <v>121000</v>
+        <v>112320</v>
       </c>
       <c r="BP4" t="n">
-        <v>86568060</v>
+        <v>79143060</v>
       </c>
       <c r="BQ4" t="n">
-        <v>1822441950</v>
+        <v>1383993266.666667</v>
       </c>
       <c r="BR4" t="n">
-        <v>385590560</v>
+        <v>305469720</v>
       </c>
       <c r="BS4" t="n">
-        <v>114817520</v>
+        <v>113793920</v>
       </c>
       <c r="BT4" t="n">
-        <v>107356060</v>
+        <v>118662180</v>
       </c>
       <c r="BU4" t="n">
-        <v>91259340</v>
+        <v>74449720</v>
       </c>
       <c r="BV4" t="n">
-        <v>76451260</v>
+        <v>67033160</v>
       </c>
       <c r="BW4" t="n">
-        <v>48844340</v>
+        <v>61452380</v>
       </c>
       <c r="BX4" t="n">
-        <v>86568060</v>
+        <v>79143060</v>
       </c>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr"/>
@@ -1446,17 +1440,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1492,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>683</v>
+        <v>677</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -1530,30 +1524,30 @@
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
+      <c r="AJ5" t="n">
+        <v>49900</v>
+      </c>
       <c r="AK5" t="n">
-        <v>49900</v>
+        <v>56200</v>
       </c>
       <c r="AL5" t="n">
-        <v>56200</v>
-      </c>
-      <c r="AM5" t="n">
         <v>59600</v>
       </c>
+      <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
+      <c r="AR5" t="n">
+        <v>0</v>
+      </c>
       <c r="AS5" t="n">
         <v>0</v>
       </c>
       <c r="AT5" t="n">
         <v>0</v>
       </c>
-      <c r="AU5" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr"/>
       <c r="AW5" t="inlineStr"/>
       <c r="AX5" t="inlineStr"/>
@@ -1566,42 +1560,42 @@
       <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="n">
-        <v>18880</v>
+        <v>24520</v>
       </c>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="inlineStr"/>
       <c r="BK5" t="inlineStr"/>
       <c r="BL5" t="n">
-        <v>494650</v>
+        <v>406400</v>
       </c>
       <c r="BM5" t="n">
-        <v>81840</v>
+        <v>38440</v>
       </c>
       <c r="BN5" t="n">
-        <v>19340</v>
+        <v>20400</v>
       </c>
       <c r="BO5" t="n">
-        <v>18880</v>
+        <v>24520</v>
       </c>
       <c r="BP5" t="n">
-        <v>12876700</v>
+        <v>16635960</v>
       </c>
       <c r="BQ5" t="inlineStr"/>
       <c r="BR5" t="inlineStr"/>
       <c r="BS5" t="inlineStr"/>
       <c r="BT5" t="inlineStr"/>
       <c r="BU5" t="n">
-        <v>394376800</v>
+        <v>316942333.3333333</v>
       </c>
       <c r="BV5" t="n">
-        <v>56793080</v>
+        <v>26133940</v>
       </c>
       <c r="BW5" t="n">
-        <v>13185240</v>
+        <v>13911860</v>
       </c>
       <c r="BX5" t="n">
-        <v>12876700</v>
+        <v>16635960</v>
       </c>
       <c r="BY5" t="inlineStr"/>
       <c r="BZ5" t="inlineStr"/>
@@ -1609,17 +1603,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1655,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
@@ -1693,30 +1687,30 @@
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
       <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
+      <c r="AJ6" t="n">
+        <v>70700</v>
+      </c>
       <c r="AK6" t="n">
-        <v>70700</v>
+        <v>106000</v>
       </c>
       <c r="AL6" t="n">
-        <v>106000</v>
-      </c>
-      <c r="AM6" t="n">
         <v>181100</v>
       </c>
+      <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
       <c r="AO6" t="inlineStr"/>
       <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
+      <c r="AR6" t="n">
+        <v>1000</v>
+      </c>
       <c r="AS6" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="AT6" t="n">
         <v>0</v>
       </c>
-      <c r="AU6" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU6" t="inlineStr"/>
       <c r="AV6" t="inlineStr"/>
       <c r="AW6" t="inlineStr"/>
       <c r="AX6" t="inlineStr"/>
@@ -1729,42 +1723,42 @@
       <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="n">
-        <v>41880</v>
+        <v>37160</v>
       </c>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="inlineStr"/>
       <c r="BK6" t="inlineStr"/>
       <c r="BL6" t="n">
-        <v>662250</v>
+        <v>608533.3333333334</v>
       </c>
       <c r="BM6" t="n">
-        <v>268820</v>
+        <v>187780</v>
       </c>
       <c r="BN6" t="n">
-        <v>63160</v>
+        <v>54260</v>
       </c>
       <c r="BO6" t="n">
-        <v>41880</v>
+        <v>37160</v>
       </c>
       <c r="BP6" t="n">
-        <v>27433920</v>
+        <v>24111600</v>
       </c>
       <c r="BQ6" t="inlineStr"/>
       <c r="BR6" t="inlineStr"/>
       <c r="BS6" t="inlineStr"/>
       <c r="BT6" t="inlineStr"/>
       <c r="BU6" t="n">
-        <v>486764000</v>
+        <v>445297133.3333333</v>
       </c>
       <c r="BV6" t="n">
-        <v>189029760</v>
+        <v>129544760</v>
       </c>
       <c r="BW6" t="n">
-        <v>42663760</v>
+        <v>36525580</v>
       </c>
       <c r="BX6" t="n">
-        <v>27433920</v>
+        <v>24111600</v>
       </c>
       <c r="BY6" t="inlineStr"/>
       <c r="BZ6" t="inlineStr"/>
@@ -1772,17 +1766,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1818,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
@@ -1857,25 +1851,25 @@
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+      <c r="AK7" t="n">
+        <v>3478500</v>
+      </c>
       <c r="AL7" t="n">
-        <v>3478500</v>
-      </c>
-      <c r="AM7" t="n">
         <v>8141200</v>
       </c>
+      <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr"/>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
+      <c r="AS7" t="n">
+        <v>673100</v>
+      </c>
       <c r="AT7" t="n">
-        <v>673100</v>
-      </c>
-      <c r="AU7" t="n">
         <v>92700</v>
       </c>
+      <c r="AU7" t="inlineStr"/>
       <c r="AV7" t="inlineStr">
         <is>
           <t>モルガン・スタンレーMUFG証券株式会社</t>
@@ -1894,9 +1888,11 @@
       <c r="BC7" t="inlineStr"/>
       <c r="BD7" t="inlineStr"/>
       <c r="BE7" t="inlineStr"/>
-      <c r="BF7" t="inlineStr"/>
+      <c r="BF7" t="n">
+        <v>12978337</v>
+      </c>
       <c r="BG7" t="n">
-        <v>7053860</v>
+        <v>5900920</v>
       </c>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
@@ -1904,16 +1900,16 @@
       <c r="BK7" t="inlineStr"/>
       <c r="BL7" t="inlineStr"/>
       <c r="BM7" t="n">
-        <v>10922450</v>
+        <v>15476400</v>
       </c>
       <c r="BN7" t="n">
-        <v>24024360</v>
+        <v>21291380</v>
       </c>
       <c r="BO7" t="n">
-        <v>7053860</v>
+        <v>5900920</v>
       </c>
       <c r="BP7" t="n">
-        <v>2864719100</v>
+        <v>2376518140</v>
       </c>
       <c r="BQ7" t="inlineStr"/>
       <c r="BR7" t="inlineStr"/>
@@ -1921,13 +1917,13 @@
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
       <c r="BV7" t="n">
-        <v>4758047550</v>
+        <v>7270849000</v>
       </c>
       <c r="BW7" t="n">
-        <v>11174434740</v>
+        <v>9604040680</v>
       </c>
       <c r="BX7" t="n">
-        <v>2864719100</v>
+        <v>2376518140</v>
       </c>
       <c r="BY7" t="inlineStr"/>
       <c r="BZ7" t="inlineStr"/>
@@ -1935,17 +1931,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1983,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
@@ -2020,25 +2016,25 @@
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+      <c r="AK8" t="n">
+        <v>126500</v>
+      </c>
       <c r="AL8" t="n">
-        <v>126500</v>
-      </c>
-      <c r="AM8" t="n">
         <v>187000</v>
       </c>
+      <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
+      <c r="AS8" t="n">
+        <v>39200</v>
+      </c>
       <c r="AT8" t="n">
-        <v>39200</v>
-      </c>
-      <c r="AU8" t="n">
         <v>21600</v>
       </c>
+      <c r="AU8" t="inlineStr"/>
       <c r="AV8" t="inlineStr">
         <is>
           <t>GOLDMAN SACHS INTERNATIONAL</t>
@@ -2056,12 +2052,14 @@
       <c r="BB8" t="inlineStr"/>
       <c r="BC8" t="inlineStr"/>
       <c r="BD8" t="inlineStr"/>
-      <c r="BE8" t="inlineStr"/>
+      <c r="BE8" t="n">
+        <v>379285</v>
+      </c>
       <c r="BF8" t="n">
         <v>379285</v>
       </c>
       <c r="BG8" t="n">
-        <v>159720</v>
+        <v>133560</v>
       </c>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
@@ -2069,16 +2067,16 @@
       <c r="BK8" t="inlineStr"/>
       <c r="BL8" t="inlineStr"/>
       <c r="BM8" t="n">
-        <v>247150</v>
+        <v>245833.3333333333</v>
       </c>
       <c r="BN8" t="n">
-        <v>201040</v>
+        <v>192000</v>
       </c>
       <c r="BO8" t="n">
-        <v>159720</v>
+        <v>133560</v>
       </c>
       <c r="BP8" t="n">
-        <v>65665880</v>
+        <v>54947440</v>
       </c>
       <c r="BQ8" t="inlineStr"/>
       <c r="BR8" t="inlineStr"/>
@@ -2086,13 +2084,13 @@
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
       <c r="BV8" t="n">
-        <v>102748250</v>
+        <v>102468266.6666667</v>
       </c>
       <c r="BW8" t="n">
-        <v>83837520</v>
+        <v>79708300</v>
       </c>
       <c r="BX8" t="n">
-        <v>65665880</v>
+        <v>54947440</v>
       </c>
       <c r="BY8" t="inlineStr"/>
       <c r="BZ8" t="inlineStr"/>
@@ -2100,17 +2098,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -2152,7 +2150,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>929</v>
+        <v>922</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
@@ -2185,25 +2183,25 @@
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
+      <c r="AK9" t="n">
+        <v>62800</v>
+      </c>
       <c r="AL9" t="n">
-        <v>62800</v>
-      </c>
-      <c r="AM9" t="n">
         <v>62400</v>
       </c>
+      <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
       <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="inlineStr"/>
       <c r="AR9" t="inlineStr"/>
-      <c r="AS9" t="inlineStr"/>
+      <c r="AS9" t="n">
+        <v>2200</v>
+      </c>
       <c r="AT9" t="n">
         <v>2200</v>
       </c>
-      <c r="AU9" t="n">
-        <v>2200</v>
-      </c>
+      <c r="AU9" t="inlineStr"/>
       <c r="AV9" t="inlineStr"/>
       <c r="AW9" t="inlineStr"/>
       <c r="AX9" t="inlineStr"/>
@@ -2216,7 +2214,7 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="n">
-        <v>45760</v>
+        <v>43500</v>
       </c>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
@@ -2224,16 +2222,16 @@
       <c r="BK9" t="inlineStr"/>
       <c r="BL9" t="inlineStr"/>
       <c r="BM9" t="n">
-        <v>155450</v>
+        <v>198733.3333333333</v>
       </c>
       <c r="BN9" t="n">
-        <v>150280</v>
+        <v>103320</v>
       </c>
       <c r="BO9" t="n">
-        <v>45760</v>
+        <v>43500</v>
       </c>
       <c r="BP9" t="n">
-        <v>43020500</v>
+        <v>40706260</v>
       </c>
       <c r="BQ9" t="inlineStr"/>
       <c r="BR9" t="inlineStr"/>
@@ -2241,13 +2239,13 @@
       <c r="BT9" t="inlineStr"/>
       <c r="BU9" t="inlineStr"/>
       <c r="BV9" t="n">
-        <v>144927050</v>
+        <v>185306366.6666667</v>
       </c>
       <c r="BW9" t="n">
-        <v>140007220</v>
+        <v>96350860</v>
       </c>
       <c r="BX9" t="n">
-        <v>43020500</v>
+        <v>40706260</v>
       </c>
       <c r="BY9" t="inlineStr"/>
       <c r="BZ9" t="inlineStr"/>
@@ -2255,17 +2253,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -2307,7 +2305,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>1962</v>
+        <v>1935</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2340,25 +2338,25 @@
       <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
+      <c r="AK10" t="n">
+        <v>546000</v>
+      </c>
       <c r="AL10" t="n">
-        <v>546000</v>
-      </c>
-      <c r="AM10" t="n">
         <v>512700</v>
       </c>
+      <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
       <c r="AP10" t="inlineStr"/>
       <c r="AQ10" t="inlineStr"/>
       <c r="AR10" t="inlineStr"/>
-      <c r="AS10" t="inlineStr"/>
+      <c r="AS10" t="n">
+        <v>6700</v>
+      </c>
       <c r="AT10" t="n">
-        <v>6700</v>
-      </c>
-      <c r="AU10" t="n">
         <v>12900</v>
       </c>
+      <c r="AU10" t="inlineStr"/>
       <c r="AV10" t="inlineStr">
         <is>
           <t>GOLDMAN SACHS INTERNATIONAL</t>
@@ -2375,15 +2373,17 @@
       <c r="BA10" t="inlineStr"/>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
-      <c r="BD10" t="inlineStr"/>
+      <c r="BD10" t="n">
+        <v>194633</v>
+      </c>
       <c r="BE10" t="n">
-        <v>194633</v>
+        <v>146386</v>
       </c>
       <c r="BF10" t="n">
         <v>146386</v>
       </c>
       <c r="BG10" t="n">
-        <v>164860</v>
+        <v>151500</v>
       </c>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
@@ -2391,16 +2391,16 @@
       <c r="BK10" t="inlineStr"/>
       <c r="BL10" t="inlineStr"/>
       <c r="BM10" t="n">
-        <v>195250</v>
+        <v>206866.6666666667</v>
       </c>
       <c r="BN10" t="n">
-        <v>184180</v>
+        <v>167780</v>
       </c>
       <c r="BO10" t="n">
-        <v>164860</v>
+        <v>151500</v>
       </c>
       <c r="BP10" t="n">
-        <v>314149400</v>
+        <v>290372980</v>
       </c>
       <c r="BQ10" t="inlineStr"/>
       <c r="BR10" t="inlineStr"/>
@@ -2408,13 +2408,13 @@
       <c r="BT10" t="inlineStr"/>
       <c r="BU10" t="inlineStr"/>
       <c r="BV10" t="n">
-        <v>351530650</v>
+        <v>375613033.3333333</v>
       </c>
       <c r="BW10" t="n">
-        <v>343918960</v>
+        <v>314505480</v>
       </c>
       <c r="BX10" t="n">
-        <v>314149400</v>
+        <v>290372980</v>
       </c>
       <c r="BY10" t="inlineStr"/>
       <c r="BZ10" t="inlineStr"/>
@@ -2422,17 +2422,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>442</v>
+        <v>460</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2507,25 +2507,25 @@
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
+      <c r="AK11" t="n">
+        <v>11624300</v>
+      </c>
       <c r="AL11" t="n">
-        <v>11624300</v>
-      </c>
-      <c r="AM11" t="n">
         <v>12401300</v>
       </c>
+      <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
       <c r="AP11" t="inlineStr"/>
       <c r="AQ11" t="inlineStr"/>
       <c r="AR11" t="inlineStr"/>
-      <c r="AS11" t="inlineStr"/>
+      <c r="AS11" t="n">
+        <v>86900</v>
+      </c>
       <c r="AT11" t="n">
-        <v>86900</v>
-      </c>
-      <c r="AU11" t="n">
         <v>84500</v>
       </c>
+      <c r="AU11" t="inlineStr"/>
       <c r="AV11" t="inlineStr"/>
       <c r="AW11" t="inlineStr"/>
       <c r="AX11" t="inlineStr"/>
@@ -2538,7 +2538,7 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="n">
-        <v>2531780</v>
+        <v>2334260</v>
       </c>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
@@ -2546,16 +2546,16 @@
       <c r="BK11" t="inlineStr"/>
       <c r="BL11" t="inlineStr"/>
       <c r="BM11" t="n">
-        <v>2210850</v>
+        <v>2252600</v>
       </c>
       <c r="BN11" t="n">
-        <v>1845660</v>
+        <v>2157100</v>
       </c>
       <c r="BO11" t="n">
-        <v>2531780</v>
+        <v>2334260</v>
       </c>
       <c r="BP11" t="n">
-        <v>1073563280</v>
+        <v>1010391360</v>
       </c>
       <c r="BQ11" t="inlineStr"/>
       <c r="BR11" t="inlineStr"/>
@@ -2563,13 +2563,13 @@
       <c r="BT11" t="inlineStr"/>
       <c r="BU11" t="inlineStr"/>
       <c r="BV11" t="n">
-        <v>984957200</v>
+        <v>988981966.6666666</v>
       </c>
       <c r="BW11" t="n">
-        <v>791971060</v>
+        <v>920704780</v>
       </c>
       <c r="BX11" t="n">
-        <v>1073563280</v>
+        <v>1010391360</v>
       </c>
       <c r="BY11" t="inlineStr"/>
       <c r="BZ11" t="inlineStr"/>
@@ -2577,17 +2577,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>1009</v>
+        <v>978</v>
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2663,30 +2663,30 @@
       <c r="AI12" t="inlineStr"/>
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="n">
+      <c r="AL12" t="n">
         <v>353800</v>
       </c>
+      <c r="AM12" t="inlineStr"/>
       <c r="AN12" t="inlineStr"/>
       <c r="AO12" t="inlineStr"/>
       <c r="AP12" t="inlineStr"/>
       <c r="AQ12" t="inlineStr"/>
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="inlineStr"/>
-      <c r="AU12" t="n">
-        <v>0</v>
-      </c>
+      <c r="AT12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU12" t="inlineStr"/>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>モルガン・スタンレーMUFG証券株式会社、Nomura International plc、Jump Trading Pacific Pte Ltd</t>
+          <t>Jump Trading Pacific Pte Ltd、Nomura International plc、モルガン・スタンレーMUFG証券株式会社</t>
         </is>
       </c>
       <c r="AW12" t="n">
-        <v>0.0398</v>
+        <v>0.0343</v>
       </c>
       <c r="AX12" t="n">
-        <v>293100</v>
+        <v>234400</v>
       </c>
       <c r="AY12" t="inlineStr"/>
       <c r="AZ12" t="inlineStr"/>
@@ -2695,9 +2695,11 @@
       <c r="BC12" t="inlineStr"/>
       <c r="BD12" t="inlineStr"/>
       <c r="BE12" t="inlineStr"/>
-      <c r="BF12" t="inlineStr"/>
+      <c r="BF12" t="n">
+        <v>234400</v>
+      </c>
       <c r="BG12" t="n">
-        <v>543420</v>
+        <v>361580</v>
       </c>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
@@ -2706,13 +2708,13 @@
       <c r="BL12" t="inlineStr"/>
       <c r="BM12" t="inlineStr"/>
       <c r="BN12" t="n">
-        <v>2872425</v>
+        <v>2510860</v>
       </c>
       <c r="BO12" t="n">
-        <v>543420</v>
+        <v>361580</v>
       </c>
       <c r="BP12" t="n">
-        <v>530125660</v>
+        <v>348711880</v>
       </c>
       <c r="BQ12" t="inlineStr"/>
       <c r="BR12" t="inlineStr"/>
@@ -2721,10 +2723,10 @@
       <c r="BU12" t="inlineStr"/>
       <c r="BV12" t="inlineStr"/>
       <c r="BW12" t="n">
-        <v>3084106450</v>
+        <v>2679272900</v>
       </c>
       <c r="BX12" t="n">
-        <v>530125660</v>
+        <v>348711880</v>
       </c>
       <c r="BY12" t="inlineStr"/>
       <c r="BZ12" t="inlineStr"/>
@@ -2732,17 +2734,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2786,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>467</v>
+        <v>508</v>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2818,20 +2820,20 @@
       <c r="AI13" t="inlineStr"/>
       <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="n">
+      <c r="AL13" t="n">
         <v>867300</v>
       </c>
+      <c r="AM13" t="inlineStr"/>
       <c r="AN13" t="inlineStr"/>
       <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr"/>
       <c r="AQ13" t="inlineStr"/>
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="n">
+      <c r="AT13" t="n">
         <v>1500</v>
       </c>
+      <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr">
         <is>
           <t>野村證券株式会社、Nomura International plc</t>
@@ -2849,12 +2851,14 @@
       <c r="BB13" t="inlineStr"/>
       <c r="BC13" t="inlineStr"/>
       <c r="BD13" t="inlineStr"/>
-      <c r="BE13" t="inlineStr"/>
+      <c r="BE13" t="n">
+        <v>525000</v>
+      </c>
       <c r="BF13" t="n">
-        <v>525000</v>
+        <v>766300</v>
       </c>
       <c r="BG13" t="n">
-        <v>5339820</v>
+        <v>2967840</v>
       </c>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
@@ -2863,13 +2867,13 @@
       <c r="BL13" t="inlineStr"/>
       <c r="BM13" t="inlineStr"/>
       <c r="BN13" t="n">
-        <v>3251933.333333333</v>
+        <v>6937850</v>
       </c>
       <c r="BO13" t="n">
-        <v>5339820</v>
+        <v>2967840</v>
       </c>
       <c r="BP13" t="n">
-        <v>3184952700</v>
+        <v>1612993800</v>
       </c>
       <c r="BQ13" t="inlineStr"/>
       <c r="BR13" t="inlineStr"/>
@@ -2878,10 +2882,10 @@
       <c r="BU13" t="inlineStr"/>
       <c r="BV13" t="inlineStr"/>
       <c r="BW13" t="n">
-        <v>1553883300</v>
+        <v>3931852700</v>
       </c>
       <c r="BX13" t="n">
-        <v>3184952700</v>
+        <v>1612993800</v>
       </c>
       <c r="BY13" t="inlineStr"/>
       <c r="BZ13" t="inlineStr"/>
@@ -2889,17 +2893,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2945,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>3835</v>
+        <v>3580</v>
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -2975,20 +2979,20 @@
       <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="n">
+      <c r="AL14" t="n">
         <v>78200</v>
       </c>
+      <c r="AM14" t="inlineStr"/>
       <c r="AN14" t="inlineStr"/>
       <c r="AO14" t="inlineStr"/>
       <c r="AP14" t="inlineStr"/>
       <c r="AQ14" t="inlineStr"/>
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
-      <c r="AT14" t="inlineStr"/>
-      <c r="AU14" t="n">
+      <c r="AT14" t="n">
         <v>6900</v>
       </c>
+      <c r="AU14" t="inlineStr"/>
       <c r="AV14" t="inlineStr"/>
       <c r="AW14" t="inlineStr"/>
       <c r="AX14" t="inlineStr"/>
@@ -3001,7 +3005,7 @@
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="inlineStr"/>
       <c r="BG14" t="n">
-        <v>390100</v>
+        <v>351560</v>
       </c>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
@@ -3010,13 +3014,13 @@
       <c r="BL14" t="inlineStr"/>
       <c r="BM14" t="inlineStr"/>
       <c r="BN14" t="n">
-        <v>1185300</v>
+        <v>818800</v>
       </c>
       <c r="BO14" t="n">
-        <v>390100</v>
+        <v>351560</v>
       </c>
       <c r="BP14" t="n">
-        <v>1547782700</v>
+        <v>1479464800</v>
       </c>
       <c r="BQ14" t="inlineStr"/>
       <c r="BR14" t="inlineStr"/>
@@ -3025,10 +3029,10 @@
       <c r="BU14" t="inlineStr"/>
       <c r="BV14" t="inlineStr"/>
       <c r="BW14" t="n">
-        <v>3532839500</v>
+        <v>2428380250</v>
       </c>
       <c r="BX14" t="n">
-        <v>1547782700</v>
+        <v>1479464800</v>
       </c>
       <c r="BY14" t="inlineStr"/>
       <c r="BZ14" t="inlineStr"/>
@@ -3036,17 +3040,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3142,7 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="n">
-        <v>166.6666666666667</v>
+        <v>200</v>
       </c>
       <c r="BH15" t="n">
         <v>100</v>
@@ -3147,25 +3151,25 @@
         <v>450</v>
       </c>
       <c r="BJ15" t="n">
-        <v>166.6666666666667</v>
+        <v>200</v>
       </c>
       <c r="BK15" t="n">
-        <v>325</v>
+        <v>300</v>
       </c>
       <c r="BL15" t="n">
-        <v>233.3333333333333</v>
+        <v>250</v>
       </c>
       <c r="BM15" t="n">
         <v>300</v>
       </c>
       <c r="BN15" t="n">
-        <v>150</v>
+        <v>133.3333333333333</v>
       </c>
       <c r="BO15" t="n">
-        <v>166.6666666666667</v>
+        <v>200</v>
       </c>
       <c r="BP15" t="n">
-        <v>4153666.666666667</v>
+        <v>4980500</v>
       </c>
       <c r="BQ15" t="n">
         <v>2645000</v>
@@ -3174,22 +3178,22 @@
         <v>11285000</v>
       </c>
       <c r="BS15" t="n">
-        <v>4161000</v>
+        <v>4993250</v>
       </c>
       <c r="BT15" t="n">
-        <v>8085750</v>
+        <v>7443250</v>
       </c>
       <c r="BU15" t="n">
-        <v>5813333.333333333</v>
+        <v>6260000</v>
       </c>
       <c r="BV15" t="n">
         <v>7372000</v>
       </c>
       <c r="BW15" t="n">
-        <v>3750500</v>
+        <v>3333666.666666667</v>
       </c>
       <c r="BX15" t="n">
-        <v>4153666.666666667</v>
+        <v>4980500</v>
       </c>
       <c r="BY15" t="inlineStr"/>
       <c r="BZ15" t="inlineStr"/>
@@ -3197,17 +3201,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3253,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -3278,29 +3282,27 @@
         <v>112008</v>
       </c>
       <c r="AF16" t="n">
-        <v>204885</v>
+        <v>97185</v>
       </c>
       <c r="AG16" t="n">
-        <v>97185</v>
+        <v>93675</v>
       </c>
       <c r="AH16" t="n">
-        <v>93675</v>
+        <v>126528</v>
       </c>
       <c r="AI16" t="n">
-        <v>126528</v>
+        <v>99264</v>
       </c>
       <c r="AJ16" t="n">
-        <v>99264</v>
+        <v>96080</v>
       </c>
       <c r="AK16" t="n">
-        <v>96080</v>
+        <v>122230</v>
       </c>
       <c r="AL16" t="n">
-        <v>122230</v>
-      </c>
-      <c r="AM16" t="n">
         <v>112008</v>
       </c>
+      <c r="AM16" t="inlineStr"/>
       <c r="AN16" t="n">
         <v>0</v>
       </c>
@@ -3322,9 +3324,7 @@
       <c r="AT16" t="n">
         <v>0</v>
       </c>
-      <c r="AU16" t="n">
-        <v>0</v>
-      </c>
+      <c r="AU16" t="inlineStr"/>
       <c r="AV16" t="inlineStr"/>
       <c r="AW16" t="inlineStr"/>
       <c r="AX16" t="inlineStr"/>
@@ -3337,58 +3337,58 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="n">
-        <v>4111983.8</v>
+        <v>2632194.8</v>
       </c>
       <c r="BH16" t="n">
-        <v>9570452.800000001</v>
+        <v>7299611.6</v>
       </c>
       <c r="BI16" t="n">
-        <v>3267717.4</v>
+        <v>2742294</v>
       </c>
       <c r="BJ16" t="n">
-        <v>3674551.2</v>
+        <v>3912781</v>
       </c>
       <c r="BK16" t="n">
-        <v>4241035.4</v>
+        <v>4714386.8</v>
       </c>
       <c r="BL16" t="n">
-        <v>3010975.8</v>
+        <v>2238110.2</v>
       </c>
       <c r="BM16" t="n">
-        <v>1764609.6</v>
+        <v>1913806.6</v>
       </c>
       <c r="BN16" t="n">
-        <v>1690468.6</v>
+        <v>3083292.6</v>
       </c>
       <c r="BO16" t="n">
-        <v>4111983.8</v>
+        <v>2632194.8</v>
       </c>
       <c r="BP16" t="n">
-        <v>124253885.4</v>
+        <v>79842952.8</v>
       </c>
       <c r="BQ16" t="n">
-        <v>292344615.4</v>
+        <v>226772440</v>
       </c>
       <c r="BR16" t="n">
-        <v>83737882</v>
+        <v>69693452.8</v>
       </c>
       <c r="BS16" t="n">
-        <v>107086813.6</v>
+        <v>114743178.6</v>
       </c>
       <c r="BT16" t="n">
-        <v>131265781.6</v>
+        <v>148128099</v>
       </c>
       <c r="BU16" t="n">
-        <v>92793402.59999999</v>
+        <v>67164683.59999999</v>
       </c>
       <c r="BV16" t="n">
-        <v>48812478.4</v>
+        <v>52170691.2</v>
       </c>
       <c r="BW16" t="n">
-        <v>45282081.2</v>
+        <v>88928311</v>
       </c>
       <c r="BX16" t="n">
-        <v>124253885.4</v>
+        <v>79842952.8</v>
       </c>
       <c r="BY16" t="inlineStr"/>
       <c r="BZ16" t="inlineStr"/>
@@ -3396,17 +3396,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260417-001531</t>
+          <t>20260417-190047</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-16T15:15:31+00:00</t>
+          <t>2026-04-17T10:00:47+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-17T00:15:31+09:00</t>
+          <t>2026-04-17T19:00:47+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-18
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -1026,17 +1026,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1221,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1440,17 +1440,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1603,17 +1603,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1766,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -1931,17 +1931,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2253,17 +2253,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2422,17 +2422,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2577,17 +2577,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2734,17 +2734,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -2893,17 +2893,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -3040,17 +3040,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3201,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>
@@ -3396,17 +3396,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260417-233832</t>
+          <t>20260418-190053</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-17T14:38:32+00:00</t>
+          <t>2026-04-18T10:00:53+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-17T23:38:32+09:00</t>
+          <t>2026-04-18T19:00:53+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: screening master 2026-04-19
</commit_message>
<xml_diff>
--- a/bi/outputs/screening_master_data_gaps.xlsx
+++ b/bi/outputs/screening_master_data_gaps.xlsx
@@ -1026,17 +1026,17 @@
       <c r="CB2" t="inlineStr"/>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD2" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE2" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1221,17 @@
       <c r="CB3" t="inlineStr"/>
       <c r="CC3" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD3" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE3" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1440,17 +1440,17 @@
       <c r="CB4" t="inlineStr"/>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1603,17 +1603,17 @@
       <c r="CB5" t="inlineStr"/>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1766,17 @@
       <c r="CB6" t="inlineStr"/>
       <c r="CC6" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD6" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE6" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -1931,17 +1931,17 @@
       <c r="CB7" t="inlineStr"/>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE7" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2098,17 +2098,17 @@
       <c r="CB8" t="inlineStr"/>
       <c r="CC8" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD8" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE8" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2253,17 +2253,17 @@
       <c r="CB9" t="inlineStr"/>
       <c r="CC9" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD9" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE9" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2422,17 +2422,17 @@
       <c r="CB10" t="inlineStr"/>
       <c r="CC10" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD10" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE10" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2577,17 +2577,17 @@
       <c r="CB11" t="inlineStr"/>
       <c r="CC11" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD11" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE11" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2734,17 +2734,17 @@
       <c r="CB12" t="inlineStr"/>
       <c r="CC12" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD12" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE12" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -2893,17 +2893,17 @@
       <c r="CB13" t="inlineStr"/>
       <c r="CC13" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD13" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE13" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3040,17 +3040,17 @@
       <c r="CB14" t="inlineStr"/>
       <c r="CC14" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD14" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE14" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3201,17 +3201,17 @@
       <c r="CB15" t="inlineStr"/>
       <c r="CC15" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD15" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE15" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>
@@ -3396,17 +3396,17 @@
       <c r="CB16" t="inlineStr"/>
       <c r="CC16" t="inlineStr">
         <is>
-          <t>20260418-190053</t>
+          <t>20260419-190049</t>
         </is>
       </c>
       <c r="CD16" t="inlineStr">
         <is>
-          <t>2026-04-18T10:00:53+00:00</t>
+          <t>2026-04-19T10:00:49+00:00</t>
         </is>
       </c>
       <c r="CE16" t="inlineStr">
         <is>
-          <t>2026-04-18T19:00:53+09:00</t>
+          <t>2026-04-19T19:00:49+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>